<commit_message>
Actualizo tableros (2026-06-10 14:11)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1C35DBF9-9B53-4F18-8E62-95EEEB87BD0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E48008D-E5D6-439E-85BC-07B3D03B4F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-150" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -722,7 +722,7 @@
         <v>37</v>
       </c>
       <c r="C21" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="22" spans="1:3" x14ac:dyDescent="0.25">
@@ -733,7 +733,7 @@
         <v>38</v>
       </c>
       <c r="C22" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Agranda el logo de Hergo (40-42px) que se veia chico; actualiza Excel
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\layla\Documentos\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E48008D-E5D6-439E-85BC-07B3D03B4F23}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED01F78-A36B-46A4-834A-F312B5F5E391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="50">
   <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=e87b9f6f-d894-4e54-9353-f17aa155e82b&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
@@ -169,6 +169,12 @@
   </si>
   <si>
     <t>Agrupacion</t>
+  </si>
+  <si>
+    <t>DIRECTORIO</t>
+  </si>
+  <si>
+    <t>Area</t>
   </si>
 </sst>
 </file>
@@ -486,253 +492,320 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:C22"/>
+  <dimension ref="A1:D22"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="138" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="138" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
+        <v>49</v>
+      </c>
+      <c r="B1" t="s">
         <v>47</v>
       </c>
-      <c r="B1" t="s">
+      <c r="C1" t="s">
         <v>45</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>46</v>
       </c>
     </row>
-    <row r="2" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
         <v>39</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B3" t="s">
+        <v>3</v>
+      </c>
+      <c r="C3" t="s">
         <v>40</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B4" t="s">
+        <v>3</v>
+      </c>
+      <c r="C4" t="s">
         <v>41</v>
       </c>
-      <c r="C4" t="s">
+      <c r="D4" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="5" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
+        <v>48</v>
+      </c>
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="B5" t="s">
+      <c r="C5" t="s">
         <v>7</v>
       </c>
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="6" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
+        <v>48</v>
+      </c>
+      <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="B6" t="s">
+      <c r="C6" t="s">
         <v>9</v>
       </c>
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>8</v>
       </c>
     </row>
-    <row r="7" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B7" t="s">
+        <v>3</v>
+      </c>
+      <c r="C7" t="s">
         <v>11</v>
       </c>
-      <c r="C7" t="s">
+      <c r="D7" t="s">
         <v>10</v>
       </c>
     </row>
-    <row r="8" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B8" t="s">
+        <v>3</v>
+      </c>
+      <c r="C8" t="s">
         <v>13</v>
       </c>
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B9" t="s">
+        <v>3</v>
+      </c>
+      <c r="C9" t="s">
         <v>1</v>
       </c>
-      <c r="C9" t="s">
+      <c r="D9" t="s">
         <v>14</v>
       </c>
     </row>
-    <row r="10" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B10" t="s">
+        <v>3</v>
+      </c>
+      <c r="C10" t="s">
         <v>16</v>
       </c>
-      <c r="C10" t="s">
+      <c r="D10" t="s">
         <v>15</v>
       </c>
     </row>
-    <row r="11" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B11" t="s">
+        <v>3</v>
+      </c>
+      <c r="C11" t="s">
         <v>18</v>
       </c>
-      <c r="C11" t="s">
+      <c r="D11" t="s">
         <v>17</v>
       </c>
     </row>
-    <row r="12" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B12" t="s">
+        <v>3</v>
+      </c>
+      <c r="C12" t="s">
         <v>19</v>
       </c>
-      <c r="C12" t="s">
+      <c r="D12" t="s">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B13" t="s">
+        <v>3</v>
+      </c>
+      <c r="C13" t="s">
         <v>20</v>
       </c>
-      <c r="C13" t="s">
+      <c r="D13" t="s">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B14" t="s">
+        <v>3</v>
+      </c>
+      <c r="C14" t="s">
         <v>24</v>
       </c>
-      <c r="C14" t="s">
+      <c r="D14" t="s">
         <v>23</v>
       </c>
     </row>
-    <row r="15" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B15" t="s">
+        <v>3</v>
+      </c>
+      <c r="C15" t="s">
         <v>26</v>
       </c>
-      <c r="C15" t="s">
+      <c r="D15" t="s">
         <v>25</v>
       </c>
     </row>
-    <row r="16" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
+        <v>48</v>
+      </c>
+      <c r="B16" t="s">
         <v>29</v>
       </c>
-      <c r="B16" t="s">
+      <c r="C16" t="s">
         <v>28</v>
       </c>
-      <c r="C16" t="s">
+      <c r="D16" t="s">
         <v>27</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
+        <v>3</v>
+      </c>
+      <c r="C17" t="s">
         <v>31</v>
       </c>
-      <c r="C17" t="s">
+      <c r="D17" t="s">
         <v>30</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
+        <v>48</v>
+      </c>
+      <c r="B18" t="s">
         <v>29</v>
       </c>
-      <c r="B18" t="s">
+      <c r="C18" t="s">
         <v>33</v>
       </c>
-      <c r="C18" t="s">
+      <c r="D18" t="s">
         <v>32</v>
       </c>
     </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" t="s">
         <v>35</v>
       </c>
-      <c r="C19" t="s">
+      <c r="D19" t="s">
         <v>34</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B20" t="s">
+        <v>3</v>
+      </c>
+      <c r="C20" t="s">
         <v>36</v>
       </c>
-      <c r="C20" t="s">
+      <c r="D20" t="s">
         <v>42</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B21" t="s">
+        <v>3</v>
+      </c>
+      <c r="C21" t="s">
         <v>37</v>
       </c>
-      <c r="C21" t="s">
+      <c r="D21" t="s">
         <v>44</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>3</v>
+        <v>48</v>
       </c>
       <c r="B22" t="s">
+        <v>3</v>
+      </c>
+      <c r="C22" t="s">
         <v>38</v>
       </c>
-      <c r="C22" t="s">
+      <c r="D22" t="s">
         <v>43</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Agrega otro link en LINKS POWER BI.xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\layla\Documentos\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8ED01F78-A36B-46A4-834A-F312B5F5E391}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6D7FF0-9AFF-4192-8569-D0AFA21A2F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="88" uniqueCount="50">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
   <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=e87b9f6f-d894-4e54-9353-f17aa155e82b&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
@@ -175,6 +175,12 @@
   </si>
   <si>
     <t>Area</t>
+  </si>
+  <si>
+    <t>https://app.powerbi.com/reportEmbed?reportId=467411be-b152-4571-aab6-634eb4bf23fc&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
+  </si>
+  <si>
+    <t>SEGUIMIENTO DE OFERTAS</t>
   </si>
 </sst>
 </file>
@@ -492,7 +498,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D22"/>
+  <dimension ref="A1:D23"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -809,6 +815,20 @@
         <v>43</v>
       </c>
     </row>
+    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A23" t="s">
+        <v>48</v>
+      </c>
+      <c r="B23" t="s">
+        <v>3</v>
+      </c>
+      <c r="C23" t="s">
+        <v>51</v>
+      </c>
+      <c r="D23" t="s">
+        <v>50</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Actualiza un link en LINKS POWER BI.xlsx
Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1F6D7FF0-9AFF-4192-8569-D0AFA21A2F21}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7D3078FA-59BD-44B3-9B8B-D673D9BE4AC7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="52">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
   <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=e87b9f6f-d894-4e54-9353-f17aa155e82b&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
@@ -181,6 +181,12 @@
   </si>
   <si>
     <t>SEGUIMIENTO DE OFERTAS</t>
+  </si>
+  <si>
+    <t>MERMAS MC</t>
+  </si>
+  <si>
+    <t>https://app.powerbi.com/reportEmbed?reportId=dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
 </sst>
 </file>
@@ -498,7 +504,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D23"/>
+  <dimension ref="A1:D24"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
@@ -829,6 +835,20 @@
         <v>50</v>
       </c>
     </row>
+    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A24" t="s">
+        <v>48</v>
+      </c>
+      <c r="B24" t="s">
+        <v>29</v>
+      </c>
+      <c r="C24" t="s">
+        <v>52</v>
+      </c>
+      <c r="D24" t="s">
+        <v>53</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Agrega areas de apps/portales y columna Descripcion
Suma AREAS COMUNES, PREVENTA, PREVENTA MAYORISTA y DEPOSITO (apps y
portales internos) y una columna Descripcion. DIRECTORIO sin cambios.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -8,19 +8,19 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{26D6C4D0-DE4D-486E-817E-CDB1F91B31CD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AE14790E-7056-4E96-9815-040FD593964D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-150" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="96" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="157" uniqueCount="94">
   <si>
     <t>Area</t>
   </si>
@@ -182,16 +182,144 @@
   </si>
   <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
+  </si>
+  <si>
+    <t>Reserva de Sala de reuniones</t>
+  </si>
+  <si>
+    <t>ERP Nuevo (Testing)</t>
+  </si>
+  <si>
+    <t>APP Ventas (Principal)</t>
+  </si>
+  <si>
+    <t>APP Ventas (Backup)</t>
+  </si>
+  <si>
+    <t>Portal Autogestion Clientes</t>
+  </si>
+  <si>
+    <t>APP Ventas Mayorista</t>
+  </si>
+  <si>
+    <t>APP Deposito (PC + TRACK)</t>
+  </si>
+  <si>
+    <t>APP Stock (Celular)</t>
+  </si>
+  <si>
+    <t>Portal Implantacion</t>
+  </si>
+  <si>
+    <t>Giftcards</t>
+  </si>
+  <si>
+    <t>APP Verificadores Precios</t>
+  </si>
+  <si>
+    <t>http://192.168.1.140:5173</t>
+  </si>
+  <si>
+    <t>http://192.168.4.6:9013</t>
+  </si>
+  <si>
+    <t>https://portal.hergo.com.ar:9010</t>
+  </si>
+  <si>
+    <t>https://hergo-presale-front.vercel.app</t>
+  </si>
+  <si>
+    <t>https://portal.hergo.com.ar</t>
+  </si>
+  <si>
+    <t>https://hergo-api-front.vercel.app</t>
+  </si>
+  <si>
+    <t>https://portal.hergo.com.ar:9011</t>
+  </si>
+  <si>
+    <t>https://portal.hergo.com.ar:9020/Stock</t>
+  </si>
+  <si>
+    <t>https://portal.hergo.com.ar:9016</t>
+  </si>
+  <si>
+    <t>https://portal.altadistribucion.com.ar</t>
+  </si>
+  <si>
+    <t>https://giftcards-app-psi.vercel.app</t>
+  </si>
+  <si>
+    <t>https://prices-kohl.vercel.app</t>
+  </si>
+  <si>
+    <t>ADMINISTRACION</t>
+  </si>
+  <si>
+    <t>DEPOSITO</t>
+  </si>
+  <si>
+    <t>AREAS COMUNES</t>
+  </si>
+  <si>
+    <t>PREVENTA</t>
+  </si>
+  <si>
+    <t>Permite la reserva de todas las salas de reuniones disponibles del grupo</t>
+  </si>
+  <si>
+    <t>Pruebas de concepto y muestra del desarrollo del nuevo ERP</t>
+  </si>
+  <si>
+    <t>Carga de Pedidos de Vendedores de Distribucion</t>
+  </si>
+  <si>
+    <t>Carga de Pedidos de Clientes de Mayorista</t>
+  </si>
+  <si>
+    <t>Carga de pedidos de vendedores de Mayorista</t>
+  </si>
+  <si>
+    <t>Administracion de Ingresos y Armado de Pedidos</t>
+  </si>
+  <si>
+    <t>Consulta de Stock de Productos</t>
+  </si>
+  <si>
+    <t>Definicion de Gondolas y administracion de imágenes de implantación</t>
+  </si>
+  <si>
+    <t>Carga de Pedidos de Clientes de Distribucion</t>
+  </si>
+  <si>
+    <t>Administracion y uso de Giftcard para las Tiendas</t>
+  </si>
+  <si>
+    <t>Consulta de Precios de articulos de Tiendas</t>
+  </si>
+  <si>
+    <t>Descripcion</t>
+  </si>
+  <si>
+    <t>PREVENTA MAYORISTA</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <fonts count="2" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -214,13 +342,16 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -499,16 +630,17 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D24"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="11.7109375" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="26.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="138" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="27.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="139.140625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="65.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -521,8 +653,11 @@
       <c r="D1" t="s">
         <v>3</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="E1" t="s">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
         <v>4</v>
       </c>
@@ -536,7 +671,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
         <v>4</v>
       </c>
@@ -550,7 +685,7 @@
         <v>9</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
         <v>4</v>
       </c>
@@ -564,7 +699,7 @@
         <v>11</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
         <v>4</v>
       </c>
@@ -578,7 +713,7 @@
         <v>14</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
         <v>4</v>
       </c>
@@ -592,7 +727,7 @@
         <v>16</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
         <v>4</v>
       </c>
@@ -606,7 +741,7 @@
         <v>18</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
         <v>4</v>
       </c>
@@ -620,7 +755,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
         <v>4</v>
       </c>
@@ -634,7 +769,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
         <v>4</v>
       </c>
@@ -648,7 +783,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
         <v>4</v>
       </c>
@@ -662,7 +797,7 @@
         <v>26</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
         <v>4</v>
       </c>
@@ -676,7 +811,7 @@
         <v>28</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
         <v>4</v>
       </c>
@@ -690,7 +825,7 @@
         <v>30</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
         <v>4</v>
       </c>
@@ -704,7 +839,7 @@
         <v>32</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
         <v>4</v>
       </c>
@@ -718,7 +853,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
         <v>4</v>
       </c>
@@ -732,7 +867,7 @@
         <v>37</v>
       </c>
     </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
         <v>4</v>
       </c>
@@ -746,7 +881,7 @@
         <v>39</v>
       </c>
     </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
         <v>4</v>
       </c>
@@ -760,7 +895,7 @@
         <v>41</v>
       </c>
     </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
         <v>4</v>
       </c>
@@ -774,7 +909,7 @@
         <v>43</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
         <v>4</v>
       </c>
@@ -788,7 +923,7 @@
         <v>45</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
         <v>4</v>
       </c>
@@ -802,7 +937,7 @@
         <v>47</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
         <v>4</v>
       </c>
@@ -816,7 +951,7 @@
         <v>49</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
         <v>4</v>
       </c>
@@ -830,7 +965,7 @@
         <v>51</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.25">
+    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
         <v>4</v>
       </c>
@@ -844,7 +979,225 @@
         <v>53</v>
       </c>
     </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A25" t="s">
+        <v>79</v>
+      </c>
+      <c r="B25" t="s">
+        <v>77</v>
+      </c>
+      <c r="C25" t="s">
+        <v>54</v>
+      </c>
+      <c r="D25" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="E25" t="s">
+        <v>81</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A26" t="s">
+        <v>79</v>
+      </c>
+      <c r="B26" t="s">
+        <v>77</v>
+      </c>
+      <c r="C26" t="s">
+        <v>55</v>
+      </c>
+      <c r="D26" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="E26" t="s">
+        <v>82</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A27" t="s">
+        <v>80</v>
+      </c>
+      <c r="B27" t="s">
+        <v>5</v>
+      </c>
+      <c r="C27" t="s">
+        <v>56</v>
+      </c>
+      <c r="D27" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="E27" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A28" t="s">
+        <v>80</v>
+      </c>
+      <c r="B28" t="s">
+        <v>5</v>
+      </c>
+      <c r="C28" t="s">
+        <v>57</v>
+      </c>
+      <c r="D28" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="E28" t="s">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A29" t="s">
+        <v>93</v>
+      </c>
+      <c r="B29" t="s">
+        <v>5</v>
+      </c>
+      <c r="C29" t="s">
+        <v>58</v>
+      </c>
+      <c r="D29" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="E29" t="s">
+        <v>84</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A30" t="s">
+        <v>93</v>
+      </c>
+      <c r="B30" t="s">
+        <v>5</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E30" t="s">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A31" t="s">
+        <v>78</v>
+      </c>
+      <c r="B31" t="s">
+        <v>78</v>
+      </c>
+      <c r="C31" t="s">
+        <v>60</v>
+      </c>
+      <c r="D31" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="E31" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A32" t="s">
+        <v>79</v>
+      </c>
+      <c r="B32" t="s">
+        <v>78</v>
+      </c>
+      <c r="C32" t="s">
+        <v>61</v>
+      </c>
+      <c r="D32" s="1" t="s">
+        <v>72</v>
+      </c>
+      <c r="E32" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="33" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A33" t="s">
+        <v>79</v>
+      </c>
+      <c r="B33" t="s">
+        <v>77</v>
+      </c>
+      <c r="C33" t="s">
+        <v>62</v>
+      </c>
+      <c r="D33" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="E33" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="34" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A34" t="s">
+        <v>80</v>
+      </c>
+      <c r="B34" t="s">
+        <v>5</v>
+      </c>
+      <c r="C34" t="s">
+        <v>58</v>
+      </c>
+      <c r="D34" s="1" t="s">
+        <v>74</v>
+      </c>
+      <c r="E34" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A35" t="s">
+        <v>79</v>
+      </c>
+      <c r="B35" t="s">
+        <v>77</v>
+      </c>
+      <c r="C35" t="s">
+        <v>63</v>
+      </c>
+      <c r="D35" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="E35" t="s">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A36" t="s">
+        <v>79</v>
+      </c>
+      <c r="B36" t="s">
+        <v>77</v>
+      </c>
+      <c r="C36" t="s">
+        <v>64</v>
+      </c>
+      <c r="D36" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="E36" t="s">
+        <v>91</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{3C331869-98F3-4B87-ADF4-988275037827}"/>
+    <hyperlink ref="D25" r:id="rId2" xr:uid="{C8EAE465-89E0-4628-B2F4-6BE05A058D61}"/>
+    <hyperlink ref="D27" r:id="rId3" xr:uid="{75879039-BAE6-4CF6-AF43-763E9ECF0BD7}"/>
+    <hyperlink ref="D28" r:id="rId4" xr:uid="{DD4E29F3-166F-493E-8A70-5618EF533237}"/>
+    <hyperlink ref="D29" r:id="rId5" xr:uid="{25941851-C2B0-46ED-A55A-A06791D0EE0F}"/>
+    <hyperlink ref="D30" r:id="rId6" xr:uid="{E18B7B62-B80E-48E0-A060-6504BBB826E5}"/>
+    <hyperlink ref="D31" r:id="rId7" xr:uid="{58882F6E-9D0E-44A6-8F3D-AA3F518FC470}"/>
+    <hyperlink ref="D32" r:id="rId8" xr:uid="{AEF67EE1-A7B2-4C96-AD8F-EB9A98A208FD}"/>
+    <hyperlink ref="D33" r:id="rId9" xr:uid="{E10D50A9-A10A-45D2-A783-C335928BADAD}"/>
+    <hyperlink ref="D34" r:id="rId10" xr:uid="{A0AC4C5E-2431-4290-9E22-334EFC1ADF2A}"/>
+    <hyperlink ref="D35" r:id="rId11" xr:uid="{1AE79520-3345-461B-A674-520AF8AF695A}"/>
+    <hyperlink ref="D36" r:id="rId12" xr:uid="{DE513581-C953-4F03-BD77-004288A420F8}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Actualizo tableros (2026-07-30 16:59)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A2045996-D09E-4174-B93F-6FC31620A46C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68BA3D5-EAEF-4FA2-BD3B-4F40FE5BC770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28830" yWindow="4710" windowWidth="20460" windowHeight="10770" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="107">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="109">
   <si>
     <t>Area</t>
   </si>
@@ -344,6 +344,12 @@
   </si>
   <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
+  </si>
+  <si>
+    <t>SEGUIMIENTO DE OBJETIVOS</t>
+  </si>
+  <si>
+    <t>https://objetivos-hergo.vercel.app/</t>
   </si>
 </sst>
 </file>
@@ -672,7 +678,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E40"/>
+  <dimension ref="A1:E41"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -1297,6 +1303,20 @@
       </c>
       <c r="D40" t="s">
         <v>106</v>
+      </c>
+    </row>
+    <row r="41" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A41" t="s">
+        <v>4</v>
+      </c>
+      <c r="B41" t="s">
+        <v>5</v>
+      </c>
+      <c r="C41" t="s">
+        <v>107</v>
+      </c>
+      <c r="D41" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-03 08:27)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,18 +5,18 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\layla\Documentos\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A68BA3D5-EAEF-4FA2-BD3B-4F40FE5BC770}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BB32EB-116B-4EF7-A080-06B46228BF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="20370" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$E$38</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$E$39</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
@@ -313,9 +313,6 @@
     <t>https://reporteventashtml.vercel.app/</t>
   </si>
   <si>
-    <t>REPORTE DE VENTAS 07-2026</t>
-  </si>
-  <si>
     <t>https://app.powerbi.com/reportEmbed?reportId=4900a270-06ee-458b-9793-2f98b3644748&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
   <si>
@@ -350,6 +347,9 @@
   </si>
   <si>
     <t>https://objetivos-hergo.vercel.app/</t>
+  </si>
+  <si>
+    <t>REPORTE DE VENTAS</t>
   </si>
 </sst>
 </file>
@@ -713,10 +713,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
-        <v>6</v>
+        <v>106</v>
       </c>
       <c r="D2" t="s">
-        <v>7</v>
+        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -727,10 +727,10 @@
         <v>5</v>
       </c>
       <c r="C3" t="s">
-        <v>96</v>
+        <v>6</v>
       </c>
       <c r="D3" t="s">
-        <v>95</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.25">
@@ -741,10 +741,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>8</v>
+        <v>108</v>
       </c>
       <c r="D4" t="s">
-        <v>9</v>
+        <v>95</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -752,13 +752,13 @@
         <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C5" t="s">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="D5" t="s">
-        <v>12</v>
+        <v>9</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.25">
@@ -769,10 +769,10 @@
         <v>10</v>
       </c>
       <c r="C6" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="D6" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.25">
@@ -780,13 +780,13 @@
         <v>4</v>
       </c>
       <c r="B7" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C7" t="s">
-        <v>15</v>
+        <v>13</v>
       </c>
       <c r="D7" t="s">
-        <v>16</v>
+        <v>14</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.25">
@@ -797,10 +797,10 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D8" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -811,10 +811,10 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D9" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -825,10 +825,10 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D10" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -839,10 +839,10 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D11" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -853,10 +853,10 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D12" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -867,10 +867,10 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D13" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -881,10 +881,10 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D14" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -895,10 +895,10 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D15" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -906,16 +906,13 @@
         <v>4</v>
       </c>
       <c r="B16" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D16" t="s">
-        <v>35</v>
-      </c>
-      <c r="E16" t="s">
-        <v>100</v>
+        <v>32</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -923,13 +920,16 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C17" t="s">
-        <v>36</v>
+        <v>34</v>
       </c>
       <c r="D17" t="s">
-        <v>37</v>
+        <v>35</v>
+      </c>
+      <c r="E17" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -937,16 +937,13 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C18" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="D18" t="s">
-        <v>39</v>
-      </c>
-      <c r="E18" t="s">
-        <v>101</v>
+        <v>37</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -954,13 +951,16 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C19" t="s">
-        <v>40</v>
+        <v>38</v>
       </c>
       <c r="D19" t="s">
-        <v>41</v>
+        <v>39</v>
+      </c>
+      <c r="E19" t="s">
+        <v>100</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -971,10 +971,10 @@
         <v>5</v>
       </c>
       <c r="C20" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="D20" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -985,10 +985,10 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>44</v>
+        <v>42</v>
       </c>
       <c r="D21" t="s">
-        <v>45</v>
+        <v>43</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -999,10 +999,10 @@
         <v>5</v>
       </c>
       <c r="C22" t="s">
-        <v>46</v>
+        <v>44</v>
       </c>
       <c r="D22" t="s">
-        <v>47</v>
+        <v>45</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1010,33 +1010,30 @@
         <v>4</v>
       </c>
       <c r="B23" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>48</v>
+        <v>46</v>
       </c>
       <c r="D23" t="s">
-        <v>49</v>
-      </c>
-      <c r="E23" t="s">
-        <v>102</v>
+        <v>47</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>73</v>
+        <v>33</v>
       </c>
       <c r="C24" t="s">
-        <v>50</v>
-      </c>
-      <c r="D24" s="1" t="s">
-        <v>61</v>
+        <v>48</v>
+      </c>
+      <c r="D24" t="s">
+        <v>49</v>
       </c>
       <c r="E24" t="s">
-        <v>77</v>
+        <v>101</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
@@ -1047,30 +1044,30 @@
         <v>73</v>
       </c>
       <c r="C25" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="E25" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B26" t="s">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="C26" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="E26" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
@@ -1081,10 +1078,10 @@
         <v>5</v>
       </c>
       <c r="C27" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="E27" t="s">
         <v>79</v>
@@ -1092,19 +1089,19 @@
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="E28" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
@@ -1115,47 +1112,47 @@
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="E29" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>74</v>
+        <v>89</v>
       </c>
       <c r="B30" t="s">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="E30" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B31" t="s">
         <v>74</v>
       </c>
       <c r="C31" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="E31" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
@@ -1163,50 +1160,50 @@
         <v>75</v>
       </c>
       <c r="B32" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C32" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="E32" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B33" t="s">
-        <v>5</v>
+        <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>54</v>
+        <v>58</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="E33" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="B34" t="s">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="C34" t="s">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="E34" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1217,13 +1214,13 @@
         <v>73</v>
       </c>
       <c r="C35" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="E35" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
@@ -1234,13 +1231,13 @@
         <v>73</v>
       </c>
       <c r="C36" t="s">
-        <v>92</v>
+        <v>60</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="E36" t="s">
-        <v>94</v>
+        <v>87</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
@@ -1251,10 +1248,10 @@
         <v>73</v>
       </c>
       <c r="C37" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="E37" t="s">
         <v>94</v>
@@ -1262,19 +1259,19 @@
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>4</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>33</v>
+        <v>73</v>
       </c>
       <c r="C38" t="s">
-        <v>98</v>
-      </c>
-      <c r="D38" t="s">
-        <v>97</v>
+        <v>93</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>91</v>
       </c>
       <c r="E38" t="s">
-        <v>99</v>
+        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
@@ -1282,13 +1279,16 @@
         <v>4</v>
       </c>
       <c r="B39" t="s">
-        <v>5</v>
+        <v>33</v>
       </c>
       <c r="C39" t="s">
-        <v>104</v>
+        <v>97</v>
       </c>
       <c r="D39" t="s">
-        <v>103</v>
+        <v>96</v>
+      </c>
+      <c r="E39" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1296,13 +1296,13 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C40" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="D40" t="s">
-        <v>106</v>
+        <v>102</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1310,31 +1310,31 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C41" t="s">
-        <v>107</v>
+        <v>104</v>
       </c>
       <c r="D41" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D25" r:id="rId1" xr:uid="{3C331869-98F3-4B87-ADF4-988275037827}"/>
-    <hyperlink ref="D24" r:id="rId2" xr:uid="{C8EAE465-89E0-4628-B2F4-6BE05A058D61}"/>
-    <hyperlink ref="D26" r:id="rId3" xr:uid="{75879039-BAE6-4CF6-AF43-763E9ECF0BD7}"/>
-    <hyperlink ref="D27" r:id="rId4" xr:uid="{DD4E29F3-166F-493E-8A70-5618EF533237}"/>
-    <hyperlink ref="D28" r:id="rId5" xr:uid="{25941851-C2B0-46ED-A55A-A06791D0EE0F}"/>
-    <hyperlink ref="D29" r:id="rId6" xr:uid="{E18B7B62-B80E-48E0-A060-6504BBB826E5}"/>
-    <hyperlink ref="D30" r:id="rId7" xr:uid="{58882F6E-9D0E-44A6-8F3D-AA3F518FC470}"/>
-    <hyperlink ref="D31" r:id="rId8" xr:uid="{AEF67EE1-A7B2-4C96-AD8F-EB9A98A208FD}"/>
-    <hyperlink ref="D32" r:id="rId9" xr:uid="{E10D50A9-A10A-45D2-A783-C335928BADAD}"/>
-    <hyperlink ref="D33" r:id="rId10" xr:uid="{A0AC4C5E-2431-4290-9E22-334EFC1ADF2A}"/>
-    <hyperlink ref="D34" r:id="rId11" xr:uid="{1AE79520-3345-461B-A674-520AF8AF695A}"/>
-    <hyperlink ref="D35" r:id="rId12" xr:uid="{DE513581-C953-4F03-BD77-004288A420F8}"/>
-    <hyperlink ref="D36" r:id="rId13" xr:uid="{3FA9E1C7-24BA-46D5-AA2E-C46322543BB7}"/>
-    <hyperlink ref="D37" r:id="rId14" xr:uid="{E380CBA2-725F-49CA-92A2-8FF6AC19AE29}"/>
+    <hyperlink ref="D26" r:id="rId1" xr:uid="{3C331869-98F3-4B87-ADF4-988275037827}"/>
+    <hyperlink ref="D25" r:id="rId2" xr:uid="{C8EAE465-89E0-4628-B2F4-6BE05A058D61}"/>
+    <hyperlink ref="D27" r:id="rId3" xr:uid="{75879039-BAE6-4CF6-AF43-763E9ECF0BD7}"/>
+    <hyperlink ref="D28" r:id="rId4" xr:uid="{DD4E29F3-166F-493E-8A70-5618EF533237}"/>
+    <hyperlink ref="D29" r:id="rId5" xr:uid="{25941851-C2B0-46ED-A55A-A06791D0EE0F}"/>
+    <hyperlink ref="D30" r:id="rId6" xr:uid="{E18B7B62-B80E-48E0-A060-6504BBB826E5}"/>
+    <hyperlink ref="D31" r:id="rId7" xr:uid="{58882F6E-9D0E-44A6-8F3D-AA3F518FC470}"/>
+    <hyperlink ref="D32" r:id="rId8" xr:uid="{AEF67EE1-A7B2-4C96-AD8F-EB9A98A208FD}"/>
+    <hyperlink ref="D33" r:id="rId9" xr:uid="{E10D50A9-A10A-45D2-A783-C335928BADAD}"/>
+    <hyperlink ref="D34" r:id="rId10" xr:uid="{A0AC4C5E-2431-4290-9E22-334EFC1ADF2A}"/>
+    <hyperlink ref="D35" r:id="rId11" xr:uid="{1AE79520-3345-461B-A674-520AF8AF695A}"/>
+    <hyperlink ref="D36" r:id="rId12" xr:uid="{DE513581-C953-4F03-BD77-004288A420F8}"/>
+    <hyperlink ref="D37" r:id="rId13" xr:uid="{3FA9E1C7-24BA-46D5-AA2E-C46322543BB7}"/>
+    <hyperlink ref="D38" r:id="rId14" xr:uid="{E380CBA2-725F-49CA-92A2-8FF6AC19AE29}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>

</xml_diff>

<commit_message>
Agrego marca de agua RTM en el pie y actualizo tableros
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,12 +5,12 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\layla\Documentos\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{04BB32EB-116B-4EF7-A080-06B46228BF48}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10723C29-170B-4D95-B52B-1066B36FBF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -23,7 +23,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="183" uniqueCount="109">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="111">
   <si>
     <t>Area</t>
   </si>
@@ -350,6 +350,12 @@
   </si>
   <si>
     <t>REPORTE DE VENTAS</t>
+  </si>
+  <si>
+    <t>https://app.powerbi.com/reportEmbed?reportId=c6e72043-9449-4d47-992c-d5e6075ec51d&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
+  </si>
+  <si>
+    <t>COMPARATIVO 08-2026</t>
   </si>
 </sst>
 </file>
@@ -394,9 +400,12 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Hipervínculo" xfId="1" builtinId="8"/>
@@ -678,7 +687,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E41"/>
+  <dimension ref="A1:E42"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -1317,6 +1326,20 @@
       </c>
       <c r="D41" t="s">
         <v>105</v>
+      </c>
+    </row>
+    <row r="42" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A42" t="s">
+        <v>4</v>
+      </c>
+      <c r="B42" t="s">
+        <v>5</v>
+      </c>
+      <c r="C42" t="s">
+        <v>110</v>
+      </c>
+      <c r="D42" s="2" t="s">
+        <v>109</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-19 10:00)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -5,25 +5,25 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\layla\Documentos\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{10723C29-170B-4D95-B52B-1066B36FBF8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{99A2E2FC-CC0C-4687-A5DF-C80FD93B121A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Hoja1!$A$1:$E$40</definedName>
   </definedNames>
   <calcPr calcId="181029"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="187" uniqueCount="111">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="191" uniqueCount="113">
   <si>
     <t>Area</t>
   </si>
@@ -121,9 +121,6 @@
     <t>MARGENES MAYORISTA</t>
   </si>
   <si>
-    <t>https://app.powerbi.com/reportEmbed?reportId=b1e55ab9-59ad-478d-8347-d9f4b4fac173&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
-  </si>
-  <si>
     <t>MENOR COSTE</t>
   </si>
   <si>
@@ -356,6 +353,15 @@
   </si>
   <si>
     <t>COMPARATIVO 08-2026</t>
+  </si>
+  <si>
+    <t>CONSUMOS DE CLIENTES</t>
+  </si>
+  <si>
+    <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
+  </si>
+  <si>
+    <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true&amp;ctid=2c7a392d-4df9-434a-859c-2f6bb1519f7a</t>
   </si>
 </sst>
 </file>
@@ -687,7 +693,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:E42"/>
+  <dimension ref="A1:E43"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="21.42578125" bestFit="1" customWidth="1"/>
@@ -711,7 +717,7 @@
         <v>3</v>
       </c>
       <c r="E1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.25">
@@ -722,10 +728,10 @@
         <v>5</v>
       </c>
       <c r="C2" t="s">
+        <v>105</v>
+      </c>
+      <c r="D2" t="s">
         <v>106</v>
-      </c>
-      <c r="D2" t="s">
-        <v>107</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.25">
@@ -750,10 +756,10 @@
         <v>5</v>
       </c>
       <c r="C4" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="D4" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.25">
@@ -806,10 +812,10 @@
         <v>5</v>
       </c>
       <c r="C8" t="s">
-        <v>15</v>
+        <v>110</v>
       </c>
       <c r="D8" t="s">
-        <v>16</v>
+        <v>111</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.25">
@@ -820,10 +826,10 @@
         <v>5</v>
       </c>
       <c r="C9" t="s">
-        <v>17</v>
+        <v>15</v>
       </c>
       <c r="D9" t="s">
-        <v>18</v>
+        <v>16</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.25">
@@ -834,10 +840,10 @@
         <v>5</v>
       </c>
       <c r="C10" t="s">
-        <v>19</v>
+        <v>17</v>
       </c>
       <c r="D10" t="s">
-        <v>20</v>
+        <v>18</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.25">
@@ -848,10 +854,10 @@
         <v>5</v>
       </c>
       <c r="C11" t="s">
-        <v>21</v>
+        <v>19</v>
       </c>
       <c r="D11" t="s">
-        <v>22</v>
+        <v>20</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.25">
@@ -862,10 +868,10 @@
         <v>5</v>
       </c>
       <c r="C12" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="D12" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.25">
@@ -876,10 +882,10 @@
         <v>5</v>
       </c>
       <c r="C13" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="D13" t="s">
-        <v>26</v>
+        <v>24</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.25">
@@ -890,10 +896,10 @@
         <v>5</v>
       </c>
       <c r="C14" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="D14" t="s">
-        <v>28</v>
+        <v>26</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.25">
@@ -904,10 +910,10 @@
         <v>5</v>
       </c>
       <c r="C15" t="s">
-        <v>29</v>
+        <v>27</v>
       </c>
       <c r="D15" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.25">
@@ -918,10 +924,10 @@
         <v>5</v>
       </c>
       <c r="C16" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="D16" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.25">
@@ -929,16 +935,13 @@
         <v>4</v>
       </c>
       <c r="B17" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C17" t="s">
-        <v>34</v>
+        <v>31</v>
       </c>
       <c r="D17" t="s">
-        <v>35</v>
-      </c>
-      <c r="E17" t="s">
-        <v>99</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.25">
@@ -946,13 +949,16 @@
         <v>4</v>
       </c>
       <c r="B18" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C18" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="D18" t="s">
-        <v>37</v>
+        <v>34</v>
+      </c>
+      <c r="E18" t="s">
+        <v>98</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.25">
@@ -960,16 +966,13 @@
         <v>4</v>
       </c>
       <c r="B19" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C19" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="D19" t="s">
-        <v>39</v>
-      </c>
-      <c r="E19" t="s">
-        <v>100</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.25">
@@ -977,13 +980,16 @@
         <v>4</v>
       </c>
       <c r="B20" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C20" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="D20" t="s">
-        <v>41</v>
+        <v>38</v>
+      </c>
+      <c r="E20" t="s">
+        <v>99</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.25">
@@ -994,10 +1000,10 @@
         <v>5</v>
       </c>
       <c r="C21" t="s">
-        <v>42</v>
+        <v>39</v>
       </c>
       <c r="D21" t="s">
-        <v>43</v>
+        <v>40</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.25">
@@ -1008,10 +1014,10 @@
         <v>5</v>
       </c>
       <c r="C22" t="s">
-        <v>44</v>
+        <v>41</v>
       </c>
       <c r="D22" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.25">
@@ -1022,10 +1028,10 @@
         <v>5</v>
       </c>
       <c r="C23" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="D23" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.25">
@@ -1033,186 +1039,183 @@
         <v>4</v>
       </c>
       <c r="B24" t="s">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="C24" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D24" t="s">
-        <v>49</v>
-      </c>
-      <c r="E24" t="s">
-        <v>101</v>
+        <v>46</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>75</v>
+        <v>4</v>
       </c>
       <c r="B25" t="s">
-        <v>73</v>
+        <v>32</v>
       </c>
       <c r="C25" t="s">
-        <v>50</v>
-      </c>
-      <c r="D25" s="1" t="s">
-        <v>61</v>
+        <v>47</v>
+      </c>
+      <c r="D25" t="s">
+        <v>48</v>
       </c>
       <c r="E25" t="s">
-        <v>77</v>
+        <v>100</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C26" t="s">
-        <v>51</v>
+        <v>49</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>62</v>
+        <v>60</v>
       </c>
       <c r="E26" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B27" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="C27" t="s">
-        <v>52</v>
+        <v>50</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="E27" t="s">
-        <v>79</v>
+        <v>77</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A28" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B28" t="s">
         <v>5</v>
       </c>
       <c r="C28" t="s">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>64</v>
+        <v>62</v>
       </c>
       <c r="E28" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A29" t="s">
-        <v>89</v>
+        <v>75</v>
       </c>
       <c r="B29" t="s">
         <v>5</v>
       </c>
       <c r="C29" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>65</v>
+        <v>63</v>
       </c>
       <c r="E29" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A30" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B30" t="s">
         <v>5</v>
       </c>
       <c r="C30" t="s">
-        <v>55</v>
+        <v>53</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>66</v>
+        <v>64</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>79</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A31" t="s">
-        <v>74</v>
+        <v>88</v>
       </c>
       <c r="B31" t="s">
-        <v>74</v>
+        <v>5</v>
       </c>
       <c r="C31" t="s">
-        <v>56</v>
+        <v>54</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="E31" t="s">
-        <v>82</v>
+        <v>80</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A32" t="s">
-        <v>75</v>
+        <v>73</v>
       </c>
       <c r="B32" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C32" t="s">
-        <v>57</v>
+        <v>55</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="E32" t="s">
-        <v>83</v>
+        <v>81</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A33" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B33" t="s">
         <v>73</v>
       </c>
       <c r="C33" t="s">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="E33" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A34" t="s">
-        <v>76</v>
+        <v>74</v>
       </c>
       <c r="B34" t="s">
-        <v>5</v>
+        <v>72</v>
       </c>
       <c r="C34" t="s">
-        <v>54</v>
+        <v>57</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="E34" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.25">
@@ -1220,84 +1223,84 @@
         <v>75</v>
       </c>
       <c r="B35" t="s">
-        <v>73</v>
+        <v>5</v>
       </c>
       <c r="C35" t="s">
-        <v>59</v>
+        <v>53</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="E35" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A36" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B36" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C36" t="s">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="E36" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A37" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B37" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>59</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>90</v>
+        <v>71</v>
       </c>
       <c r="E37" t="s">
-        <v>94</v>
+        <v>86</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A38" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B38" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C38" t="s">
+        <v>91</v>
+      </c>
+      <c r="D38" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="E38" t="s">
         <v>93</v>
-      </c>
-      <c r="D38" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="E38" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.25">
       <c r="A39" t="s">
-        <v>4</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
-        <v>33</v>
+        <v>72</v>
       </c>
       <c r="C39" t="s">
-        <v>97</v>
-      </c>
-      <c r="D39" t="s">
-        <v>96</v>
+        <v>92</v>
+      </c>
+      <c r="D39" s="1" t="s">
+        <v>90</v>
       </c>
       <c r="E39" t="s">
-        <v>98</v>
+        <v>93</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.25">
@@ -1305,13 +1308,16 @@
         <v>4</v>
       </c>
       <c r="B40" t="s">
-        <v>5</v>
+        <v>32</v>
       </c>
       <c r="C40" t="s">
-        <v>103</v>
+        <v>96</v>
       </c>
       <c r="D40" t="s">
-        <v>102</v>
+        <v>95</v>
+      </c>
+      <c r="E40" t="s">
+        <v>97</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.25">
@@ -1319,13 +1325,13 @@
         <v>4</v>
       </c>
       <c r="B41" t="s">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="C41" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
-        <v>105</v>
+        <v>101</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.25">
@@ -1333,31 +1339,45 @@
         <v>4</v>
       </c>
       <c r="B42" t="s">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="C42" t="s">
-        <v>110</v>
-      </c>
-      <c r="D42" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="D42" t="s">
+        <v>104</v>
+      </c>
+    </row>
+    <row r="43" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A43" t="s">
+        <v>4</v>
+      </c>
+      <c r="B43" t="s">
+        <v>5</v>
+      </c>
+      <c r="C43" t="s">
         <v>109</v>
+      </c>
+      <c r="D43" s="2" t="s">
+        <v>108</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="D26" r:id="rId1" xr:uid="{3C331869-98F3-4B87-ADF4-988275037827}"/>
-    <hyperlink ref="D25" r:id="rId2" xr:uid="{C8EAE465-89E0-4628-B2F4-6BE05A058D61}"/>
-    <hyperlink ref="D27" r:id="rId3" xr:uid="{75879039-BAE6-4CF6-AF43-763E9ECF0BD7}"/>
-    <hyperlink ref="D28" r:id="rId4" xr:uid="{DD4E29F3-166F-493E-8A70-5618EF533237}"/>
-    <hyperlink ref="D29" r:id="rId5" xr:uid="{25941851-C2B0-46ED-A55A-A06791D0EE0F}"/>
-    <hyperlink ref="D30" r:id="rId6" xr:uid="{E18B7B62-B80E-48E0-A060-6504BBB826E5}"/>
-    <hyperlink ref="D31" r:id="rId7" xr:uid="{58882F6E-9D0E-44A6-8F3D-AA3F518FC470}"/>
-    <hyperlink ref="D32" r:id="rId8" xr:uid="{AEF67EE1-A7B2-4C96-AD8F-EB9A98A208FD}"/>
-    <hyperlink ref="D33" r:id="rId9" xr:uid="{E10D50A9-A10A-45D2-A783-C335928BADAD}"/>
-    <hyperlink ref="D34" r:id="rId10" xr:uid="{A0AC4C5E-2431-4290-9E22-334EFC1ADF2A}"/>
-    <hyperlink ref="D35" r:id="rId11" xr:uid="{1AE79520-3345-461B-A674-520AF8AF695A}"/>
-    <hyperlink ref="D36" r:id="rId12" xr:uid="{DE513581-C953-4F03-BD77-004288A420F8}"/>
-    <hyperlink ref="D37" r:id="rId13" xr:uid="{3FA9E1C7-24BA-46D5-AA2E-C46322543BB7}"/>
-    <hyperlink ref="D38" r:id="rId14" xr:uid="{E380CBA2-725F-49CA-92A2-8FF6AC19AE29}"/>
+    <hyperlink ref="D27" r:id="rId1" xr:uid="{3C331869-98F3-4B87-ADF4-988275037827}"/>
+    <hyperlink ref="D26" r:id="rId2" xr:uid="{C8EAE465-89E0-4628-B2F4-6BE05A058D61}"/>
+    <hyperlink ref="D28" r:id="rId3" xr:uid="{75879039-BAE6-4CF6-AF43-763E9ECF0BD7}"/>
+    <hyperlink ref="D29" r:id="rId4" xr:uid="{DD4E29F3-166F-493E-8A70-5618EF533237}"/>
+    <hyperlink ref="D30" r:id="rId5" xr:uid="{25941851-C2B0-46ED-A55A-A06791D0EE0F}"/>
+    <hyperlink ref="D31" r:id="rId6" xr:uid="{E18B7B62-B80E-48E0-A060-6504BBB826E5}"/>
+    <hyperlink ref="D32" r:id="rId7" xr:uid="{58882F6E-9D0E-44A6-8F3D-AA3F518FC470}"/>
+    <hyperlink ref="D33" r:id="rId8" xr:uid="{AEF67EE1-A7B2-4C96-AD8F-EB9A98A208FD}"/>
+    <hyperlink ref="D34" r:id="rId9" xr:uid="{E10D50A9-A10A-45D2-A783-C335928BADAD}"/>
+    <hyperlink ref="D35" r:id="rId10" xr:uid="{A0AC4C5E-2431-4290-9E22-334EFC1ADF2A}"/>
+    <hyperlink ref="D36" r:id="rId11" xr:uid="{1AE79520-3345-461B-A674-520AF8AF695A}"/>
+    <hyperlink ref="D37" r:id="rId12" xr:uid="{DE513581-C953-4F03-BD77-004288A420F8}"/>
+    <hyperlink ref="D38" r:id="rId13" xr:uid="{3FA9E1C7-24BA-46D5-AA2E-C46322543BB7}"/>
+    <hyperlink ref="D39" r:id="rId14" xr:uid="{E380CBA2-725F-49CA-92A2-8FF6AC19AE29}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId15"/>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-25 15:34)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$G$156</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$K$220</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$156</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$220</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G156"/>
+  <dimension ref="A1:H156"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -445,6 +445,7 @@
     <col width="45" customWidth="1" min="5" max="5"/>
     <col width="9" customWidth="1" min="6" max="6"/>
     <col width="9" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -483,6 +484,11 @@
           <t>Tipo</t>
         </is>
       </c>
+      <c r="H1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -516,6 +522,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -549,6 +556,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -586,6 +594,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -623,6 +632,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -660,6 +670,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -697,6 +708,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -734,6 +746,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -771,6 +784,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -808,6 +822,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -845,6 +860,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -882,6 +898,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -919,6 +936,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -956,6 +974,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -993,6 +1012,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -1030,6 +1050,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -1067,6 +1088,7 @@
           <t>APP</t>
         </is>
       </c>
+      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -1100,6 +1122,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1133,6 +1156,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1166,6 +1190,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1199,6 +1224,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1232,6 +1258,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1265,6 +1292,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1298,6 +1326,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1331,6 +1360,7 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1364,6 +1394,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1397,6 +1430,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1430,6 +1466,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1463,6 +1502,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1496,6 +1538,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1529,6 +1574,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -1562,6 +1610,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H32" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -1595,6 +1646,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H33" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -1628,6 +1682,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H34" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -1661,6 +1718,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H35" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -1694,6 +1754,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -1727,6 +1790,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -1760,6 +1826,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -1793,6 +1862,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H39" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -1826,6 +1898,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -1859,6 +1934,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H41" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -1873,12 +1951,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CACEROLA</t>
+          <t>SITUACION FINANCIERA</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7ed33ee7-275e-4af5-8ddc-3e67ce01ce50&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1892,6 +1970,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H42" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -1925,6 +2006,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H43" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -1939,12 +2023,12 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>SITUACION FINANCIERA</t>
+          <t>CACEROLA</t>
         </is>
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7ed33ee7-275e-4af5-8ddc-3e67ce01ce50&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ef4634d6-33e3-4dc4-a17c-6bd0b81ec138&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E44" t="inlineStr"/>
@@ -1958,6 +2042,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H44" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -1972,12 +2059,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>VISITAS - RESUMEN DIARIO MAYORISTA</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=01100552-0f0b-461b-9327-4bc164c5f331&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -1991,6 +2078,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H45" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -2005,12 +2095,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2024,6 +2114,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H46" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -2038,12 +2131,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=402b5c26-c94e-44f2-958b-e71cb071ff31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2057,6 +2150,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H47" t="n">
+        <v>60</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -2071,12 +2167,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>COMPARATIVO 07-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=402b5c26-c94e-44f2-958b-e71cb071ff31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2090,6 +2186,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H48" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -2104,12 +2203,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2123,6 +2222,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H49" t="n">
+        <v>57</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -2137,12 +2239,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2156,6 +2258,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H50" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -2170,12 +2275,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2189,6 +2294,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H51" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -2203,12 +2311,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ba02793b-9173-406b-b100-198d9dbaae73&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2222,6 +2330,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H52" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -2236,12 +2347,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>INCENTIVOS ALTA</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=66f1d933-90ed-49d1-89e5-dbb9e765b851&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2255,6 +2366,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H53" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -2269,12 +2383,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2288,6 +2402,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H54" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -2302,12 +2419,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2321,6 +2438,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H55" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -2335,12 +2455,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2354,6 +2474,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H56" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -2368,12 +2491,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>PRECIOS Y OFERTAS DISTR</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=74da6bde-8f40-4f5a-881e-c79da99f35a1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2387,6 +2510,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H57" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -2401,12 +2527,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=66f1d933-90ed-49d1-89e5-dbb9e765b851&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2420,6 +2546,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H58" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -2434,12 +2563,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cf82ea28-f534-4da8-9786-e89dba954b17&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2453,6 +2582,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H59" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -2467,12 +2599,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>INCENTIVOS BLACK</t>
+          <t>EFECTIVIDADES</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fee017c6-a239-4e81-987a-fede32524903&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ba02793b-9173-406b-b100-198d9dbaae73&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2486,6 +2618,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H60" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -2500,12 +2635,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9e51941e-8703-4d9c-814e-c80d8be9fde2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2519,6 +2654,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H61" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -2533,12 +2671,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCENTIVOS BLACK</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fee017c6-a239-4e81-987a-fede32524903&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2552,6 +2690,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H62" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -2566,12 +2707,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>OFERTAS DESEMPEÑO</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a22fe5fb-0b92-436c-b710-db69d8ea7c47&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2585,6 +2726,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H63" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -2599,12 +2743,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4bdda3e7-2a7d-4b74-a484-4551b4873c03&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2618,6 +2762,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H64" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -2632,12 +2779,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2651,6 +2798,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H65" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" t="inlineStr">
@@ -2665,12 +2815,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>OFERTAS DESEMPEÑO</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a22fe5fb-0b92-436c-b710-db69d8ea7c47&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2684,6 +2834,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H66" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
@@ -2698,12 +2851,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 06-2025</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -2717,6 +2870,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H67" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="68">
       <c r="A68" t="inlineStr">
@@ -2731,12 +2887,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ed3b5a8c-8ac6-4d65-8961-df938488eb29&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -2750,6 +2906,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H68" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" t="inlineStr">
@@ -2764,12 +2923,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>PRECIOS Y OFERTAS DISTR</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=74da6bde-8f40-4f5a-881e-c79da99f35a1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -2783,6 +2942,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H69" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="70">
       <c r="A70" t="inlineStr">
@@ -2797,12 +2959,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>PRESUPUESTO MARKETING</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cf5e22c9-8925-4779-8f00-d8de2fa957eb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cf82ea28-f534-4da8-9786-e89dba954b17&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -2816,6 +2978,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H70" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
@@ -2830,12 +2995,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE OFERTAS</t>
+          <t>INCENTIVOS COUSTLAIN</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=467411be-b152-4571-aab6-634eb4bf23fc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9e51941e-8703-4d9c-814e-c80d8be9fde2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -2849,6 +3014,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" t="inlineStr">
@@ -2863,12 +3031,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8cc08bae-0659-4b71-af6a-b3f830c2d9c8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -2882,6 +3050,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" t="inlineStr">
@@ -2896,12 +3067,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>PARTICIPACION VENTAS CCU 06-2025</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=2271183e-fad9-4f2f-94a4-656ddc3e2327&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -2915,6 +3086,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H73" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -2929,12 +3103,12 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D74" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ed3b5a8c-8ac6-4d65-8961-df938488eb29&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E74" t="inlineStr"/>
@@ -2948,6 +3122,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -2962,12 +3139,12 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>PRESUPUESTO MARKETING</t>
         </is>
       </c>
       <c r="D75" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cf5e22c9-8925-4779-8f00-d8de2fa957eb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E75" t="inlineStr"/>
@@ -2981,6 +3158,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -2995,12 +3175,12 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>SEGUIMIENTO DE OFERTAS</t>
         </is>
       </c>
       <c r="D76" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4bdda3e7-2a7d-4b74-a484-4551b4873c03&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=467411be-b152-4571-aab6-634eb4bf23fc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E76" t="inlineStr"/>
@@ -3014,6 +3194,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" t="inlineStr">
@@ -3028,12 +3211,12 @@
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="D77" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8cc08bae-0659-4b71-af6a-b3f830c2d9c8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E77" t="inlineStr"/>
@@ -3047,6 +3230,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" t="inlineStr">
@@ -3061,12 +3247,12 @@
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>VISITAS - RESUMEN DIARIO MAYORISTA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D78" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=01100552-0f0b-461b-9327-4bc164c5f331&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=2271183e-fad9-4f2f-94a4-656ddc3e2327&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E78" t="inlineStr"/>
@@ -3080,6 +3266,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" t="inlineStr">
@@ -3094,17 +3283,17 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>MARGENES MC</t>
+          <t>REPORTE DE VENTAS MC</t>
         </is>
       </c>
       <c r="D79" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c189c73d-9a18-477b-8c39-c855849020d0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d290f1bf-00d9-41de-aae8-0006cd919e4e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>Analiza la rentabilidad de las ventas: margen $ y % por sucursal, sección, rubro, línea, proveedor y artículo. Cruza facturación, importe s/IVA, costo, descuentos y mermas para mostrar dónde se gana y dónde se pierde rentabilidad.</t>
+          <t>Reporte transaccional de ventas: unidades, venta neta e importes por sucursal, sección, línea, rubro, medio de pago y fecha, con serie histórica de +15 meses.</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
@@ -3116,6 +3305,9 @@
         <is>
           <t>INFORME</t>
         </is>
+      </c>
+      <c r="H79" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="80">
@@ -3131,17 +3323,17 @@
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>MARGENES MC</t>
         </is>
       </c>
       <c r="D80" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c189c73d-9a18-477b-8c39-c855849020d0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E80" t="inlineStr">
         <is>
-          <t>Controla las pérdidas de mercadería (roturas, vencimientos) en unidades y valorizadas, por sucursal, sección y artículo.</t>
+          <t>Analiza la rentabilidad de las ventas: margen $ y % por sucursal, sección, rubro, línea, proveedor y artículo. Cruza facturación, importe s/IVA, costo, descuentos y mermas para mostrar dónde se gana y dónde se pierde rentabilidad.</t>
         </is>
       </c>
       <c r="F80" t="inlineStr">
@@ -3153,6 +3345,9 @@
         <is>
           <t>INFORME</t>
         </is>
+      </c>
+      <c r="H80" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="81">
@@ -3168,15 +3363,19 @@
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D81" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=48b6a50f-e36a-4be6-9fe5-ba74ff2c0afc&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E81" t="inlineStr"/>
+          <t>https://app.powerbi.com/reportEmbed?reportId=dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E81" t="inlineStr">
+        <is>
+          <t>Controla las pérdidas de mercadería (roturas, vencimientos) en unidades y valorizadas, por sucursal, sección y artículo.</t>
+        </is>
+      </c>
       <c r="F81" t="inlineStr">
         <is>
           <t>API</t>
@@ -3186,6 +3385,9 @@
         <is>
           <t>INFORME</t>
         </is>
+      </c>
+      <c r="H81" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="82">
@@ -3201,17 +3403,17 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>REPORTE DE VENTAS MC</t>
+          <t>STOCK VALORIZADO MENOR COSTE</t>
         </is>
       </c>
       <c r="D82" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d290f1bf-00d9-41de-aae8-0006cd919e4e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4900a270-06ee-458b-9793-2f98b3644748&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E82" t="inlineStr">
         <is>
-          <t>Reporte transaccional de ventas: unidades, venta neta e importes por sucursal, sección, línea, rubro, medio de pago y fecha, con serie histórica de +15 meses.</t>
+          <t>Dashboard con el stock valorizado de las sucursales de menor coste y los dias de stock por seccion/linea/producto</t>
         </is>
       </c>
       <c r="F82" t="inlineStr">
@@ -3223,6 +3425,9 @@
         <is>
           <t>INFORME</t>
         </is>
+      </c>
+      <c r="H82" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="83">
@@ -3238,19 +3443,15 @@
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MENOR COSTE</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D83" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4900a270-06ee-458b-9793-2f98b3644748&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E83" t="inlineStr">
-        <is>
-          <t>Dashboard con el stock valorizado de las sucursales de menor coste y los dias de stock por seccion/linea/producto</t>
-        </is>
-      </c>
+          <t>https://app.powerbi.com/reportEmbed?reportId=48b6a50f-e36a-4be6-9fe5-ba74ff2c0afc&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E83" t="inlineStr"/>
       <c r="F83" t="inlineStr">
         <is>
           <t>API</t>
@@ -3260,6 +3461,9 @@
         <is>
           <t>INFORME</t>
         </is>
+      </c>
+      <c r="H83" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="84">
@@ -3294,6 +3498,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" t="inlineStr">
@@ -3327,6 +3534,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" t="inlineStr">
@@ -3360,6 +3570,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" t="inlineStr">
@@ -3393,6 +3606,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" t="inlineStr">
@@ -3426,6 +3642,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H88" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" t="inlineStr">
@@ -3459,6 +3678,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" t="inlineStr">
@@ -3492,6 +3714,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H90" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="91">
       <c r="A91" t="inlineStr">
@@ -3525,6 +3750,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H91" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" t="inlineStr">
@@ -3558,6 +3786,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H92" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" t="inlineStr">
@@ -3591,6 +3822,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H93" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="94">
       <c r="A94" t="inlineStr">
@@ -3624,6 +3858,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H94" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" t="inlineStr">
@@ -3657,6 +3894,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H95" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" t="inlineStr">
@@ -3690,6 +3930,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H96" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" t="inlineStr">
@@ -3723,6 +3966,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H97" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="98">
       <c r="A98" t="inlineStr">
@@ -3756,6 +4002,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H98" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" t="inlineStr">
@@ -3789,6 +4038,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" t="inlineStr">
@@ -3822,6 +4074,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" t="inlineStr">
@@ -3855,6 +4110,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" t="inlineStr">
@@ -3888,6 +4146,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" t="inlineStr">
@@ -3921,6 +4182,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" t="inlineStr">
@@ -3954,6 +4218,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" t="inlineStr">
@@ -3987,6 +4254,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" t="inlineStr">
@@ -4020,6 +4290,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" t="inlineStr">
@@ -4053,6 +4326,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" t="inlineStr">
@@ -4086,6 +4362,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" t="inlineStr">
@@ -4119,6 +4398,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H109" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="110">
       <c r="A110" t="inlineStr">
@@ -4152,6 +4434,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" t="inlineStr">
@@ -4185,6 +4470,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" t="inlineStr">
@@ -4218,6 +4506,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" t="inlineStr">
@@ -4251,6 +4542,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" t="inlineStr">
@@ -4284,6 +4578,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" t="inlineStr">
@@ -4317,6 +4614,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" t="inlineStr">
@@ -4350,6 +4650,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" t="inlineStr">
@@ -4383,6 +4686,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" t="inlineStr">
@@ -4416,6 +4722,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" t="inlineStr">
@@ -4449,6 +4758,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" t="inlineStr">
@@ -4482,6 +4794,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" t="inlineStr">
@@ -4515,6 +4830,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" t="inlineStr">
@@ -4548,6 +4866,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" t="inlineStr">
@@ -4581,6 +4902,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" t="inlineStr">
@@ -4614,6 +4938,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" t="inlineStr">
@@ -4647,6 +4974,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" t="inlineStr">
@@ -4680,6 +5010,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H126" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" t="inlineStr">
@@ -4713,6 +5046,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" t="inlineStr">
@@ -4746,6 +5082,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H128" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" t="inlineStr">
@@ -4779,6 +5118,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H129" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" t="inlineStr">
@@ -4812,6 +5154,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H130" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" t="inlineStr">
@@ -4845,6 +5190,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" t="inlineStr">
@@ -4878,6 +5226,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H132" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" t="inlineStr">
@@ -4911,6 +5262,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H133" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" t="inlineStr">
@@ -4944,6 +5298,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H134" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" t="inlineStr">
@@ -4977,6 +5334,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" t="inlineStr">
@@ -5010,6 +5370,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H136" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
@@ -5043,6 +5406,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H137" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
@@ -5076,6 +5442,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H138" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" t="inlineStr">
@@ -5109,6 +5478,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H139" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" t="inlineStr">
@@ -5142,6 +5514,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H140" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" t="inlineStr">
@@ -5175,6 +5550,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" t="inlineStr">
@@ -5208,6 +5586,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H142" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="143">
       <c r="A143" t="inlineStr">
@@ -5241,6 +5622,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H143" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" t="inlineStr">
@@ -5274,6 +5658,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H144" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" t="inlineStr">
@@ -5307,6 +5694,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H145" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" t="inlineStr">
@@ -5340,6 +5730,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H146" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" t="inlineStr">
@@ -5373,6 +5766,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -5406,6 +5802,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H148" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -5439,6 +5838,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -5472,6 +5874,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H150" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
@@ -5505,6 +5910,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H151" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" t="inlineStr">
@@ -5538,6 +5946,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H152" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" t="inlineStr">
@@ -5571,6 +5982,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
@@ -5604,6 +6018,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" t="inlineStr">
@@ -5637,6 +6054,9 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" t="inlineStr">
@@ -5670,9 +6090,12 @@
           <t>INFORME</t>
         </is>
       </c>
+      <c r="H156" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:G156"/>
+  <autoFilter ref="A1:H156"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5683,7 +6106,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K220"/>
+  <dimension ref="A1:L220"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -5697,6 +6120,7 @@
     <col width="16" customWidth="1" min="9" max="9"/>
     <col width="26" customWidth="1" min="10" max="10"/>
     <col width="38" customWidth="1" min="11" max="11"/>
+    <col width="8" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -5755,6 +6179,11 @@
           <t>reportId</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Vistas</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -5796,6 +6225,9 @@
           <t>e3a781e9-fe9b-4885-9e7d-8de8c003cfdd</t>
         </is>
       </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -5837,6 +6269,9 @@
           <t>c6276b41-9847-4111-82e8-146d32636229</t>
         </is>
       </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
@@ -5878,6 +6313,9 @@
           <t>a1d47f19-2c75-41f6-82e6-1bcf80289b8c</t>
         </is>
       </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -5919,6 +6357,9 @@
           <t>0411b9ac-d5bf-4e97-9b38-5d2fe2deb931</t>
         </is>
       </c>
+      <c r="L5" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="2" t="inlineStr">
@@ -5960,6 +6401,9 @@
           <t>0396d9e8-9644-4db9-867b-89d090fb95a3</t>
         </is>
       </c>
+      <c r="L6" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
@@ -6001,6 +6445,9 @@
           <t>e4b97365-464a-4d0f-812e-fc26afeaf650</t>
         </is>
       </c>
+      <c r="L7" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="2" t="inlineStr">
@@ -6042,6 +6489,9 @@
           <t>c1204b39-2269-43bc-935f-4525283b089e</t>
         </is>
       </c>
+      <c r="L8" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
@@ -6083,6 +6533,9 @@
           <t>5f8aa5de-6aa2-4988-9c94-be9e74274da5</t>
         </is>
       </c>
+      <c r="L9" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
@@ -6124,6 +6577,9 @@
           <t>d0552e68-9c0f-4d49-839f-f22fdc6c6f8e</t>
         </is>
       </c>
+      <c r="L10" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
@@ -6165,6 +6621,9 @@
           <t>b211b66a-e672-46e9-8c77-c5e12f4a48a4</t>
         </is>
       </c>
+      <c r="L11" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
@@ -6206,6 +6665,9 @@
           <t>116294d5-89b6-4122-9414-f0b870db64fd</t>
         </is>
       </c>
+      <c r="L12" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
@@ -6247,6 +6709,9 @@
           <t>8c1c6f46-8451-443e-a14d-2927530fd512</t>
         </is>
       </c>
+      <c r="L13" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
@@ -6288,6 +6753,9 @@
           <t>241c4fec-e190-4c24-9226-3b2781655a51</t>
         </is>
       </c>
+      <c r="L14" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
@@ -6329,6 +6797,9 @@
           <t>6d8bba6a-0f85-418a-a3de-a46559c081dd</t>
         </is>
       </c>
+      <c r="L15" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
@@ -6370,6 +6841,9 @@
           <t>362f0557-5f53-45e4-a162-67584d13a444</t>
         </is>
       </c>
+      <c r="L16" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
@@ -6411,6 +6885,9 @@
           <t>1e8b9fa1-30f3-4eba-966b-6804248342f7</t>
         </is>
       </c>
+      <c r="L17" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
@@ -6452,6 +6929,9 @@
           <t>18fd2917-e128-47d7-b930-81698225d577</t>
         </is>
       </c>
+      <c r="L18" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="2" t="inlineStr">
@@ -6493,6 +6973,9 @@
           <t>ef4634d6-33e3-4dc4-a17c-6bd0b81ec138</t>
         </is>
       </c>
+      <c r="L19" t="n">
+        <v>12</v>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="2" t="inlineStr">
@@ -6534,6 +7017,9 @@
           <t>e6339ca7-bf01-48b1-a5ce-930d679671a2</t>
         </is>
       </c>
+      <c r="L20" t="n">
+        <v>22</v>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="2" t="inlineStr">
@@ -6587,6 +7073,9 @@
           <t>e9341165-ec5f-48f9-abfd-d7fe80c14842</t>
         </is>
       </c>
+      <c r="L21" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="22">
       <c r="A22" s="2" t="inlineStr">
@@ -6640,6 +7129,9 @@
           <t>0a2ec774-224d-49f8-be1c-a0bf9568e471</t>
         </is>
       </c>
+      <c r="L22" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="23">
       <c r="A23" s="2" t="inlineStr">
@@ -6693,6 +7185,9 @@
           <t>e15c4cf7-8e43-4586-b5d6-3f23aa9e5738</t>
         </is>
       </c>
+      <c r="L23" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="A24" s="2" t="inlineStr">
@@ -6746,6 +7241,9 @@
           <t>9c210891-9419-44fd-8ba4-e3857e7d805b</t>
         </is>
       </c>
+      <c r="L24" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="25">
       <c r="A25" s="2" t="inlineStr">
@@ -6799,6 +7297,9 @@
           <t>0fe483f9-028b-417e-8ef5-8f93156abcbe</t>
         </is>
       </c>
+      <c r="L25" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="26">
       <c r="A26" s="2" t="inlineStr">
@@ -6852,6 +7353,9 @@
           <t>07f8cb25-b8f7-48a3-af1e-b5c1fd3e109f</t>
         </is>
       </c>
+      <c r="L26" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="27">
       <c r="A27" s="2" t="inlineStr">
@@ -6905,6 +7409,9 @@
           <t>9ece0bac-ba3c-4063-a0eb-03b231f021d5</t>
         </is>
       </c>
+      <c r="L27" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="28">
       <c r="A28" s="2" t="inlineStr">
@@ -6958,6 +7465,9 @@
           <t>d94dbbd9-6cd5-4c9a-94a4-4e5a8bc7c8a1</t>
         </is>
       </c>
+      <c r="L28" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="2" t="inlineStr">
@@ -7011,6 +7521,9 @@
           <t>3832edd0-03c0-4ff1-8a1f-abf56dd93932</t>
         </is>
       </c>
+      <c r="L29" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="30">
       <c r="A30" s="2" t="inlineStr">
@@ -7064,6 +7577,9 @@
           <t>20d7c15a-131e-4488-831e-d1fe0804779c</t>
         </is>
       </c>
+      <c r="L30" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="2" t="inlineStr">
@@ -7117,6 +7633,9 @@
           <t>ddc96523-0162-4bc1-8a67-c5b00e1a7b5c</t>
         </is>
       </c>
+      <c r="L31" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="32">
       <c r="A32" s="2" t="inlineStr">
@@ -7170,6 +7689,9 @@
           <t>7d56118f-e9a2-4439-af4e-3f6d4eb77929</t>
         </is>
       </c>
+      <c r="L32" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="33">
       <c r="A33" s="2" t="inlineStr">
@@ -7223,6 +7745,9 @@
           <t>e87b9f6f-d894-4e54-9353-f17aa155e82b</t>
         </is>
       </c>
+      <c r="L33" t="n">
+        <v>32</v>
+      </c>
     </row>
     <row r="34">
       <c r="A34" s="2" t="inlineStr">
@@ -7276,6 +7801,9 @@
           <t>402b5c26-c94e-44f2-958b-e71cb071ff31</t>
         </is>
       </c>
+      <c r="L34" t="n">
+        <v>25</v>
+      </c>
     </row>
     <row r="35">
       <c r="A35" s="2" t="inlineStr">
@@ -7328,6 +7856,9 @@
         <is>
           <t>4e0903c4-5dde-45ce-ad9f-6aed6e2a4136</t>
         </is>
+      </c>
+      <c r="L35" t="n">
+        <v>32</v>
       </c>
     </row>
     <row r="36">
@@ -7370,6 +7901,9 @@
           <t>b427136c-6785-4e5f-8e88-026b03a2bbe1</t>
         </is>
       </c>
+      <c r="L36" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" s="2" t="inlineStr">
@@ -7411,6 +7945,9 @@
           <t>45ca0371-6f94-430e-be96-2ec8fc691b21</t>
         </is>
       </c>
+      <c r="L37" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" s="2" t="inlineStr">
@@ -7452,6 +7989,9 @@
           <t>27dfaf71-9641-46a8-a9d2-21a7299ca705</t>
         </is>
       </c>
+      <c r="L38" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" s="2" t="inlineStr">
@@ -7493,6 +8033,9 @@
           <t>ba02793b-9173-406b-b100-198d9dbaae73</t>
         </is>
       </c>
+      <c r="L39" t="n">
+        <v>4</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" s="2" t="inlineStr">
@@ -7534,6 +8077,9 @@
           <t>899444c9-cd01-4bcf-b726-d4ae8d7fa432</t>
         </is>
       </c>
+      <c r="L40" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" s="2" t="inlineStr">
@@ -7575,6 +8121,9 @@
           <t>595175a9-fe3a-49ce-abde-bd1b578273ff</t>
         </is>
       </c>
+      <c r="L41" t="n">
+        <v>28</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" s="2" t="inlineStr">
@@ -7616,6 +8165,9 @@
           <t>883ebe8e-09ee-4631-b55b-337f9560d8ac</t>
         </is>
       </c>
+      <c r="L42" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" s="2" t="inlineStr">
@@ -7657,6 +8209,9 @@
           <t>363d9b37-f245-4192-9224-0b00b4fd1ea5</t>
         </is>
       </c>
+      <c r="L43" t="n">
+        <v>2</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" s="2" t="inlineStr">
@@ -7710,6 +8265,9 @@
           <t>e03d8d14-befe-40b7-b6ab-4472bef23ff7</t>
         </is>
       </c>
+      <c r="L44" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="45">
       <c r="A45" s="2" t="inlineStr">
@@ -7763,6 +8321,9 @@
           <t>9e7a5358-3efa-4301-ad21-e924721689b5</t>
         </is>
       </c>
+      <c r="L45" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="46">
       <c r="A46" s="2" t="inlineStr">
@@ -7816,6 +8377,9 @@
           <t>9e294012-4f82-47df-9c9f-5375df0a5e69</t>
         </is>
       </c>
+      <c r="L46" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="47">
       <c r="A47" s="2" t="inlineStr">
@@ -7869,6 +8433,9 @@
           <t>43799b86-b983-4162-8c36-dd40b7aac74b</t>
         </is>
       </c>
+      <c r="L47" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="48">
       <c r="A48" s="2" t="inlineStr">
@@ -7922,6 +8489,9 @@
           <t>1c86f6da-ba1b-4e21-b7b1-e91107da1bee</t>
         </is>
       </c>
+      <c r="L48" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="49">
       <c r="A49" s="2" t="inlineStr">
@@ -7975,6 +8545,9 @@
           <t>d1aed816-e28a-4ffb-a158-06ef60b75add</t>
         </is>
       </c>
+      <c r="L49" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="50">
       <c r="A50" s="2" t="inlineStr">
@@ -8028,6 +8601,9 @@
           <t>11c20815-6856-4b18-8729-d9a7e64c6496</t>
         </is>
       </c>
+      <c r="L50" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="51">
       <c r="A51" s="2" t="inlineStr">
@@ -8081,6 +8657,9 @@
           <t>044d5eda-11e1-4f03-8af6-58eea7a265e5</t>
         </is>
       </c>
+      <c r="L51" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="52">
       <c r="A52" s="2" t="inlineStr">
@@ -8134,6 +8713,9 @@
           <t>f160738c-ce43-45ce-87a3-3da53b3cb493</t>
         </is>
       </c>
+      <c r="L52" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="53">
       <c r="A53" s="2" t="inlineStr">
@@ -8187,6 +8769,9 @@
           <t>f5923390-9c4e-43ab-9848-de3e4e5e09f0</t>
         </is>
       </c>
+      <c r="L53" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="54">
       <c r="A54" s="2" t="inlineStr">
@@ -8240,6 +8825,9 @@
           <t>bb82063a-b49c-48c3-b898-66f8d7550169</t>
         </is>
       </c>
+      <c r="L54" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="55">
       <c r="A55" s="2" t="inlineStr">
@@ -8293,6 +8881,9 @@
           <t>3e50d2a1-e143-431c-9480-dd556374f28a</t>
         </is>
       </c>
+      <c r="L55" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="56">
       <c r="A56" s="2" t="inlineStr">
@@ -8346,6 +8937,9 @@
           <t>32fc6955-cc43-4154-9769-e57335f68ef1</t>
         </is>
       </c>
+      <c r="L56" t="n">
+        <v>43</v>
+      </c>
     </row>
     <row r="57">
       <c r="A57" s="2" t="inlineStr">
@@ -8399,6 +8993,9 @@
           <t>d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8</t>
         </is>
       </c>
+      <c r="L57" t="n">
+        <v>48</v>
+      </c>
     </row>
     <row r="58">
       <c r="A58" s="2" t="inlineStr">
@@ -8451,6 +9048,9 @@
         <is>
           <t>db3b1962-96b8-49b8-ab8b-c7c13fd197df</t>
         </is>
+      </c>
+      <c r="L58" t="n">
+        <v>12</v>
       </c>
     </row>
     <row r="59">
@@ -8493,6 +9093,9 @@
           <t>66f1d933-90ed-49d1-89e5-dbb9e765b851</t>
         </is>
       </c>
+      <c r="L59" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="60">
       <c r="A60" s="2" t="inlineStr">
@@ -8534,6 +9137,9 @@
           <t>cf82ea28-f534-4da8-9786-e89dba954b17</t>
         </is>
       </c>
+      <c r="L60" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="61">
       <c r="A61" s="2" t="inlineStr">
@@ -8575,6 +9181,9 @@
           <t>fee017c6-a239-4e81-987a-fede32524903</t>
         </is>
       </c>
+      <c r="L61" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="62">
       <c r="A62" s="2" t="inlineStr">
@@ -8616,6 +9225,9 @@
           <t>9e51941e-8703-4d9c-814e-c80d8be9fde2</t>
         </is>
       </c>
+      <c r="L62" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="63">
       <c r="A63" s="2" t="inlineStr">
@@ -8657,6 +9269,9 @@
           <t>34982d0f-52be-4a8b-935f-9aa3ee3915bb</t>
         </is>
       </c>
+      <c r="L63" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="64">
       <c r="A64" s="2" t="inlineStr">
@@ -8698,6 +9313,9 @@
           <t>220bac31-1b58-44ff-8b44-2e0dffd8fc5a</t>
         </is>
       </c>
+      <c r="L64" t="n">
+        <v>8</v>
+      </c>
     </row>
     <row r="65">
       <c r="A65" s="2" t="inlineStr">
@@ -8739,6 +9357,9 @@
           <t>74da6bde-8f40-4f5a-881e-c79da99f35a1</t>
         </is>
       </c>
+      <c r="L65" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="66">
       <c r="A66" s="2" t="inlineStr">
@@ -8780,6 +9401,9 @@
           <t>3bc172f4-88c0-403c-9c60-483089c17d75</t>
         </is>
       </c>
+      <c r="L66" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="67">
       <c r="A67" s="2" t="inlineStr">
@@ -8824,6 +9448,9 @@
         <is>
           <t>c189c73d-9a18-477b-8c39-c855849020d0</t>
         </is>
+      </c>
+      <c r="L67" t="n">
+        <v>45</v>
       </c>
     </row>
     <row r="68">
@@ -8866,6 +9493,9 @@
           <t>e00515fb-8071-400a-bf39-fa070c0f663c</t>
         </is>
       </c>
+      <c r="L68" t="n">
+        <v>20</v>
+      </c>
     </row>
     <row r="69">
       <c r="A69" s="2" t="inlineStr">
@@ -8910,6 +9540,9 @@
         <is>
           <t>dff3f8a8-0ec4-40c5-9776-8e11d1e39e9b</t>
         </is>
+      </c>
+      <c r="L69" t="n">
+        <v>20</v>
       </c>
     </row>
     <row r="70">
@@ -8952,6 +9585,9 @@
           <t>a22fe5fb-0b92-436c-b710-db69d8ea7c47</t>
         </is>
       </c>
+      <c r="L70" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="71">
       <c r="A71" s="2" t="inlineStr">
@@ -8993,6 +9629,9 @@
           <t>467411be-b152-4571-aab6-634eb4bf23fc</t>
         </is>
       </c>
+      <c r="L71" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="72">
       <c r="A72" s="2" t="inlineStr">
@@ -9046,6 +9685,9 @@
           <t>a33091fb-b612-4c2c-aaf8-3f0d7c1dcac3</t>
         </is>
       </c>
+      <c r="L72" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="73">
       <c r="A73" s="2" t="inlineStr">
@@ -9098,6 +9740,9 @@
         <is>
           <t>ed3b5a8c-8ac6-4d65-8961-df938488eb29</t>
         </is>
+      </c>
+      <c r="L73" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="74">
@@ -9140,6 +9785,9 @@
           <t>48b6a50f-e36a-4be6-9fe5-ba74ff2c0afc</t>
         </is>
       </c>
+      <c r="L74" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="75">
       <c r="A75" s="2" t="inlineStr">
@@ -9181,6 +9829,9 @@
           <t>cf5e22c9-8925-4779-8f00-d8de2fa957eb</t>
         </is>
       </c>
+      <c r="L75" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="76">
       <c r="A76" s="2" t="inlineStr">
@@ -9234,6 +9885,9 @@
           <t>b2a5fae9-92c4-46d3-b364-372aea858f72</t>
         </is>
       </c>
+      <c r="L76" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="77">
       <c r="A77" s="2" t="inlineStr">
@@ -9287,6 +9941,9 @@
           <t>0a3ae277-8590-4478-b8d5-804f67d03891</t>
         </is>
       </c>
+      <c r="L77" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="78">
       <c r="A78" s="2" t="inlineStr">
@@ -9340,6 +9997,9 @@
           <t>abf8c306-8989-4b41-b690-61b081be32e6</t>
         </is>
       </c>
+      <c r="L78" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="79">
       <c r="A79" s="2" t="inlineStr">
@@ -9393,6 +10053,9 @@
           <t>f0d47671-2942-4899-ba80-022688764653</t>
         </is>
       </c>
+      <c r="L79" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="80">
       <c r="A80" s="2" t="inlineStr">
@@ -9446,6 +10109,9 @@
           <t>ecc0aee3-c751-4e88-b738-4d0611d42f0a</t>
         </is>
       </c>
+      <c r="L80" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="81">
       <c r="A81" s="2" t="inlineStr">
@@ -9499,6 +10165,9 @@
           <t>8be45a46-a4fe-47f7-8e14-0d8b88c8bc08</t>
         </is>
       </c>
+      <c r="L81" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="82">
       <c r="A82" s="2" t="inlineStr">
@@ -9552,6 +10221,9 @@
           <t>0ed4d6a9-e127-48da-bb35-b80be311a816</t>
         </is>
       </c>
+      <c r="L82" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="83">
       <c r="A83" s="2" t="inlineStr">
@@ -9605,6 +10277,9 @@
           <t>9bb19246-4084-4e1b-98b3-751e272d0cd9</t>
         </is>
       </c>
+      <c r="L83" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="84">
       <c r="A84" s="2" t="inlineStr">
@@ -9658,6 +10333,9 @@
           <t>33609288-f489-4d89-84b7-70823a5a276d</t>
         </is>
       </c>
+      <c r="L84" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="85">
       <c r="A85" s="2" t="inlineStr">
@@ -9711,6 +10389,9 @@
           <t>3c08fbd5-25e3-47fb-9f66-a076efa2ab2e</t>
         </is>
       </c>
+      <c r="L85" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="86">
       <c r="A86" s="2" t="inlineStr">
@@ -9764,6 +10445,9 @@
           <t>3f0a1b1b-e90e-4324-8479-bdf6259f6040</t>
         </is>
       </c>
+      <c r="L86" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="87">
       <c r="A87" s="2" t="inlineStr">
@@ -9817,6 +10501,9 @@
           <t>c7ec947a-c40b-4710-a08f-0a436442ba97</t>
         </is>
       </c>
+      <c r="L87" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="88">
       <c r="A88" s="2" t="inlineStr">
@@ -9870,6 +10557,9 @@
           <t>1a7a09ca-f8b7-4f55-8441-ffb04e0d63f6</t>
         </is>
       </c>
+      <c r="L88" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="89">
       <c r="A89" s="2" t="inlineStr">
@@ -9923,6 +10613,9 @@
           <t>8cc08bae-0659-4b71-af6a-b3f830c2d9c8</t>
         </is>
       </c>
+      <c r="L89" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="90">
       <c r="A90" s="2" t="inlineStr">
@@ -9975,6 +10668,9 @@
         <is>
           <t>2271183e-fad9-4f2f-94a4-656ddc3e2327</t>
         </is>
+      </c>
+      <c r="L90" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="91">
@@ -10017,6 +10713,9 @@
           <t>7ed33ee7-275e-4af5-8ddc-3e67ce01ce50</t>
         </is>
       </c>
+      <c r="L91" t="n">
+        <v>106</v>
+      </c>
     </row>
     <row r="92">
       <c r="A92" s="2" t="inlineStr">
@@ -10058,6 +10757,9 @@
           <t>589dc885-5ca9-4b06-9776-ebb80e7ea81d</t>
         </is>
       </c>
+      <c r="L92" t="n">
+        <v>42</v>
+      </c>
     </row>
     <row r="93">
       <c r="A93" s="2" t="inlineStr">
@@ -10102,6 +10804,9 @@
         <is>
           <t>4900a270-06ee-458b-9793-2f98b3644748</t>
         </is>
+      </c>
+      <c r="L93" t="n">
+        <v>9</v>
       </c>
     </row>
     <row r="94">
@@ -10144,6 +10849,9 @@
           <t>3d9a0917-34b5-4ac6-8b6a-f2244892db15</t>
         </is>
       </c>
+      <c r="L94" t="n">
+        <v>5</v>
+      </c>
     </row>
     <row r="95">
       <c r="A95" s="2" t="inlineStr">
@@ -10185,6 +10893,9 @@
           <t>01100552-0f0b-461b-9327-4bc164c5f331</t>
         </is>
       </c>
+      <c r="L95" t="n">
+        <v>206</v>
+      </c>
     </row>
     <row r="96">
       <c r="A96" s="2" t="inlineStr">
@@ -10226,6 +10937,9 @@
           <t>4bdda3e7-2a7d-4b74-a484-4551b4873c03</t>
         </is>
       </c>
+      <c r="L96" t="n">
+        <v>1</v>
+      </c>
     </row>
     <row r="97">
       <c r="A97" s="2" t="inlineStr">
@@ -10270,6 +10984,9 @@
         <is>
           <t>d290f1bf-00d9-41de-aae8-0006cd919e4e</t>
         </is>
+      </c>
+      <c r="L97" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="98">
@@ -10312,6 +11029,9 @@
           <t>ae8549ef-1d06-44e3-b0ec-228ba42aaafe</t>
         </is>
       </c>
+      <c r="L98" t="n">
+        <v>11</v>
+      </c>
     </row>
     <row r="99">
       <c r="A99" s="2" t="inlineStr">
@@ -10353,6 +11073,9 @@
           <t>2c4fb5d8-ccf7-4e0a-8361-362399f22c0c</t>
         </is>
       </c>
+      <c r="L99" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="100">
       <c r="A100" s="2" t="inlineStr">
@@ -10394,6 +11117,9 @@
           <t>18668d79-2a2c-47bf-b666-33ac22fe1b6f</t>
         </is>
       </c>
+      <c r="L100" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="101">
       <c r="A101" s="2" t="inlineStr">
@@ -10435,6 +11161,9 @@
           <t>cddfdfd9-8261-4403-9f7d-ede767a414ea</t>
         </is>
       </c>
+      <c r="L101" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="102">
       <c r="A102" s="2" t="inlineStr">
@@ -10476,6 +11205,9 @@
           <t>785ded3c-9ed4-4463-8373-7992a07cc40c</t>
         </is>
       </c>
+      <c r="L102" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="103">
       <c r="A103" s="2" t="inlineStr">
@@ -10517,6 +11249,9 @@
           <t>d977bfb1-99bc-4c6a-ab6d-18f297149a36</t>
         </is>
       </c>
+      <c r="L103" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="104">
       <c r="A104" s="2" t="inlineStr">
@@ -10558,6 +11293,9 @@
           <t>fc182951-77ad-488d-8feb-5acc78e0c7e9</t>
         </is>
       </c>
+      <c r="L104" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="105">
       <c r="A105" s="2" t="inlineStr">
@@ -10599,6 +11337,9 @@
           <t>b6e41938-7e3e-48e9-996b-d491e37541f9</t>
         </is>
       </c>
+      <c r="L105" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="106">
       <c r="A106" s="2" t="inlineStr">
@@ -10640,6 +11381,9 @@
           <t>d1c92403-15f2-4bf6-b077-dc5cb6f7b490</t>
         </is>
       </c>
+      <c r="L106" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="107">
       <c r="A107" s="2" t="inlineStr">
@@ -10689,6 +11433,9 @@
           <t>af98c80e-9345-4da9-b743-018b9285fa5e</t>
         </is>
       </c>
+      <c r="L107" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="108">
       <c r="A108" s="2" t="inlineStr">
@@ -10738,6 +11485,9 @@
           <t>31a2dc0d-9967-47eb-8ecf-4f61f0e5e3b8</t>
         </is>
       </c>
+      <c r="L108" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="109">
       <c r="A109" s="2" t="inlineStr">
@@ -10786,6 +11536,9 @@
         <is>
           <t>855b1a3d-085c-4aa0-a601-07463be25697</t>
         </is>
+      </c>
+      <c r="L109" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="110">
@@ -10828,6 +11581,9 @@
           <t>293fe003-6ee2-4215-8c40-a47893f8447c</t>
         </is>
       </c>
+      <c r="L110" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="111">
       <c r="A111" s="2" t="inlineStr">
@@ -10869,6 +11625,9 @@
           <t>09e9193a-f463-498d-9e90-493d77f30de4</t>
         </is>
       </c>
+      <c r="L111" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="112">
       <c r="A112" s="2" t="inlineStr">
@@ -10910,6 +11669,9 @@
           <t>5454cf95-0660-40a2-8768-67b20b4a707a</t>
         </is>
       </c>
+      <c r="L112" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="113">
       <c r="A113" s="2" t="inlineStr">
@@ -10951,6 +11713,9 @@
           <t>e8151a94-ab3c-4362-8aeb-160dc3ff5ed9</t>
         </is>
       </c>
+      <c r="L113" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="114">
       <c r="A114" s="2" t="inlineStr">
@@ -10992,6 +11757,9 @@
           <t>6f91c54d-24ae-4d7a-a580-596cc52ec510</t>
         </is>
       </c>
+      <c r="L114" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="115">
       <c r="A115" s="2" t="inlineStr">
@@ -11033,6 +11801,9 @@
           <t>f47ca5f4-a334-4064-94a1-564f810c0b7c</t>
         </is>
       </c>
+      <c r="L115" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="116">
       <c r="A116" s="2" t="inlineStr">
@@ -11074,6 +11845,9 @@
           <t>5dd96eea-eef1-4663-be56-4b7a8f9a3087</t>
         </is>
       </c>
+      <c r="L116" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="117">
       <c r="A117" s="2" t="inlineStr">
@@ -11115,6 +11889,9 @@
           <t>8bdb45d1-c1c9-4ee3-9658-d4ab30fb67b9</t>
         </is>
       </c>
+      <c r="L117" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="118">
       <c r="A118" s="2" t="inlineStr">
@@ -11156,6 +11933,9 @@
           <t>b82ed9fb-5d10-495d-9a6d-b0b617fdd487</t>
         </is>
       </c>
+      <c r="L118" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="119">
       <c r="A119" s="2" t="inlineStr">
@@ -11197,6 +11977,9 @@
           <t>a698bdc2-d8e9-45f8-b668-1d321e44a201</t>
         </is>
       </c>
+      <c r="L119" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="120">
       <c r="A120" s="2" t="inlineStr">
@@ -11238,6 +12021,9 @@
           <t>164998e9-90bc-46f7-8360-efbbe3f5da7f</t>
         </is>
       </c>
+      <c r="L120" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="121">
       <c r="A121" s="2" t="inlineStr">
@@ -11279,6 +12065,9 @@
           <t>243f52b1-78cb-4c1a-9689-e0f18217f77a</t>
         </is>
       </c>
+      <c r="L121" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="122">
       <c r="A122" s="2" t="inlineStr">
@@ -11320,6 +12109,9 @@
           <t>f04b41aa-2bd1-4166-8005-a78fcad04720</t>
         </is>
       </c>
+      <c r="L122" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="123">
       <c r="A123" s="2" t="inlineStr">
@@ -11361,6 +12153,9 @@
           <t>093abf07-4090-4b19-a222-999c87fb18d0</t>
         </is>
       </c>
+      <c r="L123" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="124">
       <c r="A124" s="2" t="inlineStr">
@@ -11402,6 +12197,9 @@
           <t>90289651-9e74-492e-bb7d-55d173267b57</t>
         </is>
       </c>
+      <c r="L124" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="125">
       <c r="A125" s="2" t="inlineStr">
@@ -11443,6 +12241,9 @@
           <t>dae0e788-84c1-460b-8961-54fc6b766e2e</t>
         </is>
       </c>
+      <c r="L125" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="126">
       <c r="A126" s="2" t="inlineStr">
@@ -11484,6 +12285,9 @@
           <t>c6b3722f-f2be-40b3-a553-6fb690c3adea</t>
         </is>
       </c>
+      <c r="L126" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="127">
       <c r="A127" s="2" t="inlineStr">
@@ -11525,6 +12329,9 @@
           <t>5d2131f2-f6b5-41f6-b864-e0534c499950</t>
         </is>
       </c>
+      <c r="L127" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="128">
       <c r="A128" s="2" t="inlineStr">
@@ -11566,6 +12373,9 @@
           <t>034fc54a-d18c-44b2-9915-aa86bd8b02f1</t>
         </is>
       </c>
+      <c r="L128" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="129">
       <c r="A129" s="2" t="inlineStr">
@@ -11619,6 +12429,9 @@
           <t>3d26ba08-de7b-4635-b801-959f2751c0ea</t>
         </is>
       </c>
+      <c r="L129" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="130">
       <c r="A130" s="2" t="inlineStr">
@@ -11672,6 +12485,9 @@
           <t>2ebaf008-5151-4818-941c-1fb09e7ece5d</t>
         </is>
       </c>
+      <c r="L130" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="131">
       <c r="A131" s="2" t="inlineStr">
@@ -11725,6 +12541,9 @@
           <t>5b114d82-e229-482c-9756-a9461a47fa76</t>
         </is>
       </c>
+      <c r="L131" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="132">
       <c r="A132" s="2" t="inlineStr">
@@ -11778,6 +12597,9 @@
           <t>79627458-97b4-408e-b057-93369d32e0fc</t>
         </is>
       </c>
+      <c r="L132" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="133">
       <c r="A133" s="2" t="inlineStr">
@@ -11831,6 +12653,9 @@
           <t>4c69e9ea-c9fe-4853-8b65-0944c71c846f</t>
         </is>
       </c>
+      <c r="L133" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="134">
       <c r="A134" s="2" t="inlineStr">
@@ -11884,6 +12709,9 @@
           <t>bb053133-fab4-44ba-beef-b3cc5a883d8b</t>
         </is>
       </c>
+      <c r="L134" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="135">
       <c r="A135" s="2" t="inlineStr">
@@ -11937,6 +12765,9 @@
           <t>be821246-ab66-4f6d-8723-345a31c51584</t>
         </is>
       </c>
+      <c r="L135" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="136">
       <c r="A136" s="2" t="inlineStr">
@@ -11990,6 +12821,9 @@
           <t>864f9511-ae08-4152-be61-da8b02e0d10d</t>
         </is>
       </c>
+      <c r="L136" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="137">
       <c r="A137" s="2" t="inlineStr">
@@ -12043,6 +12877,9 @@
           <t>62dad30f-7d22-4048-80a6-dda3df482533</t>
         </is>
       </c>
+      <c r="L137" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="138">
       <c r="A138" s="2" t="inlineStr">
@@ -12096,6 +12933,9 @@
           <t>7a756d76-6d55-4541-ac3c-9c9f20aa3bb6</t>
         </is>
       </c>
+      <c r="L138" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="139">
       <c r="A139" s="2" t="inlineStr">
@@ -12149,6 +12989,9 @@
           <t>a34b1e3d-829e-467c-81fb-9e7e446afeee</t>
         </is>
       </c>
+      <c r="L139" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="140">
       <c r="A140" s="2" t="inlineStr">
@@ -12202,6 +13045,9 @@
           <t>8e1fe016-e2ae-4085-8c03-6ba689cd0be0</t>
         </is>
       </c>
+      <c r="L140" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="141">
       <c r="A141" s="2" t="inlineStr">
@@ -12255,6 +13101,9 @@
           <t>ef671aec-c05d-4a42-b941-bc2f967d6226</t>
         </is>
       </c>
+      <c r="L141" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="142">
       <c r="A142" s="2" t="inlineStr">
@@ -12307,6 +13156,9 @@
         <is>
           <t>c6e72043-9449-4d47-992c-d5e6075ec51d</t>
         </is>
+      </c>
+      <c r="L142" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -12349,6 +13201,9 @@
           <t>30580dcd-18a8-4764-b965-e447e8860cf4</t>
         </is>
       </c>
+      <c r="L143" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="144">
       <c r="A144" s="2" t="inlineStr">
@@ -12390,6 +13245,9 @@
           <t>7de99d39-41a8-4578-994d-377c9a1c334e</t>
         </is>
       </c>
+      <c r="L144" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="145">
       <c r="A145" s="2" t="inlineStr">
@@ -12431,6 +13289,9 @@
           <t>e6b113ec-729a-4d3c-934c-f54c1f9689d9</t>
         </is>
       </c>
+      <c r="L145" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="146">
       <c r="A146" s="2" t="inlineStr">
@@ -12472,6 +13333,9 @@
           <t>fe7147dc-d416-463e-a43b-8f14fbc59ad5</t>
         </is>
       </c>
+      <c r="L146" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="147">
       <c r="A147" s="2" t="inlineStr">
@@ -12513,6 +13377,9 @@
           <t>7657aa6c-a1bf-4d2f-b760-671fbcb055bd</t>
         </is>
       </c>
+      <c r="L147" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="148">
       <c r="A148" s="2" t="inlineStr">
@@ -12554,6 +13421,9 @@
           <t>e637610f-e023-4a95-8366-31bbf7a60ea7</t>
         </is>
       </c>
+      <c r="L148" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="149">
       <c r="A149" s="2" t="inlineStr">
@@ -12595,6 +13465,9 @@
           <t>55c09f7e-7339-4cda-a232-4593c1874b8a</t>
         </is>
       </c>
+      <c r="L149" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="150">
       <c r="A150" s="2" t="inlineStr">
@@ -12636,6 +13509,9 @@
           <t>0b3f58f9-25ad-4967-aad6-049cda1d532f</t>
         </is>
       </c>
+      <c r="L150" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="151">
       <c r="A151" s="2" t="inlineStr">
@@ -12677,6 +13553,9 @@
           <t>f8aebfcb-d153-4d3b-a118-60c1a7876a2c</t>
         </is>
       </c>
+      <c r="L151" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="152">
       <c r="A152" s="2" t="inlineStr">
@@ -12718,6 +13597,9 @@
           <t>1632e5a1-1d96-42be-b9c6-a2d58321335e</t>
         </is>
       </c>
+      <c r="L152" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="153">
       <c r="A153" s="2" t="inlineStr">
@@ -12759,6 +13641,9 @@
           <t>849ac12f-c28b-4306-a0fe-6a00c6c9c8e8</t>
         </is>
       </c>
+      <c r="L153" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="154">
       <c r="A154" s="2" t="inlineStr">
@@ -12800,6 +13685,9 @@
           <t>aacc1cbf-8839-4b44-933e-085a3fe7eb66</t>
         </is>
       </c>
+      <c r="L154" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="155">
       <c r="A155" s="2" t="inlineStr">
@@ -12853,6 +13741,9 @@
           <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
         </is>
       </c>
+      <c r="L155" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="156">
       <c r="A156" s="2" t="inlineStr">
@@ -12906,6 +13797,9 @@
           <t>b4d6b026-7a58-416c-918b-834458a06075</t>
         </is>
       </c>
+      <c r="L156" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="157">
       <c r="A157" s="2" t="inlineStr">
@@ -12959,6 +13853,9 @@
           <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
         </is>
       </c>
+      <c r="L157" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="158">
       <c r="A158" s="2" t="inlineStr">
@@ -13012,6 +13909,9 @@
           <t>002d561c-4948-4eed-8a69-c915d548675e</t>
         </is>
       </c>
+      <c r="L158" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="159">
       <c r="A159" s="2" t="inlineStr">
@@ -13065,6 +13965,9 @@
           <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
         </is>
       </c>
+      <c r="L159" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="160">
       <c r="A160" s="2" t="inlineStr">
@@ -13118,6 +14021,9 @@
           <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
         </is>
       </c>
+      <c r="L160" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="161">
       <c r="A161" s="2" t="inlineStr">
@@ -13171,6 +14077,9 @@
           <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
         </is>
       </c>
+      <c r="L161" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="162">
       <c r="A162" s="2" t="inlineStr">
@@ -13224,6 +14133,9 @@
           <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
         </is>
       </c>
+      <c r="L162" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="163">
       <c r="A163" s="2" t="inlineStr">
@@ -13277,6 +14189,9 @@
           <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
         </is>
       </c>
+      <c r="L163" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="164">
       <c r="A164" s="2" t="inlineStr">
@@ -13330,6 +14245,9 @@
           <t>24c5543f-4401-4463-905d-783c3592b69c</t>
         </is>
       </c>
+      <c r="L164" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="165">
       <c r="A165" s="2" t="inlineStr">
@@ -13383,6 +14301,9 @@
           <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
         </is>
       </c>
+      <c r="L165" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="166">
       <c r="A166" s="2" t="inlineStr">
@@ -13436,6 +14357,9 @@
           <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
         </is>
       </c>
+      <c r="L166" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="167">
       <c r="A167" s="2" t="inlineStr">
@@ -13489,6 +14413,9 @@
           <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
         </is>
       </c>
+      <c r="L167" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="168">
       <c r="A168" s="2" t="inlineStr">
@@ -13541,6 +14468,9 @@
         <is>
           <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
         </is>
+      </c>
+      <c r="L168" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="169">
@@ -13583,6 +14513,9 @@
           <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
         </is>
       </c>
+      <c r="L169" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="170">
       <c r="A170" s="2" t="inlineStr">
@@ -13624,6 +14557,9 @@
           <t>fce7fec8-1591-4d36-937a-104080c89b4f</t>
         </is>
       </c>
+      <c r="L170" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="171">
       <c r="A171" s="2" t="inlineStr">
@@ -13665,6 +14601,9 @@
           <t>14432aec-0724-4c98-905f-1f2681948b2f</t>
         </is>
       </c>
+      <c r="L171" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="172">
       <c r="A172" s="2" t="inlineStr">
@@ -13706,6 +14645,9 @@
           <t>ca6214b2-3622-4950-9f7f-cb22dc1697f8</t>
         </is>
       </c>
+      <c r="L172" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="173">
       <c r="A173" s="2" t="inlineStr">
@@ -13747,6 +14689,9 @@
           <t>f62bbf09-eca6-4bb8-8caa-e88da0c3184d</t>
         </is>
       </c>
+      <c r="L173" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="174">
       <c r="A174" s="2" t="inlineStr">
@@ -13788,6 +14733,9 @@
           <t>7f57b337-e918-4c13-aa6e-3e42d193d9b4</t>
         </is>
       </c>
+      <c r="L174" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="175">
       <c r="A175" s="2" t="inlineStr">
@@ -13829,6 +14777,9 @@
           <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
         </is>
       </c>
+      <c r="L175" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="176">
       <c r="A176" s="2" t="inlineStr">
@@ -13870,6 +14821,9 @@
           <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
         </is>
       </c>
+      <c r="L176" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="177">
       <c r="A177" s="2" t="inlineStr">
@@ -13911,6 +14865,9 @@
           <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
         </is>
       </c>
+      <c r="L177" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="178">
       <c r="A178" s="2" t="inlineStr">
@@ -13952,6 +14909,9 @@
           <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
+      <c r="L178" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="179">
       <c r="A179" s="2" t="inlineStr">
@@ -13993,6 +14953,9 @@
           <t>41d0a85e-4b61-46bc-9850-5984ff419dd1</t>
         </is>
       </c>
+      <c r="L179" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="180">
       <c r="A180" s="2" t="inlineStr">
@@ -14045,6 +15008,9 @@
         <is>
           <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
+      </c>
+      <c r="L180" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="181">
@@ -14087,6 +15053,9 @@
           <t>784d6896-dd8a-4b7a-9c5c-962ea6c5e49c</t>
         </is>
       </c>
+      <c r="L181" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="182">
       <c r="A182" s="2" t="inlineStr">
@@ -14139,6 +15108,9 @@
         <is>
           <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
+      </c>
+      <c r="L182" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="183">
@@ -14181,6 +15153,9 @@
           <t>08eee5c2-f90d-483d-9382-0726090489f7</t>
         </is>
       </c>
+      <c r="L183" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="184">
       <c r="A184" s="2" t="inlineStr">
@@ -14233,6 +15208,9 @@
         <is>
           <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
+      </c>
+      <c r="L184" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="185">
@@ -14275,6 +15253,9 @@
           <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
+      <c r="L185" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="186">
       <c r="A186" s="2" t="inlineStr">
@@ -14328,6 +15309,9 @@
           <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
+      <c r="L186" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="187">
       <c r="A187" s="2" t="inlineStr">
@@ -14381,6 +15365,9 @@
           <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
+      <c r="L187" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="188">
       <c r="A188" s="2" t="inlineStr">
@@ -14434,6 +15421,9 @@
           <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
+      <c r="L188" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="189">
       <c r="A189" s="2" t="inlineStr">
@@ -14487,6 +15477,9 @@
           <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
+      <c r="L189" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="190">
       <c r="A190" s="2" t="inlineStr">
@@ -14540,6 +15533,9 @@
           <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
+      <c r="L190" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="191">
       <c r="A191" s="2" t="inlineStr">
@@ -14593,6 +15589,9 @@
           <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
+      <c r="L191" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="192">
       <c r="A192" s="2" t="inlineStr">
@@ -14646,6 +15645,9 @@
           <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
+      <c r="L192" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="193">
       <c r="A193" s="2" t="inlineStr">
@@ -14699,6 +15701,9 @@
           <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
+      <c r="L193" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="194">
       <c r="A194" s="2" t="inlineStr">
@@ -14752,6 +15757,9 @@
           <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
+      <c r="L194" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="195">
       <c r="A195" s="2" t="inlineStr">
@@ -14805,6 +15813,9 @@
           <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
+      <c r="L195" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="196">
       <c r="A196" s="2" t="inlineStr">
@@ -14858,6 +15869,9 @@
           <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
+      <c r="L196" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="197">
       <c r="A197" s="2" t="inlineStr">
@@ -14911,6 +15925,9 @@
           <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
+      <c r="L197" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="198">
       <c r="A198" s="2" t="inlineStr">
@@ -14964,6 +15981,9 @@
           <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
+      <c r="L198" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="199">
       <c r="A199" s="2" t="inlineStr">
@@ -15017,6 +16037,9 @@
           <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
+      <c r="L199" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="200">
       <c r="A200" s="2" t="inlineStr">
@@ -15070,6 +16093,9 @@
           <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
+      <c r="L200" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="201">
       <c r="A201" s="2" t="inlineStr">
@@ -15123,6 +16149,9 @@
           <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
+      <c r="L201" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="202">
       <c r="A202" s="2" t="inlineStr">
@@ -15176,6 +16205,9 @@
           <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
+      <c r="L202" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="203">
       <c r="A203" s="2" t="inlineStr">
@@ -15229,6 +16261,9 @@
           <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
+      <c r="L203" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="204">
       <c r="A204" s="2" t="inlineStr">
@@ -15282,6 +16317,9 @@
           <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
+      <c r="L204" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="205">
       <c r="A205" s="2" t="inlineStr">
@@ -15335,6 +16373,9 @@
           <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
+      <c r="L205" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="206">
       <c r="A206" s="2" t="inlineStr">
@@ -15388,6 +16429,9 @@
           <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
+      <c r="L206" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="207">
       <c r="A207" s="2" t="inlineStr">
@@ -15441,6 +16485,9 @@
           <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
+      <c r="L207" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="208">
       <c r="A208" s="2" t="inlineStr">
@@ -15494,6 +16541,9 @@
           <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
+      <c r="L208" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="209">
       <c r="A209" s="2" t="inlineStr">
@@ -15547,6 +16597,9 @@
           <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
+      <c r="L209" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="210">
       <c r="A210" s="2" t="inlineStr">
@@ -15600,6 +16653,9 @@
           <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
+      <c r="L210" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="211">
       <c r="A211" s="2" t="inlineStr">
@@ -15653,6 +16709,9 @@
           <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
+      <c r="L211" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="212">
       <c r="A212" s="2" t="inlineStr">
@@ -15706,6 +16765,9 @@
           <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
+      <c r="L212" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="213">
       <c r="A213" s="2" t="inlineStr">
@@ -15758,6 +16820,9 @@
         <is>
           <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
+      </c>
+      <c r="L213" t="n">
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -15800,6 +16865,9 @@
           <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
         </is>
       </c>
+      <c r="L214" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="215">
       <c r="A215" s="2" t="inlineStr">
@@ -15841,6 +16909,9 @@
           <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
         </is>
       </c>
+      <c r="L215" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="216">
       <c r="A216" s="2" t="inlineStr">
@@ -15882,6 +16953,9 @@
           <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
+      <c r="L216" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="217">
       <c r="A217" s="2" t="inlineStr">
@@ -15923,6 +16997,9 @@
           <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
+      <c r="L217" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="218">
       <c r="A218" s="2" t="inlineStr">
@@ -15964,6 +17041,9 @@
           <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
+      <c r="L218" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="219">
       <c r="A219" s="2" t="inlineStr">
@@ -16005,6 +17085,9 @@
           <t>648d45b0-2231-4e56-a018-4e83792a3115</t>
         </is>
       </c>
+      <c r="L219" t="n">
+        <v>0</v>
+      </c>
     </row>
     <row r="220">
       <c r="A220" s="2" t="inlineStr">
@@ -16046,9 +17129,12 @@
           <t>bdfe582a-c303-4732-b9b7-2390e04aa58e</t>
         </is>
       </c>
+      <c r="L220" t="n">
+        <v>0</v>
+      </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:K220"/>
+  <autoFilter ref="A1:L220"/>
   <dataValidations count="1">
     <dataValidation sqref="A2:A220" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-25 15:56)
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="H:\Automatizacion de reportes\PowerBI\Links POWER BI\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{054CC8A4-E487-40CF-812D-830D36E9ABEF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{706B63C6-9DE9-462F-BFA1-B3613F982611}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="20370" yWindow="-150" windowWidth="20640" windowHeight="11040" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tableros" sheetId="1" r:id="rId1"/>
@@ -18,14 +18,14 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">Catalogo!$A$1:$L$214</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tableros!$A$1:$H$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">Tableros!$A$1:$H$148</definedName>
   </definedNames>
   <calcPr calcId="0"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2745" uniqueCount="662">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2739" uniqueCount="662">
   <si>
     <t>Area</t>
   </si>
@@ -2371,7 +2371,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:H149"/>
+  <dimension ref="A1:H148"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="9.140625" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -2833,16 +2833,16 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B21" t="s">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="C21" t="s">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D21" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F21" t="s">
         <v>12</v>
@@ -2853,7 +2853,7 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="B22" t="s">
         <v>14</v>
@@ -2873,7 +2873,7 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="B23" t="s">
         <v>14</v>
@@ -2893,22 +2893,25 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>65</v>
+        <v>62</v>
       </c>
       <c r="B24" t="s">
-        <v>14</v>
+        <v>9</v>
       </c>
       <c r="C24" t="s">
-        <v>15</v>
+        <v>66</v>
       </c>
       <c r="D24" t="s">
-        <v>16</v>
+        <v>67</v>
       </c>
       <c r="F24" t="s">
-        <v>12</v>
+        <v>68</v>
       </c>
       <c r="G24" t="s">
         <v>13</v>
+      </c>
+      <c r="H24">
+        <v>42</v>
       </c>
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
@@ -2919,10 +2922,10 @@
         <v>9</v>
       </c>
       <c r="C25" t="s">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="D25" t="s">
-        <v>67</v>
+        <v>70</v>
       </c>
       <c r="F25" t="s">
         <v>68</v>
@@ -2931,7 +2934,7 @@
         <v>13</v>
       </c>
       <c r="H25">
-        <v>42</v>
+        <v>24</v>
       </c>
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
@@ -2942,10 +2945,10 @@
         <v>9</v>
       </c>
       <c r="C26" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="D26" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="F26" t="s">
         <v>68</v>
@@ -2965,10 +2968,10 @@
         <v>9</v>
       </c>
       <c r="C27" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D27" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="F27" t="s">
         <v>68</v>
@@ -2977,7 +2980,7 @@
         <v>13</v>
       </c>
       <c r="H27">
-        <v>24</v>
+        <v>18</v>
       </c>
     </row>
     <row r="28" spans="1:8" x14ac:dyDescent="0.25">
@@ -2988,10 +2991,10 @@
         <v>9</v>
       </c>
       <c r="C28" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D28" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="F28" t="s">
         <v>68</v>
@@ -3000,7 +3003,7 @@
         <v>13</v>
       </c>
       <c r="H28">
-        <v>18</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29" spans="1:8" x14ac:dyDescent="0.25">
@@ -3011,10 +3014,10 @@
         <v>9</v>
       </c>
       <c r="C29" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="D29" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="F29" t="s">
         <v>68</v>
@@ -3023,7 +3026,7 @@
         <v>13</v>
       </c>
       <c r="H29">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="30" spans="1:8" x14ac:dyDescent="0.25">
@@ -3034,10 +3037,10 @@
         <v>9</v>
       </c>
       <c r="C30" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="D30" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="F30" t="s">
         <v>68</v>
@@ -3046,7 +3049,7 @@
         <v>13</v>
       </c>
       <c r="H30">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="31" spans="1:8" x14ac:dyDescent="0.25">
@@ -3057,10 +3060,10 @@
         <v>9</v>
       </c>
       <c r="C31" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="D31" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="F31" t="s">
         <v>68</v>
@@ -3080,10 +3083,10 @@
         <v>9</v>
       </c>
       <c r="C32" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="D32" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="F32" t="s">
         <v>68</v>
@@ -3100,13 +3103,13 @@
         <v>62</v>
       </c>
       <c r="B33" t="s">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="C33" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D33" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F33" t="s">
         <v>68</v>
@@ -3115,7 +3118,7 @@
         <v>13</v>
       </c>
       <c r="H33">
-        <v>0</v>
+        <v>46</v>
       </c>
     </row>
     <row r="34" spans="1:8" x14ac:dyDescent="0.25">
@@ -3126,10 +3129,10 @@
         <v>85</v>
       </c>
       <c r="C34" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="D34" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="F34" t="s">
         <v>68</v>
@@ -3138,7 +3141,7 @@
         <v>13</v>
       </c>
       <c r="H34">
-        <v>46</v>
+        <v>36</v>
       </c>
     </row>
     <row r="35" spans="1:8" x14ac:dyDescent="0.25">
@@ -3149,10 +3152,10 @@
         <v>85</v>
       </c>
       <c r="C35" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="D35" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="F35" t="s">
         <v>68</v>
@@ -3161,7 +3164,7 @@
         <v>13</v>
       </c>
       <c r="H35">
-        <v>36</v>
+        <v>8</v>
       </c>
     </row>
     <row r="36" spans="1:8" x14ac:dyDescent="0.25">
@@ -3172,10 +3175,10 @@
         <v>85</v>
       </c>
       <c r="C36" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="D36" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="F36" t="s">
         <v>68</v>
@@ -3184,7 +3187,7 @@
         <v>13</v>
       </c>
       <c r="H36">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.25">
@@ -3195,10 +3198,10 @@
         <v>85</v>
       </c>
       <c r="C37" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="D37" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="F37" t="s">
         <v>68</v>
@@ -3207,7 +3210,7 @@
         <v>13</v>
       </c>
       <c r="H37">
-        <v>6</v>
+        <v>3</v>
       </c>
     </row>
     <row r="38" spans="1:8" x14ac:dyDescent="0.25">
@@ -3218,10 +3221,10 @@
         <v>85</v>
       </c>
       <c r="C38" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
       <c r="D38" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F38" t="s">
         <v>68</v>
@@ -3230,7 +3233,7 @@
         <v>13</v>
       </c>
       <c r="H38">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.25">
@@ -3241,10 +3244,10 @@
         <v>85</v>
       </c>
       <c r="C39" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="D39" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="F39" t="s">
         <v>68</v>
@@ -3253,21 +3256,21 @@
         <v>13</v>
       </c>
       <c r="H39">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="40" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A40" t="s">
-        <v>62</v>
+        <v>8</v>
       </c>
       <c r="B40" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="C40" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="D40" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="F40" t="s">
         <v>68</v>
@@ -3276,7 +3279,7 @@
         <v>13</v>
       </c>
       <c r="H40">
-        <v>0</v>
+        <v>55</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.25">
@@ -3287,10 +3290,10 @@
         <v>65</v>
       </c>
       <c r="C41" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="D41" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="F41" t="s">
         <v>68</v>
@@ -3299,7 +3302,7 @@
         <v>13</v>
       </c>
       <c r="H41">
-        <v>55</v>
+        <v>7</v>
       </c>
     </row>
     <row r="42" spans="1:8" x14ac:dyDescent="0.25">
@@ -3310,10 +3313,10 @@
         <v>65</v>
       </c>
       <c r="C42" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="D42" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="F42" t="s">
         <v>68</v>
@@ -3322,7 +3325,7 @@
         <v>13</v>
       </c>
       <c r="H42">
-        <v>7</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.25">
@@ -3330,13 +3333,13 @@
         <v>8</v>
       </c>
       <c r="B43" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C43" t="s">
-        <v>104</v>
+        <v>69</v>
       </c>
       <c r="D43" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="F43" t="s">
         <v>68</v>
@@ -3345,7 +3348,7 @@
         <v>13</v>
       </c>
       <c r="H43">
-        <v>4</v>
+        <v>26</v>
       </c>
     </row>
     <row r="44" spans="1:8" x14ac:dyDescent="0.25">
@@ -3356,10 +3359,10 @@
         <v>9</v>
       </c>
       <c r="C44" t="s">
-        <v>69</v>
+        <v>107</v>
       </c>
       <c r="D44" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="F44" t="s">
         <v>68</v>
@@ -3379,10 +3382,10 @@
         <v>9</v>
       </c>
       <c r="C45" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D45" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="F45" t="s">
         <v>68</v>
@@ -3402,10 +3405,10 @@
         <v>9</v>
       </c>
       <c r="C46" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="D46" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="F46" t="s">
         <v>68</v>
@@ -3414,7 +3417,7 @@
         <v>13</v>
       </c>
       <c r="H46">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.25">
@@ -3425,10 +3428,10 @@
         <v>9</v>
       </c>
       <c r="C47" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D47" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="F47" t="s">
         <v>68</v>
@@ -3448,10 +3451,10 @@
         <v>9</v>
       </c>
       <c r="C48" t="s">
-        <v>113</v>
+        <v>73</v>
       </c>
       <c r="D48" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="F48" t="s">
         <v>68</v>
@@ -3460,7 +3463,7 @@
         <v>13</v>
       </c>
       <c r="H48">
-        <v>25</v>
+        <v>10</v>
       </c>
     </row>
     <row r="49" spans="1:8" x14ac:dyDescent="0.25">
@@ -3471,10 +3474,10 @@
         <v>9</v>
       </c>
       <c r="C49" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="D49" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="F49" t="s">
         <v>68</v>
@@ -3494,10 +3497,10 @@
         <v>9</v>
       </c>
       <c r="C50" t="s">
-        <v>71</v>
+        <v>117</v>
       </c>
       <c r="D50" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="F50" t="s">
         <v>68</v>
@@ -3506,7 +3509,7 @@
         <v>13</v>
       </c>
       <c r="H50">
-        <v>10</v>
+        <v>6</v>
       </c>
     </row>
     <row r="51" spans="1:8" x14ac:dyDescent="0.25">
@@ -3517,10 +3520,10 @@
         <v>9</v>
       </c>
       <c r="C51" t="s">
-        <v>117</v>
+        <v>81</v>
       </c>
       <c r="D51" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="F51" t="s">
         <v>68</v>
@@ -3529,7 +3532,7 @@
         <v>13</v>
       </c>
       <c r="H51">
-        <v>6</v>
+        <v>4</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.25">
@@ -3540,10 +3543,10 @@
         <v>9</v>
       </c>
       <c r="C52" t="s">
-        <v>81</v>
+        <v>120</v>
       </c>
       <c r="D52" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="F52" t="s">
         <v>68</v>
@@ -3552,7 +3555,7 @@
         <v>13</v>
       </c>
       <c r="H52">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="53" spans="1:8" x14ac:dyDescent="0.25">
@@ -3563,10 +3566,10 @@
         <v>9</v>
       </c>
       <c r="C53" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="D53" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="F53" t="s">
         <v>68</v>
@@ -3575,7 +3578,7 @@
         <v>13</v>
       </c>
       <c r="H53">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.25">
@@ -3586,10 +3589,10 @@
         <v>9</v>
       </c>
       <c r="C54" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="D54" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
       <c r="F54" t="s">
         <v>68</v>
@@ -3609,10 +3612,10 @@
         <v>9</v>
       </c>
       <c r="C55" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="D55" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
       <c r="F55" t="s">
         <v>68</v>
@@ -3621,7 +3624,7 @@
         <v>13</v>
       </c>
       <c r="H55">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.25">
@@ -3632,10 +3635,10 @@
         <v>9</v>
       </c>
       <c r="C56" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="D56" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F56" t="s">
         <v>68</v>
@@ -3655,10 +3658,10 @@
         <v>9</v>
       </c>
       <c r="C57" t="s">
-        <v>128</v>
+        <v>79</v>
       </c>
       <c r="D57" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="F57" t="s">
         <v>68</v>
@@ -3678,10 +3681,10 @@
         <v>9</v>
       </c>
       <c r="C58" t="s">
-        <v>79</v>
+        <v>131</v>
       </c>
       <c r="D58" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="F58" t="s">
         <v>68</v>
@@ -3701,10 +3704,10 @@
         <v>9</v>
       </c>
       <c r="C59" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
       <c r="D59" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="F59" t="s">
         <v>68</v>
@@ -3724,10 +3727,10 @@
         <v>9</v>
       </c>
       <c r="C60" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="D60" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="F60" t="s">
         <v>68</v>
@@ -3744,13 +3747,13 @@
         <v>8</v>
       </c>
       <c r="B61" t="s">
-        <v>9</v>
+        <v>65</v>
       </c>
       <c r="C61" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="D61" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="F61" t="s">
         <v>68</v>
@@ -3770,10 +3773,10 @@
         <v>9</v>
       </c>
       <c r="C62" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="D62" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="F62" t="s">
         <v>68</v>
@@ -3793,10 +3796,10 @@
         <v>9</v>
       </c>
       <c r="C63" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="D63" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="F63" t="s">
         <v>68</v>
@@ -3816,10 +3819,10 @@
         <v>9</v>
       </c>
       <c r="C64" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="D64" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="F64" t="s">
         <v>68</v>
@@ -3839,10 +3842,10 @@
         <v>9</v>
       </c>
       <c r="C65" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="D65" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="F65" t="s">
         <v>68</v>
@@ -3862,10 +3865,10 @@
         <v>9</v>
       </c>
       <c r="C66" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="D66" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="F66" t="s">
         <v>68</v>
@@ -3885,10 +3888,10 @@
         <v>9</v>
       </c>
       <c r="C67" t="s">
-        <v>147</v>
+        <v>149</v>
       </c>
       <c r="D67" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="F67" t="s">
         <v>68</v>
@@ -3908,10 +3911,10 @@
         <v>9</v>
       </c>
       <c r="C68" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="D68" t="s">
-        <v>150</v>
+        <v>152</v>
       </c>
       <c r="F68" t="s">
         <v>68</v>
@@ -3931,10 +3934,10 @@
         <v>9</v>
       </c>
       <c r="C69" t="s">
-        <v>151</v>
+        <v>153</v>
       </c>
       <c r="D69" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="F69" t="s">
         <v>68</v>
@@ -3954,10 +3957,10 @@
         <v>9</v>
       </c>
       <c r="C70" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
       <c r="D70" t="s">
-        <v>154</v>
+        <v>156</v>
       </c>
       <c r="F70" t="s">
         <v>68</v>
@@ -3977,10 +3980,10 @@
         <v>9</v>
       </c>
       <c r="C71" t="s">
-        <v>155</v>
+        <v>157</v>
       </c>
       <c r="D71" t="s">
-        <v>156</v>
+        <v>158</v>
       </c>
       <c r="F71" t="s">
         <v>68</v>
@@ -4000,10 +4003,10 @@
         <v>9</v>
       </c>
       <c r="C72" t="s">
-        <v>157</v>
+        <v>159</v>
       </c>
       <c r="D72" t="s">
-        <v>158</v>
+        <v>160</v>
       </c>
       <c r="F72" t="s">
         <v>68</v>
@@ -4023,10 +4026,10 @@
         <v>9</v>
       </c>
       <c r="C73" t="s">
-        <v>159</v>
+        <v>161</v>
       </c>
       <c r="D73" t="s">
-        <v>160</v>
+        <v>162</v>
       </c>
       <c r="F73" t="s">
         <v>68</v>
@@ -4046,10 +4049,10 @@
         <v>9</v>
       </c>
       <c r="C74" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D74" t="s">
-        <v>162</v>
+        <v>164</v>
       </c>
       <c r="F74" t="s">
         <v>68</v>
@@ -4069,10 +4072,10 @@
         <v>9</v>
       </c>
       <c r="C75" t="s">
-        <v>163</v>
+        <v>165</v>
       </c>
       <c r="D75" t="s">
-        <v>164</v>
+        <v>166</v>
       </c>
       <c r="F75" t="s">
         <v>68</v>
@@ -4089,13 +4092,16 @@
         <v>8</v>
       </c>
       <c r="B76" t="s">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="C76" t="s">
-        <v>165</v>
+        <v>167</v>
       </c>
       <c r="D76" t="s">
-        <v>166</v>
+        <v>168</v>
+      </c>
+      <c r="E76" t="s">
+        <v>169</v>
       </c>
       <c r="F76" t="s">
         <v>68</v>
@@ -4104,7 +4110,7 @@
         <v>13</v>
       </c>
       <c r="H76">
-        <v>0</v>
+        <v>17</v>
       </c>
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.25">
@@ -4115,13 +4121,13 @@
         <v>85</v>
       </c>
       <c r="C77" t="s">
-        <v>167</v>
+        <v>86</v>
       </c>
       <c r="D77" t="s">
-        <v>168</v>
+        <v>170</v>
       </c>
       <c r="E77" t="s">
-        <v>169</v>
+        <v>171</v>
       </c>
       <c r="F77" t="s">
         <v>68</v>
@@ -4130,7 +4136,7 @@
         <v>13</v>
       </c>
       <c r="H77">
-        <v>17</v>
+        <v>15</v>
       </c>
     </row>
     <row r="78" spans="1:8" x14ac:dyDescent="0.25">
@@ -4141,13 +4147,13 @@
         <v>85</v>
       </c>
       <c r="C78" t="s">
-        <v>86</v>
+        <v>172</v>
       </c>
       <c r="D78" t="s">
-        <v>170</v>
+        <v>173</v>
       </c>
       <c r="E78" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="F78" t="s">
         <v>68</v>
@@ -4156,7 +4162,7 @@
         <v>13</v>
       </c>
       <c r="H78">
-        <v>15</v>
+        <v>2</v>
       </c>
     </row>
     <row r="79" spans="1:8" x14ac:dyDescent="0.25">
@@ -4167,13 +4173,13 @@
         <v>85</v>
       </c>
       <c r="C79" t="s">
-        <v>172</v>
+        <v>92</v>
       </c>
       <c r="D79" t="s">
-        <v>173</v>
+        <v>175</v>
       </c>
       <c r="E79" t="s">
-        <v>174</v>
+        <v>176</v>
       </c>
       <c r="F79" t="s">
         <v>68</v>
@@ -4182,7 +4188,7 @@
         <v>13</v>
       </c>
       <c r="H79">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="80" spans="1:8" x14ac:dyDescent="0.25">
@@ -4193,13 +4199,10 @@
         <v>85</v>
       </c>
       <c r="C80" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D80" t="s">
-        <v>175</v>
-      </c>
-      <c r="E80" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="F80" t="s">
         <v>68</v>
@@ -4213,16 +4216,16 @@
     </row>
     <row r="81" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A81" t="s">
-        <v>8</v>
+        <v>65</v>
       </c>
       <c r="B81" t="s">
-        <v>85</v>
+        <v>65</v>
       </c>
       <c r="C81" t="s">
-        <v>96</v>
+        <v>100</v>
       </c>
       <c r="D81" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="F81" t="s">
         <v>68</v>
@@ -4231,7 +4234,7 @@
         <v>13</v>
       </c>
       <c r="H81">
-        <v>0</v>
+        <v>138</v>
       </c>
     </row>
     <row r="82" spans="1:8" x14ac:dyDescent="0.25">
@@ -4242,10 +4245,10 @@
         <v>65</v>
       </c>
       <c r="C82" t="s">
-        <v>100</v>
+        <v>69</v>
       </c>
       <c r="D82" t="s">
-        <v>178</v>
+        <v>179</v>
       </c>
       <c r="F82" t="s">
         <v>68</v>
@@ -4254,7 +4257,7 @@
         <v>13</v>
       </c>
       <c r="H82">
-        <v>138</v>
+        <v>97</v>
       </c>
     </row>
     <row r="83" spans="1:8" x14ac:dyDescent="0.25">
@@ -4265,10 +4268,10 @@
         <v>65</v>
       </c>
       <c r="C83" t="s">
-        <v>69</v>
+        <v>102</v>
       </c>
       <c r="D83" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="F83" t="s">
         <v>68</v>
@@ -4277,7 +4280,7 @@
         <v>13</v>
       </c>
       <c r="H83">
-        <v>97</v>
+        <v>90</v>
       </c>
     </row>
     <row r="84" spans="1:8" x14ac:dyDescent="0.25">
@@ -4288,10 +4291,10 @@
         <v>65</v>
       </c>
       <c r="C84" t="s">
-        <v>102</v>
+        <v>73</v>
       </c>
       <c r="D84" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="F84" t="s">
         <v>68</v>
@@ -4300,7 +4303,7 @@
         <v>13</v>
       </c>
       <c r="H84">
-        <v>90</v>
+        <v>41</v>
       </c>
     </row>
     <row r="85" spans="1:8" x14ac:dyDescent="0.25">
@@ -4311,10 +4314,10 @@
         <v>65</v>
       </c>
       <c r="C85" t="s">
-        <v>73</v>
+        <v>104</v>
       </c>
       <c r="D85" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="F85" t="s">
         <v>68</v>
@@ -4323,7 +4326,7 @@
         <v>13</v>
       </c>
       <c r="H85">
-        <v>41</v>
+        <v>31</v>
       </c>
     </row>
     <row r="86" spans="1:8" x14ac:dyDescent="0.25">
@@ -4334,10 +4337,10 @@
         <v>65</v>
       </c>
       <c r="C86" t="s">
-        <v>104</v>
+        <v>137</v>
       </c>
       <c r="D86" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="F86" t="s">
         <v>68</v>
@@ -4346,7 +4349,7 @@
         <v>13</v>
       </c>
       <c r="H86">
-        <v>31</v>
+        <v>10</v>
       </c>
     </row>
     <row r="87" spans="1:8" x14ac:dyDescent="0.25">
@@ -4357,10 +4360,10 @@
         <v>65</v>
       </c>
       <c r="C87" t="s">
-        <v>137</v>
+        <v>71</v>
       </c>
       <c r="D87" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
       <c r="F87" t="s">
         <v>68</v>
@@ -4369,21 +4372,21 @@
         <v>13</v>
       </c>
       <c r="H87">
-        <v>10</v>
+        <v>0</v>
       </c>
     </row>
     <row r="88" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A88" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B88" t="s">
-        <v>65</v>
+        <v>9</v>
       </c>
       <c r="C88" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="D88" t="s">
-        <v>184</v>
+        <v>185</v>
       </c>
       <c r="F88" t="s">
         <v>68</v>
@@ -4392,7 +4395,7 @@
         <v>13</v>
       </c>
       <c r="H88">
-        <v>0</v>
+        <v>113</v>
       </c>
     </row>
     <row r="89" spans="1:8" x14ac:dyDescent="0.25">
@@ -4403,10 +4406,10 @@
         <v>9</v>
       </c>
       <c r="C89" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="D89" t="s">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="F89" t="s">
         <v>68</v>
@@ -4415,7 +4418,7 @@
         <v>13</v>
       </c>
       <c r="H89">
-        <v>113</v>
+        <v>84</v>
       </c>
     </row>
     <row r="90" spans="1:8" x14ac:dyDescent="0.25">
@@ -4426,10 +4429,10 @@
         <v>9</v>
       </c>
       <c r="C90" t="s">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="D90" t="s">
-        <v>186</v>
+        <v>187</v>
       </c>
       <c r="F90" t="s">
         <v>68</v>
@@ -4438,7 +4441,7 @@
         <v>13</v>
       </c>
       <c r="H90">
-        <v>84</v>
+        <v>63</v>
       </c>
     </row>
     <row r="91" spans="1:8" x14ac:dyDescent="0.25">
@@ -4449,10 +4452,10 @@
         <v>9</v>
       </c>
       <c r="C91" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="D91" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
       <c r="F91" t="s">
         <v>68</v>
@@ -4461,7 +4464,7 @@
         <v>13</v>
       </c>
       <c r="H91">
-        <v>63</v>
+        <v>43</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.25">
@@ -4472,10 +4475,10 @@
         <v>9</v>
       </c>
       <c r="C92" t="s">
-        <v>69</v>
+        <v>77</v>
       </c>
       <c r="D92" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="F92" t="s">
         <v>68</v>
@@ -4484,7 +4487,7 @@
         <v>13</v>
       </c>
       <c r="H92">
-        <v>43</v>
+        <v>20</v>
       </c>
     </row>
     <row r="93" spans="1:8" x14ac:dyDescent="0.25">
@@ -4495,10 +4498,10 @@
         <v>9</v>
       </c>
       <c r="C93" t="s">
-        <v>77</v>
+        <v>83</v>
       </c>
       <c r="D93" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="F93" t="s">
         <v>68</v>
@@ -4507,7 +4510,7 @@
         <v>13</v>
       </c>
       <c r="H93">
-        <v>20</v>
+        <v>8</v>
       </c>
     </row>
     <row r="94" spans="1:8" x14ac:dyDescent="0.25">
@@ -4518,10 +4521,10 @@
         <v>9</v>
       </c>
       <c r="C94" t="s">
-        <v>83</v>
+        <v>111</v>
       </c>
       <c r="D94" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="F94" t="s">
         <v>68</v>
@@ -4530,7 +4533,7 @@
         <v>13</v>
       </c>
       <c r="H94">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="95" spans="1:8" x14ac:dyDescent="0.25">
@@ -4541,10 +4544,10 @@
         <v>9</v>
       </c>
       <c r="C95" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D95" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="F95" t="s">
         <v>68</v>
@@ -4564,10 +4567,10 @@
         <v>9</v>
       </c>
       <c r="C96" t="s">
-        <v>113</v>
+        <v>193</v>
       </c>
       <c r="D96" t="s">
-        <v>192</v>
+        <v>194</v>
       </c>
       <c r="F96" t="s">
         <v>68</v>
@@ -4587,10 +4590,10 @@
         <v>9</v>
       </c>
       <c r="C97" t="s">
-        <v>193</v>
+        <v>126</v>
       </c>
       <c r="D97" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="F97" t="s">
         <v>68</v>
@@ -4599,7 +4602,7 @@
         <v>13</v>
       </c>
       <c r="H97">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.25">
@@ -4610,10 +4613,10 @@
         <v>9</v>
       </c>
       <c r="C98" t="s">
-        <v>126</v>
+        <v>79</v>
       </c>
       <c r="D98" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="F98" t="s">
         <v>68</v>
@@ -4633,10 +4636,10 @@
         <v>9</v>
       </c>
       <c r="C99" t="s">
-        <v>79</v>
+        <v>197</v>
       </c>
       <c r="D99" t="s">
-        <v>196</v>
+        <v>198</v>
       </c>
       <c r="F99" t="s">
         <v>68</v>
@@ -4656,10 +4659,10 @@
         <v>9</v>
       </c>
       <c r="C100" t="s">
-        <v>197</v>
+        <v>66</v>
       </c>
       <c r="D100" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="F100" t="s">
         <v>68</v>
@@ -4679,10 +4682,10 @@
         <v>9</v>
       </c>
       <c r="C101" t="s">
-        <v>66</v>
+        <v>81</v>
       </c>
       <c r="D101" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="F101" t="s">
         <v>68</v>
@@ -4702,10 +4705,10 @@
         <v>9</v>
       </c>
       <c r="C102" t="s">
-        <v>81</v>
+        <v>149</v>
       </c>
       <c r="D102" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="F102" t="s">
         <v>68</v>
@@ -4722,13 +4725,13 @@
         <v>64</v>
       </c>
       <c r="B103" t="s">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="C103" t="s">
-        <v>149</v>
+        <v>90</v>
       </c>
       <c r="D103" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="F103" t="s">
         <v>68</v>
@@ -4737,7 +4740,7 @@
         <v>13</v>
       </c>
       <c r="H103">
-        <v>0</v>
+        <v>30</v>
       </c>
     </row>
     <row r="104" spans="1:8" x14ac:dyDescent="0.25">
@@ -4748,10 +4751,10 @@
         <v>85</v>
       </c>
       <c r="C104" t="s">
-        <v>90</v>
+        <v>86</v>
       </c>
       <c r="D104" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="F104" t="s">
         <v>68</v>
@@ -4760,7 +4763,7 @@
         <v>13</v>
       </c>
       <c r="H104">
-        <v>30</v>
+        <v>27</v>
       </c>
     </row>
     <row r="105" spans="1:8" x14ac:dyDescent="0.25">
@@ -4771,10 +4774,10 @@
         <v>85</v>
       </c>
       <c r="C105" t="s">
-        <v>86</v>
+        <v>94</v>
       </c>
       <c r="D105" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="F105" t="s">
         <v>68</v>
@@ -4783,7 +4786,7 @@
         <v>13</v>
       </c>
       <c r="H105">
-        <v>27</v>
+        <v>6</v>
       </c>
     </row>
     <row r="106" spans="1:8" x14ac:dyDescent="0.25">
@@ -4794,10 +4797,10 @@
         <v>85</v>
       </c>
       <c r="C106" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="D106" t="s">
-        <v>204</v>
+        <v>205</v>
       </c>
       <c r="F106" t="s">
         <v>68</v>
@@ -4806,7 +4809,7 @@
         <v>13</v>
       </c>
       <c r="H106">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="107" spans="1:8" x14ac:dyDescent="0.25">
@@ -4817,10 +4820,10 @@
         <v>85</v>
       </c>
       <c r="C107" t="s">
-        <v>92</v>
+        <v>96</v>
       </c>
       <c r="D107" t="s">
-        <v>205</v>
+        <v>206</v>
       </c>
       <c r="F107" t="s">
         <v>68</v>
@@ -4834,16 +4837,16 @@
     </row>
     <row r="108" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A108" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="B108" t="s">
-        <v>85</v>
+        <v>9</v>
       </c>
       <c r="C108" t="s">
-        <v>96</v>
+        <v>139</v>
       </c>
       <c r="D108" t="s">
-        <v>206</v>
+        <v>207</v>
       </c>
       <c r="F108" t="s">
         <v>68</v>
@@ -4852,7 +4855,7 @@
         <v>13</v>
       </c>
       <c r="H108">
-        <v>0</v>
+        <v>1387</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.25">
@@ -4863,10 +4866,10 @@
         <v>9</v>
       </c>
       <c r="C109" t="s">
-        <v>139</v>
+        <v>111</v>
       </c>
       <c r="D109" t="s">
-        <v>207</v>
+        <v>208</v>
       </c>
       <c r="F109" t="s">
         <v>68</v>
@@ -4875,7 +4878,7 @@
         <v>13</v>
       </c>
       <c r="H109">
-        <v>1387</v>
+        <v>531</v>
       </c>
     </row>
     <row r="110" spans="1:8" x14ac:dyDescent="0.25">
@@ -4886,10 +4889,10 @@
         <v>9</v>
       </c>
       <c r="C110" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="D110" t="s">
-        <v>208</v>
+        <v>209</v>
       </c>
       <c r="F110" t="s">
         <v>68</v>
@@ -4909,10 +4912,10 @@
         <v>9</v>
       </c>
       <c r="C111" t="s">
-        <v>113</v>
+        <v>210</v>
       </c>
       <c r="D111" t="s">
-        <v>209</v>
+        <v>211</v>
       </c>
       <c r="F111" t="s">
         <v>68</v>
@@ -4921,7 +4924,7 @@
         <v>13</v>
       </c>
       <c r="H111">
-        <v>531</v>
+        <v>501</v>
       </c>
     </row>
     <row r="112" spans="1:8" x14ac:dyDescent="0.25">
@@ -4932,10 +4935,10 @@
         <v>9</v>
       </c>
       <c r="C112" t="s">
-        <v>210</v>
+        <v>143</v>
       </c>
       <c r="D112" t="s">
-        <v>211</v>
+        <v>212</v>
       </c>
       <c r="F112" t="s">
         <v>68</v>
@@ -4944,7 +4947,7 @@
         <v>13</v>
       </c>
       <c r="H112">
-        <v>501</v>
+        <v>375</v>
       </c>
     </row>
     <row r="113" spans="1:8" x14ac:dyDescent="0.25">
@@ -4955,10 +4958,10 @@
         <v>9</v>
       </c>
       <c r="C113" t="s">
-        <v>143</v>
+        <v>69</v>
       </c>
       <c r="D113" t="s">
-        <v>212</v>
+        <v>213</v>
       </c>
       <c r="F113" t="s">
         <v>68</v>
@@ -4967,7 +4970,7 @@
         <v>13</v>
       </c>
       <c r="H113">
-        <v>375</v>
+        <v>283</v>
       </c>
     </row>
     <row r="114" spans="1:8" x14ac:dyDescent="0.25">
@@ -4978,10 +4981,10 @@
         <v>9</v>
       </c>
       <c r="C114" t="s">
-        <v>69</v>
+        <v>145</v>
       </c>
       <c r="D114" t="s">
-        <v>213</v>
+        <v>214</v>
       </c>
       <c r="F114" t="s">
         <v>68</v>
@@ -4990,7 +4993,7 @@
         <v>13</v>
       </c>
       <c r="H114">
-        <v>283</v>
+        <v>269</v>
       </c>
     </row>
     <row r="115" spans="1:8" x14ac:dyDescent="0.25">
@@ -5001,10 +5004,10 @@
         <v>9</v>
       </c>
       <c r="C115" t="s">
-        <v>145</v>
+        <v>83</v>
       </c>
       <c r="D115" t="s">
-        <v>214</v>
+        <v>215</v>
       </c>
       <c r="F115" t="s">
         <v>68</v>
@@ -5013,7 +5016,7 @@
         <v>13</v>
       </c>
       <c r="H115">
-        <v>269</v>
+        <v>241</v>
       </c>
     </row>
     <row r="116" spans="1:8" x14ac:dyDescent="0.25">
@@ -5024,10 +5027,10 @@
         <v>9</v>
       </c>
       <c r="C116" t="s">
-        <v>83</v>
+        <v>73</v>
       </c>
       <c r="D116" t="s">
-        <v>215</v>
+        <v>216</v>
       </c>
       <c r="F116" t="s">
         <v>68</v>
@@ -5036,7 +5039,7 @@
         <v>13</v>
       </c>
       <c r="H116">
-        <v>241</v>
+        <v>59</v>
       </c>
     </row>
     <row r="117" spans="1:8" x14ac:dyDescent="0.25">
@@ -5047,10 +5050,10 @@
         <v>9</v>
       </c>
       <c r="C117" t="s">
-        <v>73</v>
+        <v>107</v>
       </c>
       <c r="D117" t="s">
-        <v>216</v>
+        <v>217</v>
       </c>
       <c r="F117" t="s">
         <v>68</v>
@@ -5059,7 +5062,7 @@
         <v>13</v>
       </c>
       <c r="H117">
-        <v>59</v>
+        <v>52</v>
       </c>
     </row>
     <row r="118" spans="1:8" x14ac:dyDescent="0.25">
@@ -5070,10 +5073,10 @@
         <v>9</v>
       </c>
       <c r="C118" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="D118" t="s">
-        <v>217</v>
+        <v>218</v>
       </c>
       <c r="F118" t="s">
         <v>68</v>
@@ -5093,10 +5096,10 @@
         <v>9</v>
       </c>
       <c r="C119" t="s">
-        <v>109</v>
+        <v>165</v>
       </c>
       <c r="D119" t="s">
-        <v>218</v>
+        <v>219</v>
       </c>
       <c r="F119" t="s">
         <v>68</v>
@@ -5105,7 +5108,7 @@
         <v>13</v>
       </c>
       <c r="H119">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="120" spans="1:8" x14ac:dyDescent="0.25">
@@ -5116,10 +5119,10 @@
         <v>9</v>
       </c>
       <c r="C120" t="s">
-        <v>165</v>
+        <v>220</v>
       </c>
       <c r="D120" t="s">
-        <v>219</v>
+        <v>221</v>
       </c>
       <c r="F120" t="s">
         <v>68</v>
@@ -5128,7 +5131,7 @@
         <v>13</v>
       </c>
       <c r="H120">
-        <v>51</v>
+        <v>31</v>
       </c>
     </row>
     <row r="121" spans="1:8" x14ac:dyDescent="0.25">
@@ -5139,10 +5142,10 @@
         <v>9</v>
       </c>
       <c r="C121" t="s">
-        <v>220</v>
+        <v>66</v>
       </c>
       <c r="D121" t="s">
-        <v>221</v>
+        <v>222</v>
       </c>
       <c r="F121" t="s">
         <v>68</v>
@@ -5151,7 +5154,7 @@
         <v>13</v>
       </c>
       <c r="H121">
-        <v>31</v>
+        <v>14</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.25">
@@ -5162,10 +5165,10 @@
         <v>9</v>
       </c>
       <c r="C122" t="s">
-        <v>66</v>
+        <v>223</v>
       </c>
       <c r="D122" t="s">
-        <v>222</v>
+        <v>224</v>
       </c>
       <c r="F122" t="s">
         <v>68</v>
@@ -5174,7 +5177,7 @@
         <v>13</v>
       </c>
       <c r="H122">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="123" spans="1:8" x14ac:dyDescent="0.25">
@@ -5185,10 +5188,10 @@
         <v>9</v>
       </c>
       <c r="C123" t="s">
-        <v>223</v>
+        <v>225</v>
       </c>
       <c r="D123" t="s">
-        <v>224</v>
+        <v>226</v>
       </c>
       <c r="F123" t="s">
         <v>68</v>
@@ -5197,7 +5200,7 @@
         <v>13</v>
       </c>
       <c r="H123">
-        <v>12</v>
+        <v>7</v>
       </c>
     </row>
     <row r="124" spans="1:8" x14ac:dyDescent="0.25">
@@ -5208,10 +5211,10 @@
         <v>9</v>
       </c>
       <c r="C124" t="s">
-        <v>225</v>
+        <v>126</v>
       </c>
       <c r="D124" t="s">
-        <v>226</v>
+        <v>227</v>
       </c>
       <c r="F124" t="s">
         <v>68</v>
@@ -5220,7 +5223,7 @@
         <v>13</v>
       </c>
       <c r="H124">
-        <v>7</v>
+        <v>5</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.25">
@@ -5231,10 +5234,10 @@
         <v>9</v>
       </c>
       <c r="C125" t="s">
-        <v>126</v>
+        <v>161</v>
       </c>
       <c r="D125" t="s">
-        <v>227</v>
+        <v>228</v>
       </c>
       <c r="F125" t="s">
         <v>68</v>
@@ -5243,7 +5246,7 @@
         <v>13</v>
       </c>
       <c r="H125">
-        <v>5</v>
+        <v>3</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.25">
@@ -5254,10 +5257,10 @@
         <v>9</v>
       </c>
       <c r="C126" t="s">
-        <v>161</v>
+        <v>163</v>
       </c>
       <c r="D126" t="s">
-        <v>228</v>
+        <v>229</v>
       </c>
       <c r="F126" t="s">
         <v>68</v>
@@ -5277,10 +5280,10 @@
         <v>9</v>
       </c>
       <c r="C127" t="s">
-        <v>163</v>
+        <v>230</v>
       </c>
       <c r="D127" t="s">
-        <v>229</v>
+        <v>231</v>
       </c>
       <c r="F127" t="s">
         <v>68</v>
@@ -5289,7 +5292,7 @@
         <v>13</v>
       </c>
       <c r="H127">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.25">
@@ -5300,10 +5303,10 @@
         <v>9</v>
       </c>
       <c r="C128" t="s">
-        <v>230</v>
+        <v>81</v>
       </c>
       <c r="D128" t="s">
-        <v>231</v>
+        <v>232</v>
       </c>
       <c r="F128" t="s">
         <v>68</v>
@@ -5323,10 +5326,10 @@
         <v>9</v>
       </c>
       <c r="C129" t="s">
-        <v>81</v>
+        <v>124</v>
       </c>
       <c r="D129" t="s">
-        <v>232</v>
+        <v>233</v>
       </c>
       <c r="F129" t="s">
         <v>68</v>
@@ -5346,10 +5349,10 @@
         <v>9</v>
       </c>
       <c r="C130" t="s">
-        <v>124</v>
+        <v>128</v>
       </c>
       <c r="D130" t="s">
-        <v>233</v>
+        <v>234</v>
       </c>
       <c r="F130" t="s">
         <v>68</v>
@@ -5358,7 +5361,7 @@
         <v>13</v>
       </c>
       <c r="H130">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="131" spans="1:8" x14ac:dyDescent="0.25">
@@ -5369,10 +5372,10 @@
         <v>9</v>
       </c>
       <c r="C131" t="s">
-        <v>128</v>
+        <v>147</v>
       </c>
       <c r="D131" t="s">
-        <v>234</v>
+        <v>235</v>
       </c>
       <c r="F131" t="s">
         <v>68</v>
@@ -5392,10 +5395,10 @@
         <v>9</v>
       </c>
       <c r="C132" t="s">
-        <v>147</v>
+        <v>236</v>
       </c>
       <c r="D132" t="s">
-        <v>235</v>
+        <v>237</v>
       </c>
       <c r="F132" t="s">
         <v>68</v>
@@ -5415,10 +5418,10 @@
         <v>9</v>
       </c>
       <c r="C133" t="s">
-        <v>236</v>
+        <v>79</v>
       </c>
       <c r="D133" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="F133" t="s">
         <v>68</v>
@@ -5427,7 +5430,7 @@
         <v>13</v>
       </c>
       <c r="H133">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.25">
@@ -5438,10 +5441,10 @@
         <v>9</v>
       </c>
       <c r="C134" t="s">
-        <v>79</v>
+        <v>197</v>
       </c>
       <c r="D134" t="s">
-        <v>238</v>
+        <v>239</v>
       </c>
       <c r="F134" t="s">
         <v>68</v>
@@ -5461,10 +5464,10 @@
         <v>9</v>
       </c>
       <c r="C135" t="s">
-        <v>197</v>
+        <v>135</v>
       </c>
       <c r="D135" t="s">
-        <v>239</v>
+        <v>240</v>
       </c>
       <c r="F135" t="s">
         <v>68</v>
@@ -5484,10 +5487,10 @@
         <v>9</v>
       </c>
       <c r="C136" t="s">
-        <v>135</v>
+        <v>141</v>
       </c>
       <c r="D136" t="s">
-        <v>240</v>
+        <v>241</v>
       </c>
       <c r="F136" t="s">
         <v>68</v>
@@ -5507,10 +5510,10 @@
         <v>9</v>
       </c>
       <c r="C137" t="s">
-        <v>141</v>
+        <v>242</v>
       </c>
       <c r="D137" t="s">
-        <v>241</v>
+        <v>243</v>
       </c>
       <c r="F137" t="s">
         <v>68</v>
@@ -5530,10 +5533,10 @@
         <v>9</v>
       </c>
       <c r="C138" t="s">
-        <v>242</v>
+        <v>244</v>
       </c>
       <c r="D138" t="s">
-        <v>243</v>
+        <v>245</v>
       </c>
       <c r="F138" t="s">
         <v>68</v>
@@ -5553,10 +5556,10 @@
         <v>9</v>
       </c>
       <c r="C139" t="s">
-        <v>244</v>
+        <v>153</v>
       </c>
       <c r="D139" t="s">
-        <v>245</v>
+        <v>246</v>
       </c>
       <c r="F139" t="s">
         <v>68</v>
@@ -5576,10 +5579,10 @@
         <v>9</v>
       </c>
       <c r="C140" t="s">
-        <v>153</v>
+        <v>247</v>
       </c>
       <c r="D140" t="s">
-        <v>246</v>
+        <v>248</v>
       </c>
       <c r="F140" t="s">
         <v>68</v>
@@ -5599,10 +5602,10 @@
         <v>9</v>
       </c>
       <c r="C141" t="s">
-        <v>247</v>
+        <v>249</v>
       </c>
       <c r="D141" t="s">
-        <v>248</v>
+        <v>250</v>
       </c>
       <c r="F141" t="s">
         <v>68</v>
@@ -5622,10 +5625,10 @@
         <v>9</v>
       </c>
       <c r="C142" t="s">
-        <v>249</v>
+        <v>251</v>
       </c>
       <c r="D142" t="s">
-        <v>250</v>
+        <v>252</v>
       </c>
       <c r="F142" t="s">
         <v>68</v>
@@ -5645,10 +5648,10 @@
         <v>9</v>
       </c>
       <c r="C143" t="s">
-        <v>251</v>
+        <v>253</v>
       </c>
       <c r="D143" t="s">
-        <v>252</v>
+        <v>254</v>
       </c>
       <c r="F143" t="s">
         <v>68</v>
@@ -5668,10 +5671,10 @@
         <v>9</v>
       </c>
       <c r="C144" t="s">
-        <v>253</v>
+        <v>255</v>
       </c>
       <c r="D144" t="s">
-        <v>254</v>
+        <v>256</v>
       </c>
       <c r="F144" t="s">
         <v>68</v>
@@ -5691,10 +5694,10 @@
         <v>9</v>
       </c>
       <c r="C145" t="s">
-        <v>255</v>
+        <v>257</v>
       </c>
       <c r="D145" t="s">
-        <v>256</v>
+        <v>258</v>
       </c>
       <c r="F145" t="s">
         <v>68</v>
@@ -5714,10 +5717,10 @@
         <v>9</v>
       </c>
       <c r="C146" t="s">
-        <v>257</v>
+        <v>259</v>
       </c>
       <c r="D146" t="s">
-        <v>258</v>
+        <v>260</v>
       </c>
       <c r="F146" t="s">
         <v>68</v>
@@ -5737,10 +5740,10 @@
         <v>9</v>
       </c>
       <c r="C147" t="s">
-        <v>259</v>
+        <v>261</v>
       </c>
       <c r="D147" t="s">
-        <v>260</v>
+        <v>262</v>
       </c>
       <c r="F147" t="s">
         <v>68</v>
@@ -5757,13 +5760,13 @@
         <v>63</v>
       </c>
       <c r="B148" t="s">
-        <v>9</v>
+        <v>85</v>
       </c>
       <c r="C148" t="s">
-        <v>261</v>
+        <v>96</v>
       </c>
       <c r="D148" t="s">
-        <v>262</v>
+        <v>263</v>
       </c>
       <c r="F148" t="s">
         <v>68</v>
@@ -5775,31 +5778,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="149" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A149" t="s">
-        <v>63</v>
-      </c>
-      <c r="B149" t="s">
-        <v>85</v>
-      </c>
-      <c r="C149" t="s">
-        <v>96</v>
-      </c>
-      <c r="D149" t="s">
-        <v>263</v>
-      </c>
-      <c r="F149" t="s">
-        <v>68</v>
-      </c>
-      <c r="G149" t="s">
-        <v>13</v>
-      </c>
-      <c r="H149">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H149" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
+  <autoFilter ref="A1:H148" xr:uid="{00000000-0009-0000-0000-000000000000}"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-26 16:40) - 125 informes de Power BI y 24 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -545,7 +545,11 @@
           <t>https://reporteventashtml.vercel.app/</t>
         </is>
       </c>
-      <c r="E3" t="inlineStr"/>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Resumen de ventas, objetivos, margenes y visitas. Mayorista- Distribución - MC</t>
+        </is>
+      </c>
       <c r="F3" t="inlineStr">
         <is>
           <t>MANUAL</t>
@@ -1213,7 +1217,11 @@
           <t>https://reporteventashtml.vercel.app/</t>
         </is>
       </c>
-      <c r="E21" t="inlineStr"/>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Resumen de ventas, objetivos, margenes y visitas. Mayorista- Distribución - MC</t>
+        </is>
+      </c>
       <c r="F21" t="inlineStr">
         <is>
           <t>MANUAL</t>
@@ -1247,7 +1255,11 @@
           <t>https://reporteventashtml.vercel.app/</t>
         </is>
       </c>
-      <c r="E22" t="inlineStr"/>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Resumen de ventas, objetivos, margenes y visitas. Mayorista- Distribución - MC</t>
+        </is>
+      </c>
       <c r="F22" t="inlineStr">
         <is>
           <t>MANUAL</t>
@@ -1281,7 +1293,11 @@
           <t>https://reporteventashtml.vercel.app/</t>
         </is>
       </c>
-      <c r="E23" t="inlineStr"/>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Resumen de ventas, objetivos, margenes y visitas. Mayorista- Distribución - MC</t>
+        </is>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>MANUAL</t>
@@ -1297,25 +1313,29 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>FINANZAS</t>
+          <t>JEFES</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>PRINCIPAL</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE OBJETIVOS</t>
+          <t>REPORTE DE VENTAS</t>
         </is>
       </c>
       <c r="D24" t="inlineStr">
         <is>
-          <t>https://objetivos-hergo.vercel.app/</t>
-        </is>
-      </c>
-      <c r="E24" t="inlineStr"/>
+          <t>https://reporteventashtml.vercel.app/</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Resumen de ventas, objetivos, margenes y visitas. Mayorista- Distribución - MC</t>
+        </is>
+      </c>
       <c r="F24" t="inlineStr">
         <is>
           <t>MANUAL</t>
@@ -1331,22 +1351,22 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>JEFES</t>
+          <t>FINANZAS</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>PRINCIPAL</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>REPORTE DE VENTAS</t>
+          <t>SEGUIMIENTO DE OBJETIVOS</t>
         </is>
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>https://reporteventashtml.vercel.app/</t>
+          <t>https://objetivos-hergo.vercel.app/</t>
         </is>
       </c>
       <c r="E25" t="inlineStr"/>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-27 07:44) - 125 informes de Power BI y 24 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1451,7 +1451,7 @@
         </is>
       </c>
       <c r="H27" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="28">
@@ -1487,7 +1487,7 @@
         </is>
       </c>
       <c r="H28" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="29">
@@ -1539,12 +1539,12 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D30" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E30" t="inlineStr"/>
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="31">
@@ -1575,12 +1575,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5f8aa5de-6aa2-4988-9c94-be9e74274da5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1595,7 +1595,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="32">
@@ -2079,12 +2079,12 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>COMPARATIVO 07-2026</t>
         </is>
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=402b5c26-c94e-44f2-958b-e71cb071ff31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E45" t="inlineStr"/>
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="46">
@@ -2115,12 +2115,12 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E46" t="inlineStr"/>
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="47">
@@ -2151,12 +2151,12 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="D47" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4a1bcca-eca1-41bf-bcf3-86fd0a8decd8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E47" t="inlineStr"/>
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="48">
@@ -2187,12 +2187,12 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D48" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=402b5c26-c94e-44f2-958b-e71cb071ff31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E48" t="inlineStr"/>
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>25</v>
+        <v>27</v>
       </c>
     </row>
     <row r="49">
@@ -2223,12 +2223,12 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D49" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=595175a9-fe3a-49ce-abde-bd1b578273ff&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E49" t="inlineStr"/>
@@ -2243,7 +2243,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="50">
@@ -2279,7 +2279,7 @@
         </is>
       </c>
       <c r="H50" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="51">
@@ -2403,12 +2403,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2439,12 +2439,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2459,7 +2459,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="56">
@@ -2475,12 +2475,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2511,12 +2511,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2531,7 +2531,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -3771,7 +3771,7 @@
         </is>
       </c>
       <c r="H91" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="92">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="93">
@@ -3843,7 +3843,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="94">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="95">
@@ -4311,7 +4311,7 @@
         </is>
       </c>
       <c r="H106" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="107">
@@ -4363,12 +4363,12 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MERMAS MC</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D108" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b82ed9fb-5d10-495d-9a6d-b0b617fdd487&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=243f52b1-78cb-4c1a-9689-e0f18217f77a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E108" t="inlineStr"/>
@@ -4383,7 +4383,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="109">
@@ -4399,12 +4399,12 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>MERMAS MC</t>
         </is>
       </c>
       <c r="D109" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=243f52b1-78cb-4c1a-9689-e0f18217f77a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b82ed9fb-5d10-495d-9a6d-b0b617fdd487&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E109" t="inlineStr"/>
@@ -4455,7 +4455,7 @@
         </is>
       </c>
       <c r="H110" t="n">
-        <v>1396</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="111">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>542</v>
+        <v>551</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>542</v>
+        <v>551</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>368</v>
+        <v>358</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="118">
@@ -4743,7 +4743,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="119">
@@ -4851,7 +4851,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="122">
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="126">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
     </row>
     <row r="127">
@@ -5047,12 +5047,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5067,7 +5067,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="128">
@@ -6074,7 +6074,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="4">
@@ -6250,7 +6250,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>5</v>
+        <v>9</v>
       </c>
     </row>
     <row r="8">
@@ -6470,7 +6470,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="13">
@@ -6734,7 +6734,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="19">
@@ -7662,7 +7662,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="36">
@@ -8854,7 +8854,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
     </row>
     <row r="59">
@@ -10562,7 +10562,7 @@
         </is>
       </c>
       <c r="L92" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="93">
@@ -11430,7 +11430,7 @@
         </is>
       </c>
       <c r="L111" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="112">
@@ -11562,7 +11562,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
     </row>
     <row r="115">
@@ -11606,7 +11606,7 @@
         </is>
       </c>
       <c r="L115" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="116">
@@ -11650,7 +11650,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>84</v>
+        <v>86</v>
       </c>
     </row>
     <row r="117">
@@ -11826,7 +11826,7 @@
         </is>
       </c>
       <c r="L120" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="121">
@@ -11870,7 +11870,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>70</v>
+        <v>73</v>
       </c>
     </row>
     <row r="122">
@@ -12246,7 +12246,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="130">
@@ -12302,7 +12302,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="131">
@@ -12750,7 +12750,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>107</v>
+        <v>95</v>
       </c>
     </row>
     <row r="139">
@@ -12918,7 +12918,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>182</v>
+        <v>191</v>
       </c>
     </row>
     <row r="142">
@@ -13094,7 +13094,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>496</v>
+        <v>499</v>
       </c>
     </row>
     <row r="146">
@@ -13182,7 +13182,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>270</v>
+        <v>275</v>
       </c>
     </row>
     <row r="148">
@@ -13786,7 +13786,7 @@
         </is>
       </c>
       <c r="L158" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="159">
@@ -13842,7 +13842,7 @@
         </is>
       </c>
       <c r="L159" t="n">
-        <v>23</v>
+        <v>21</v>
       </c>
     </row>
     <row r="160">
@@ -14098,7 +14098,7 @@
         </is>
       </c>
       <c r="L164" t="n">
-        <v>1396</v>
+        <v>1406</v>
       </c>
     </row>
     <row r="165">
@@ -14186,7 +14186,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>368</v>
+        <v>358</v>
       </c>
     </row>
     <row r="167">
@@ -14230,7 +14230,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>270</v>
+        <v>268</v>
       </c>
     </row>
     <row r="168">
@@ -14406,7 +14406,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>252</v>
+        <v>258</v>
       </c>
     </row>
     <row r="172">
@@ -16138,7 +16138,7 @@
         </is>
       </c>
       <c r="L203" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
     </row>
     <row r="204">
@@ -16362,7 +16362,7 @@
         </is>
       </c>
       <c r="L207" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
     </row>
     <row r="208">
@@ -16582,7 +16582,7 @@
         </is>
       </c>
       <c r="L212" t="n">
-        <v>51</v>
+        <v>50</v>
       </c>
     </row>
     <row r="213">
@@ -16670,7 +16670,7 @@
         </is>
       </c>
       <c r="L214" t="n">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-28 07:45) - 124 informes de Power BI y 24 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$150</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$214</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$149</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$213</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H150"/>
+  <dimension ref="A1:H149"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1523,7 +1523,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="30">
@@ -1559,7 +1559,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="31">
@@ -2099,7 +2099,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="46">
@@ -2135,7 +2135,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="47">
@@ -2171,7 +2171,7 @@
         </is>
       </c>
       <c r="H47" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="48">
@@ -2207,7 +2207,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="49">
@@ -3735,7 +3735,7 @@
         </is>
       </c>
       <c r="H90" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="91">
@@ -3807,7 +3807,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="93">
@@ -3879,7 +3879,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="95">
@@ -4491,7 +4491,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>551</v>
+        <v>568</v>
       </c>
     </row>
     <row r="112">
@@ -4527,7 +4527,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>551</v>
+        <v>568</v>
       </c>
     </row>
     <row r="113">
@@ -4563,7 +4563,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>499</v>
+        <v>483</v>
       </c>
     </row>
     <row r="114">
@@ -4599,7 +4599,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="115">
@@ -4635,7 +4635,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="116">
@@ -4671,7 +4671,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="117">
@@ -4707,7 +4707,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="118">
@@ -4723,12 +4723,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=bdfe582a-c303-4732-b9b7-2390e04aa58e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5a75e8c7-9e82-4d6f-975a-72bbb3434a4d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4759,12 +4759,12 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D119" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5a75e8c7-9e82-4d6f-975a-72bbb3434a4d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E119" t="inlineStr"/>
@@ -4779,7 +4779,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="120">
@@ -4795,12 +4795,12 @@
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=bdfe582a-c303-4732-b9b7-2390e04aa58e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E120" t="inlineStr"/>
@@ -4815,7 +4815,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>53</v>
+        <v>58</v>
       </c>
     </row>
     <row r="121">
@@ -4939,12 +4939,12 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>NUEVO BRANCA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="D124" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=41d0a85e-4b61-46bc-9850-5984ff419dd1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E124" t="inlineStr"/>
@@ -4959,7 +4959,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="125">
@@ -4975,12 +4975,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4995,7 +4995,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>10</v>
+        <v>13</v>
       </c>
     </row>
     <row r="126">
@@ -5011,12 +5011,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5031,7 +5031,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127">
@@ -5083,12 +5083,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5103,7 +5103,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>5</v>
+        <v>2</v>
       </c>
     </row>
     <row r="129">
@@ -5119,12 +5119,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5155,12 +5155,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5191,12 +5191,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5211,7 +5211,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="132">
@@ -5227,12 +5227,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5299,12 +5299,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ea6316b-51ca-4d99-80cb-c767aeaeb217&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5355,7 +5355,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="136">
@@ -5371,12 +5371,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5391,7 +5391,7 @@
         </is>
       </c>
       <c r="H136" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="137">
@@ -5407,12 +5407,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5443,12 +5443,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5479,12 +5479,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5515,12 +5515,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5551,12 +5551,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5587,12 +5587,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5623,12 +5623,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5659,12 +5659,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5695,12 +5695,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5731,12 +5731,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5767,12 +5767,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5803,12 +5803,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ea6316b-51ca-4d99-80cb-c767aeaeb217&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -5834,17 +5834,17 @@
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -5862,44 +5862,8 @@
         <v>0</v>
       </c>
     </row>
-    <row r="150">
-      <c r="A150" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="B150" t="inlineStr">
-        <is>
-          <t>MENOR COSTE</t>
-        </is>
-      </c>
-      <c r="C150" t="inlineStr">
-        <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="D150" t="inlineStr">
-        <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
-        </is>
-      </c>
-      <c r="E150" t="inlineStr"/>
-      <c r="F150" t="inlineStr">
-        <is>
-          <t>API</t>
-        </is>
-      </c>
-      <c r="G150" t="inlineStr">
-        <is>
-          <t>INFORME</t>
-        </is>
-      </c>
-      <c r="H150" t="n">
-        <v>0</v>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:H150"/>
+  <autoFilter ref="A1:H149"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5910,7 +5874,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L214"/>
+  <dimension ref="A1:L213"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6250,7 +6214,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="8">
@@ -6690,7 +6654,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="18">
@@ -7662,7 +7626,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -8854,7 +8818,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="59">
@@ -11562,7 +11526,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
     </row>
     <row r="115">
@@ -11870,7 +11834,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>73</v>
+        <v>75</v>
       </c>
     </row>
     <row r="122">
@@ -12046,7 +12010,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>113</v>
+        <v>114</v>
       </c>
     </row>
     <row r="126">
@@ -12090,7 +12054,7 @@
         </is>
       </c>
       <c r="L126" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="127">
@@ -12246,7 +12210,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="130">
@@ -12694,7 +12658,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>56</v>
+        <v>54</v>
       </c>
     </row>
     <row r="138">
@@ -12750,7 +12714,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>95</v>
+        <v>70</v>
       </c>
     </row>
     <row r="139">
@@ -12918,7 +12882,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>191</v>
+        <v>208</v>
       </c>
     </row>
     <row r="142">
@@ -13006,7 +12970,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -13094,7 +13058,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>499</v>
+        <v>483</v>
       </c>
     </row>
     <row r="146">
@@ -13182,7 +13146,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>275</v>
+        <v>280</v>
       </c>
     </row>
     <row r="148">
@@ -13842,7 +13806,7 @@
         </is>
       </c>
       <c r="L159" t="n">
-        <v>21</v>
+        <v>19</v>
       </c>
     </row>
     <row r="160">
@@ -14010,7 +13974,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>12</v>
+        <v>17</v>
       </c>
     </row>
     <row r="163">
@@ -14186,7 +14150,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="167">
@@ -14230,7 +14194,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>268</v>
+        <v>265</v>
       </c>
     </row>
     <row r="168">
@@ -14406,7 +14370,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>258</v>
+        <v>262</v>
       </c>
     </row>
     <row r="172">
@@ -14471,18 +14435,30 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>NUEVO BRANCA</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>PARTICIPACION VENTAS CCU</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>NUEVO BRANCA</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr"/>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14490,11 +14466,11 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>41d0a85e-4b61-46bc-9850-5984ff419dd1</t>
+          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
       </c>
       <c r="L173" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
     </row>
     <row r="174">
@@ -14515,30 +14491,18 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
-      <c r="F174" t="inlineStr">
-        <is>
-          <t>PARTICIPACION VENTAS CCU</t>
-        </is>
-      </c>
-      <c r="G174" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F174" t="inlineStr"/>
+      <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
-        </is>
-      </c>
-      <c r="I174" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>PLAN ESPACIO APP ALTA</t>
+        </is>
+      </c>
+      <c r="I174" t="inlineStr"/>
       <c r="J174" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14546,7 +14510,7 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
+          <t>784d6896-dd8a-4b7a-9c5c-962ea6c5e49c</t>
         </is>
       </c>
       <c r="L174" t="n">
@@ -14571,18 +14535,30 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+        </is>
+      </c>
+      <c r="E175" t="inlineStr"/>
+      <c r="F175" t="inlineStr">
+        <is>
           <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
-      <c r="E175" t="inlineStr"/>
-      <c r="F175" t="inlineStr"/>
-      <c r="G175" t="inlineStr"/>
+      <c r="G175" t="inlineStr">
+        <is>
+          <t>08-2025</t>
+        </is>
+      </c>
       <c r="H175" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
-        </is>
-      </c>
-      <c r="I175" t="inlineStr"/>
+          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
+        </is>
+      </c>
+      <c r="I175" t="inlineStr">
+        <is>
+          <t>Agosto - 25</t>
+        </is>
+      </c>
       <c r="J175" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14590,7 +14566,7 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>784d6896-dd8a-4b7a-9c5c-962ea6c5e49c</t>
+          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
       </c>
       <c r="L175" t="n">
@@ -14615,30 +14591,18 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
-      <c r="F176" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP ALTA</t>
-        </is>
-      </c>
-      <c r="G176" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
+      <c r="F176" t="inlineStr"/>
+      <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
-        </is>
-      </c>
-      <c r="I176" t="inlineStr">
-        <is>
-          <t>Agosto - 25</t>
-        </is>
-      </c>
+          <t>PLAN ESPACIO APP COSTA</t>
+        </is>
+      </c>
+      <c r="I176" t="inlineStr"/>
       <c r="J176" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14646,7 +14610,7 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
+          <t>08eee5c2-f90d-483d-9382-0726090489f7</t>
         </is>
       </c>
       <c r="L176" t="n">
@@ -14671,18 +14635,30 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+        </is>
+      </c>
+      <c r="E177" t="inlineStr"/>
+      <c r="F177" t="inlineStr">
+        <is>
           <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
-      <c r="E177" t="inlineStr"/>
-      <c r="F177" t="inlineStr"/>
-      <c r="G177" t="inlineStr"/>
+      <c r="G177" t="inlineStr">
+        <is>
+          <t>08-2025</t>
+        </is>
+      </c>
       <c r="H177" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
-        </is>
-      </c>
-      <c r="I177" t="inlineStr"/>
+          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
+        </is>
+      </c>
+      <c r="I177" t="inlineStr">
+        <is>
+          <t>Agosto - 25</t>
+        </is>
+      </c>
       <c r="J177" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14690,7 +14666,7 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>08eee5c2-f90d-483d-9382-0726090489f7</t>
+          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
       </c>
       <c r="L177" t="n">
@@ -14710,35 +14686,23 @@
       </c>
       <c r="C178" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
-      <c r="F178" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP COSTA</t>
-        </is>
-      </c>
-      <c r="G178" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
+      <c r="F178" t="inlineStr"/>
+      <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
-        </is>
-      </c>
-      <c r="I178" t="inlineStr">
-        <is>
-          <t>Agosto - 25</t>
-        </is>
-      </c>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+        </is>
+      </c>
+      <c r="I178" t="inlineStr"/>
       <c r="J178" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14746,7 +14710,7 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
+          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
       <c r="L178" t="n">
@@ -14766,23 +14730,35 @@
       </c>
       <c r="C179" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
-      <c r="F179" t="inlineStr"/>
-      <c r="G179" t="inlineStr"/>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO DE MARCAS</t>
+        </is>
+      </c>
+      <c r="G179" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H179" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
-        </is>
-      </c>
-      <c r="I179" t="inlineStr"/>
+          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+        </is>
+      </c>
+      <c r="I179" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J179" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14790,7 +14766,7 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
+          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
       <c r="L179" t="n">
@@ -14815,7 +14791,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -14826,17 +14802,17 @@
       </c>
       <c r="G180" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H180" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
         </is>
       </c>
       <c r="I180" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J180" t="inlineStr">
@@ -14846,7 +14822,7 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
+          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
       <c r="L180" t="n">
@@ -14871,7 +14847,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -14882,17 +14858,17 @@
       </c>
       <c r="G181" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H181" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
         </is>
       </c>
       <c r="I181" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J181" t="inlineStr">
@@ -14902,7 +14878,7 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
+          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
       <c r="L181" t="n">
@@ -14927,7 +14903,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
@@ -14938,17 +14914,17 @@
       </c>
       <c r="G182" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H182" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
         </is>
       </c>
       <c r="I182" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J182" t="inlineStr">
@@ -14958,7 +14934,7 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
+          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
       <c r="L182" t="n">
@@ -14983,7 +14959,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
@@ -14994,17 +14970,17 @@
       </c>
       <c r="G183" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H183" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
         </is>
       </c>
       <c r="I183" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J183" t="inlineStr">
@@ -15014,7 +14990,7 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
+          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
       <c r="L183" t="n">
@@ -15039,7 +15015,7 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
@@ -15050,17 +15026,17 @@
       </c>
       <c r="G184" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H184" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
         </is>
       </c>
       <c r="I184" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J184" t="inlineStr">
@@ -15070,7 +15046,7 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
+          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
       <c r="L184" t="n">
@@ -15095,7 +15071,7 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
@@ -15106,17 +15082,17 @@
       </c>
       <c r="G185" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
         </is>
       </c>
       <c r="I185" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J185" t="inlineStr">
@@ -15126,7 +15102,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
+          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
       <c r="L185" t="n">
@@ -15151,7 +15127,7 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
@@ -15162,17 +15138,17 @@
       </c>
       <c r="G186" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H186" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
         </is>
       </c>
       <c r="I186" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J186" t="inlineStr">
@@ -15182,7 +15158,7 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
+          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
       <c r="L186" t="n">
@@ -15207,7 +15183,7 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
@@ -15218,17 +15194,17 @@
       </c>
       <c r="G187" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
         </is>
       </c>
       <c r="I187" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J187" t="inlineStr">
@@ -15238,7 +15214,7 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
+          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
       <c r="L187" t="n">
@@ -15263,7 +15239,7 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
@@ -15274,17 +15250,17 @@
       </c>
       <c r="G188" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H188" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
         </is>
       </c>
       <c r="I188" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J188" t="inlineStr">
@@ -15294,11 +15270,11 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
+          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
       <c r="L188" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="189">
@@ -15319,7 +15295,7 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
@@ -15330,17 +15306,17 @@
       </c>
       <c r="G189" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
         </is>
       </c>
       <c r="I189" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J189" t="inlineStr">
@@ -15350,11 +15326,11 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
+          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
       <c r="L189" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190">
@@ -15375,7 +15351,7 @@
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -15386,17 +15362,17 @@
       </c>
       <c r="G190" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H190" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
         </is>
       </c>
       <c r="I190" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J190" t="inlineStr">
@@ -15406,7 +15382,7 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
+          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
       <c r="L190" t="n">
@@ -15431,7 +15407,7 @@
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -15442,17 +15418,17 @@
       </c>
       <c r="G191" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H191" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
         </is>
       </c>
       <c r="I191" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J191" t="inlineStr">
@@ -15462,7 +15438,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
+          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
       <c r="L191" t="n">
@@ -15487,7 +15463,7 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
@@ -15498,17 +15474,17 @@
       </c>
       <c r="G192" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
         </is>
       </c>
       <c r="I192" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J192" t="inlineStr">
@@ -15518,11 +15494,11 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
+          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
       <c r="L192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="193">
@@ -15543,28 +15519,28 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
       <c r="F193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
         </is>
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -15574,11 +15550,11 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L193" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="194">
@@ -15599,7 +15575,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -15610,17 +15586,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15630,11 +15606,11 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L194" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="195">
@@ -15655,7 +15631,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -15666,17 +15642,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15686,7 +15662,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L195" t="n">
@@ -15711,7 +15687,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -15722,17 +15698,17 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -15742,11 +15718,11 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="197">
@@ -15767,7 +15743,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -15778,17 +15754,17 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -15798,11 +15774,11 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L197" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="198">
@@ -15823,7 +15799,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -15834,17 +15810,17 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -15854,7 +15830,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L198" t="n">
@@ -15879,7 +15855,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -15890,17 +15866,17 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -15910,7 +15886,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L199" t="n">
@@ -15935,7 +15911,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -15946,17 +15922,17 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15966,7 +15942,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L200" t="n">
@@ -15991,7 +15967,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -16002,17 +15978,17 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -16022,7 +15998,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L201" t="n">
@@ -16047,7 +16023,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
@@ -16058,17 +16034,17 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -16078,11 +16054,11 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L202" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="203">
@@ -16103,7 +16079,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
@@ -16114,17 +16090,17 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -16134,11 +16110,11 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L203" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="204">
@@ -16159,7 +16135,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16170,17 +16146,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16190,11 +16166,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>2</v>
+        <v>9</v>
       </c>
     </row>
     <row r="205">
@@ -16215,7 +16191,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16226,17 +16202,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16246,11 +16222,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
     </row>
     <row r="206">
@@ -16271,7 +16247,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16282,17 +16258,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16302,11 +16278,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="207">
@@ -16327,30 +16303,18 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
-      <c r="F207" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
-        </is>
-      </c>
-      <c r="G207" t="inlineStr">
-        <is>
-          <t>08-2026</t>
-        </is>
-      </c>
+      <c r="F207" t="inlineStr"/>
+      <c r="G207" t="inlineStr"/>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
-        </is>
-      </c>
-      <c r="I207" t="inlineStr">
-        <is>
-          <t>Agosto - 26</t>
-        </is>
-      </c>
+          <t>Sabores por PDV - ALTA</t>
+        </is>
+      </c>
+      <c r="I207" t="inlineStr"/>
       <c r="J207" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16358,11 +16322,11 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
         </is>
       </c>
       <c r="L207" t="n">
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -16383,7 +16347,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -16391,7 +16355,7 @@
       <c r="G208" t="inlineStr"/>
       <c r="H208" t="inlineStr">
         <is>
-          <t>Sabores por PDV - ALTA</t>
+          <t>Sabores por PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="I208" t="inlineStr"/>
@@ -16402,7 +16366,7 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
+          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
         </is>
       </c>
       <c r="L208" t="n">
@@ -16427,7 +16391,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16435,7 +16399,7 @@
       <c r="G209" t="inlineStr"/>
       <c r="H209" t="inlineStr">
         <is>
-          <t>Sabores por PDV - COUSTLAIN</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I209" t="inlineStr"/>
@@ -16446,11 +16410,11 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L209" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="210">
@@ -16471,7 +16435,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16479,7 +16443,7 @@
       <c r="G210" t="inlineStr"/>
       <c r="H210" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I210" t="inlineStr"/>
@@ -16490,11 +16454,11 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L210" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="211">
@@ -16515,7 +16479,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16523,7 +16487,7 @@
       <c r="G211" t="inlineStr"/>
       <c r="H211" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I211" t="inlineStr"/>
@@ -16534,11 +16498,11 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
         </is>
       </c>
       <c r="L211" t="n">
-        <v>2</v>
+        <v>50</v>
       </c>
     </row>
     <row r="212">
@@ -16559,7 +16523,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>CONTROL DE COSTOS</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16567,7 +16531,7 @@
       <c r="G212" t="inlineStr"/>
       <c r="H212" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>control de costos</t>
         </is>
       </c>
       <c r="I212" t="inlineStr"/>
@@ -16578,11 +16542,11 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
+          <t>648d45b0-2231-4e56-a018-4e83792a3115</t>
         </is>
       </c>
       <c r="L212" t="n">
-        <v>50</v>
+        <v>14</v>
       </c>
     </row>
     <row r="213">
@@ -16603,7 +16567,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>CONTROL DE COSTOS</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16611,7 +16575,7 @@
       <c r="G213" t="inlineStr"/>
       <c r="H213" t="inlineStr">
         <is>
-          <t>control de costos</t>
+          <t>stock por proveedores</t>
         </is>
       </c>
       <c r="I213" t="inlineStr"/>
@@ -16622,61 +16586,17 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>648d45b0-2231-4e56-a018-4e83792a3115</t>
+          <t>bdfe582a-c303-4732-b9b7-2390e04aa58e</t>
         </is>
       </c>
       <c r="L213" t="n">
-        <v>14</v>
-      </c>
-    </row>
-    <row r="214">
-      <c r="A214" s="2" t="inlineStr">
-        <is>
-          <t>SI</t>
-        </is>
-      </c>
-      <c r="B214" t="inlineStr">
-        <is>
-          <t>JEFES</t>
-        </is>
-      </c>
-      <c r="C214" t="inlineStr">
-        <is>
-          <t>HERGO - DISTRIBUCION</t>
-        </is>
-      </c>
-      <c r="D214" t="inlineStr">
-        <is>
-          <t>STOCK POR PROVEEDORES</t>
-        </is>
-      </c>
-      <c r="E214" t="inlineStr"/>
-      <c r="F214" t="inlineStr"/>
-      <c r="G214" t="inlineStr"/>
-      <c r="H214" t="inlineStr">
-        <is>
-          <t>stock por proveedores</t>
-        </is>
-      </c>
-      <c r="I214" t="inlineStr"/>
-      <c r="J214" t="inlineStr">
-        <is>
-          <t>Grupo Hergo - Jefes</t>
-        </is>
-      </c>
-      <c r="K214" t="inlineStr">
-        <is>
-          <t>bdfe582a-c303-4732-b9b7-2390e04aa58e</t>
-        </is>
-      </c>
-      <c r="L214" t="n">
         <v>58</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L214"/>
+  <autoFilter ref="A1:L213"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A214" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A213" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-29 07:44) - 123 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="30">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31">
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="32">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1717,12 +1717,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1737,7 +1737,7 @@
         </is>
       </c>
       <c r="H35" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="36">
@@ -1753,12 +1753,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="39">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="40">
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="82">
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="94">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="98">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="100">
@@ -4073,12 +4073,12 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COMPARATIVO 07-2026</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D100" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=31a2dc0d-9967-47eb-8ecf-4f61f0e5e3b8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E100" t="inlineStr"/>
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101">
@@ -4109,12 +4109,12 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D101" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E101" t="inlineStr"/>
@@ -4129,7 +4129,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="102">
@@ -4145,12 +4145,12 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>COMPARATIVO 07-2026</t>
         </is>
       </c>
       <c r="D102" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=31a2dc0d-9967-47eb-8ecf-4f61f0e5e3b8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E102" t="inlineStr"/>
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4345,7 +4345,7 @@
         </is>
       </c>
       <c r="H107" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="108">
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="109">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="110">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>1406</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="113">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>568</v>
+        <v>596</v>
       </c>
     </row>
     <row r="114">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>568</v>
+        <v>596</v>
       </c>
     </row>
     <row r="115">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="119">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="128">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="129">
@@ -5297,12 +5297,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ea6316b-51ca-4d99-80cb-c767aeaeb217&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ea6316b-51ca-4d99-80cb-c767aeaeb217&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5441,12 +5441,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -6108,7 +6108,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="4">
@@ -6196,7 +6196,7 @@
         </is>
       </c>
       <c r="L5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -6284,7 +6284,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
     </row>
     <row r="8">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
     <row r="9">
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="13">
@@ -6592,7 +6592,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="15">
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="17">
@@ -10780,7 +10780,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>17</v>
+        <v>20</v>
       </c>
     </row>
     <row r="97">
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="L111" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
     </row>
     <row r="112">
@@ -11508,7 +11508,7 @@
         </is>
       </c>
       <c r="L112" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="113">
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>24</v>
+        <v>29</v>
       </c>
     </row>
     <row r="115">
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="L115" t="n">
-        <v>30</v>
+        <v>33</v>
       </c>
     </row>
     <row r="116">
@@ -11684,7 +11684,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>86</v>
+        <v>87</v>
       </c>
     </row>
     <row r="117">
@@ -11772,7 +11772,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="119">
@@ -11816,7 +11816,7 @@
         </is>
       </c>
       <c r="L119" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="120">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>75</v>
+        <v>85</v>
       </c>
     </row>
     <row r="122">
@@ -11948,7 +11948,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="123">
@@ -11992,7 +11992,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="124">
@@ -12036,7 +12036,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>114</v>
+        <v>120</v>
       </c>
     </row>
     <row r="125">
@@ -12080,7 +12080,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="126">
@@ -12236,7 +12236,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="129">
@@ -12292,7 +12292,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="130">
@@ -12796,7 +12796,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>413</v>
+        <v>415</v>
       </c>
     </row>
     <row r="139">
@@ -12908,7 +12908,7 @@
         </is>
       </c>
       <c r="L140" t="n">
-        <v>208</v>
+        <v>236</v>
       </c>
     </row>
     <row r="141">
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="144">
@@ -13084,7 +13084,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>483</v>
+        <v>485</v>
       </c>
     </row>
     <row r="145">
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>280</v>
+        <v>283</v>
       </c>
     </row>
     <row r="147">
@@ -14088,7 +14088,7 @@
         </is>
       </c>
       <c r="L163" t="n">
-        <v>1406</v>
+        <v>1429</v>
       </c>
     </row>
     <row r="164">
@@ -14176,7 +14176,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>357</v>
+        <v>360</v>
       </c>
     </row>
     <row r="166">
@@ -14220,7 +14220,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>265</v>
+        <v>271</v>
       </c>
     </row>
     <row r="167">
@@ -14440,7 +14440,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
     </row>
     <row r="172">

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-30 07:44) - 123 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="31">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="39">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="40">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53">
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>147</v>
+        <v>156</v>
       </c>
     </row>
     <row r="87">
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="94">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="96">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="98">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>1429</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="113">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>596</v>
+        <v>606</v>
       </c>
     </row>
     <row r="114">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>596</v>
+        <v>606</v>
       </c>
     </row>
     <row r="115">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>485</v>
+        <v>477</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>283</v>
+        <v>275</v>
       </c>
     </row>
     <row r="118">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>58</v>
+        <v>59</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
     <row r="123">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="128">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>2</v>
+        <v>8</v>
       </c>
     </row>
     <row r="130">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="133">
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5297,12 +5297,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>49</v>
+        <v>50</v>
       </c>
     </row>
     <row r="9">
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="13">
@@ -6592,7 +6592,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>41</v>
+        <v>42</v>
       </c>
     </row>
     <row r="15">
@@ -7960,7 +7960,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="42">
@@ -10824,7 +10824,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="98">
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>147</v>
+        <v>156</v>
       </c>
     </row>
     <row r="103">
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>29</v>
+        <v>32</v>
       </c>
     </row>
     <row r="115">
@@ -11684,7 +11684,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>87</v>
+        <v>89</v>
       </c>
     </row>
     <row r="117">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="122">
@@ -12036,7 +12036,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>120</v>
+        <v>122</v>
       </c>
     </row>
     <row r="125">
@@ -12236,7 +12236,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="129">
@@ -12684,7 +12684,7 @@
         </is>
       </c>
       <c r="L136" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="137">
@@ -12740,7 +12740,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>70</v>
+        <v>60</v>
       </c>
     </row>
     <row r="138">
@@ -12908,7 +12908,7 @@
         </is>
       </c>
       <c r="L140" t="n">
-        <v>236</v>
+        <v>246</v>
       </c>
     </row>
     <row r="141">
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="144">
@@ -13084,7 +13084,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>485</v>
+        <v>477</v>
       </c>
     </row>
     <row r="145">
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>283</v>
+        <v>275</v>
       </c>
     </row>
     <row r="147">
@@ -14000,7 +14000,7 @@
         </is>
       </c>
       <c r="L161" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="162">
@@ -14088,7 +14088,7 @@
         </is>
       </c>
       <c r="L163" t="n">
-        <v>1429</v>
+        <v>1422</v>
       </c>
     </row>
     <row r="164">
@@ -14176,7 +14176,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>360</v>
+        <v>359</v>
       </c>
     </row>
     <row r="166">
@@ -14396,7 +14396,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>262</v>
+        <v>257</v>
       </c>
     </row>
     <row r="171">
@@ -14440,7 +14440,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="172">
@@ -15344,7 +15344,7 @@
         </is>
       </c>
       <c r="L188" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="189">
@@ -16616,7 +16616,7 @@
         </is>
       </c>
       <c r="L212" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-08-31 07:44) - 123 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="55">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>1422</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="113">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>477</v>
+        <v>472</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="118">
@@ -10824,7 +10824,7 @@
         </is>
       </c>
       <c r="L97" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98">
@@ -12684,7 +12684,7 @@
         </is>
       </c>
       <c r="L136" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="137">
@@ -12740,7 +12740,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>60</v>
+        <v>48</v>
       </c>
     </row>
     <row r="138">
@@ -13084,7 +13084,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>477</v>
+        <v>472</v>
       </c>
     </row>
     <row r="145">
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="147">
@@ -13832,7 +13832,7 @@
         </is>
       </c>
       <c r="L158" t="n">
-        <v>19</v>
+        <v>14</v>
       </c>
     </row>
     <row r="159">
@@ -14088,7 +14088,7 @@
         </is>
       </c>
       <c r="L163" t="n">
-        <v>1422</v>
+        <v>1418</v>
       </c>
     </row>
     <row r="164">
@@ -14176,7 +14176,7 @@
         </is>
       </c>
       <c r="L165" t="n">
-        <v>359</v>
+        <v>357</v>
       </c>
     </row>
     <row r="166">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-01 08:18) - 123 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="30">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="31">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="34">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="39">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="41">
@@ -1953,7 +1953,7 @@
         </is>
       </c>
       <c r="H41" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="42">
@@ -1969,12 +1969,12 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>STOCK VALORIZADO MC</t>
+          <t>EVOLUCION MENOR COSTE</t>
         </is>
       </c>
       <c r="D42" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E42" t="inlineStr"/>
@@ -1989,7 +1989,7 @@
         </is>
       </c>
       <c r="H42" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
     </row>
     <row r="43">
@@ -2005,12 +2005,12 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>EVOLUCION MENOR COSTE</t>
+          <t>STOCK VALORIZADO MC</t>
         </is>
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=a1d47f19-2c75-41f6-82e6-1bcf80289b8c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8c1c6f46-8451-443e-a14d-2927530fd512&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E43" t="inlineStr"/>
@@ -2025,7 +2025,7 @@
         </is>
       </c>
       <c r="H43" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="44">
@@ -2097,7 +2097,7 @@
         </is>
       </c>
       <c r="H45" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="46">
@@ -2365,12 +2365,12 @@
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>STOCK UNIFICADO</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D53" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E53" t="inlineStr"/>
@@ -2385,7 +2385,7 @@
         </is>
       </c>
       <c r="H53" t="n">
-        <v>13</v>
+        <v>21</v>
       </c>
     </row>
     <row r="54">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>STOCK UNIFICADO</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=589dc885-5ca9-4b06-9776-ebb80e7ea81d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>8</v>
+        <v>13</v>
       </c>
     </row>
     <row r="55">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
     </row>
     <row r="57">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="58">
@@ -3397,7 +3397,7 @@
         </is>
       </c>
       <c r="H81" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="82">
@@ -3589,7 +3589,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="87">
@@ -3841,7 +3841,7 @@
         </is>
       </c>
       <c r="H93" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="94">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="98">
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=09e9193a-f463-498d-9e90-493d77f30de4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4237,7 +4237,7 @@
         </is>
       </c>
       <c r="H104" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="105">
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=293fe003-6ee2-4215-8c40-a47893f8447c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d1c92403-15f2-4bf6-b077-dc5cb6f7b490&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=09e9193a-f463-498d-9e90-493d77f30de4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=293fe003-6ee2-4215-8c40-a47893f8447c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4381,7 +4381,7 @@
         </is>
       </c>
       <c r="H108" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="109">
@@ -4417,7 +4417,7 @@
         </is>
       </c>
       <c r="H109" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="110">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>1418</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="113">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>606</v>
+        <v>622</v>
       </c>
     </row>
     <row r="114">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>606</v>
+        <v>622</v>
       </c>
     </row>
     <row r="115">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>472</v>
+        <v>480</v>
       </c>
     </row>
     <row r="116">
@@ -4685,12 +4685,12 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>INCENTIVOS COUSTLAIN</t>
         </is>
       </c>
       <c r="D117" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f62bbf09-eca6-4bb8-8caa-e88da0c3184d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E117" t="inlineStr"/>
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>271</v>
+        <v>285</v>
       </c>
     </row>
     <row r="118">
@@ -4721,12 +4721,12 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D118" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f62bbf09-eca6-4bb8-8caa-e88da0c3184d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E118" t="inlineStr"/>
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="119">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
     <row r="123">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="124">
@@ -4973,12 +4973,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="126">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
     </row>
     <row r="128">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="129">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="130">
@@ -6152,7 +6152,7 @@
         </is>
       </c>
       <c r="L4" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -6284,7 +6284,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="8">
@@ -6328,7 +6328,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="9">
@@ -6416,7 +6416,7 @@
         </is>
       </c>
       <c r="L10" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="11">
@@ -6504,7 +6504,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="13">
@@ -6592,7 +6592,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>42</v>
+        <v>44</v>
       </c>
     </row>
     <row r="15">
@@ -6636,7 +6636,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
     </row>
     <row r="16">
@@ -6680,7 +6680,7 @@
         </is>
       </c>
       <c r="L16" t="n">
-        <v>43</v>
+        <v>44</v>
       </c>
     </row>
     <row r="17">
@@ -6768,7 +6768,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>2</v>
+        <v>21</v>
       </c>
     </row>
     <row r="19">
@@ -10552,7 +10552,7 @@
         </is>
       </c>
       <c r="L91" t="n">
-        <v>55</v>
+        <v>56</v>
       </c>
     </row>
     <row r="92">
@@ -10780,7 +10780,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>20</v>
+        <v>25</v>
       </c>
     </row>
     <row r="97">
@@ -11044,7 +11044,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>156</v>
+        <v>163</v>
       </c>
     </row>
     <row r="103">
@@ -11420,7 +11420,7 @@
         </is>
       </c>
       <c r="L110" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="111">
@@ -11464,7 +11464,7 @@
         </is>
       </c>
       <c r="L111" t="n">
-        <v>46</v>
+        <v>47</v>
       </c>
     </row>
     <row r="112">
@@ -11596,7 +11596,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>32</v>
+        <v>36</v>
       </c>
     </row>
     <row r="115">
@@ -11640,7 +11640,7 @@
         </is>
       </c>
       <c r="L115" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
     </row>
     <row r="116">
@@ -11684,7 +11684,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>89</v>
+        <v>98</v>
       </c>
     </row>
     <row r="117">
@@ -11904,7 +11904,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>86</v>
+        <v>92</v>
       </c>
     </row>
     <row r="122">
@@ -11948,7 +11948,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
     </row>
     <row r="123">
@@ -12036,7 +12036,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>122</v>
+        <v>127</v>
       </c>
     </row>
     <row r="125">
@@ -12080,7 +12080,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>8</v>
+        <v>14</v>
       </c>
     </row>
     <row r="126">
@@ -12236,7 +12236,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>67</v>
+        <v>69</v>
       </c>
     </row>
     <row r="129">
@@ -12684,7 +12684,7 @@
         </is>
       </c>
       <c r="L136" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="137">
@@ -12740,7 +12740,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>48</v>
+        <v>38</v>
       </c>
     </row>
     <row r="138">
@@ -12796,7 +12796,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>415</v>
+        <v>400</v>
       </c>
     </row>
     <row r="139">
@@ -12908,7 +12908,7 @@
         </is>
       </c>
       <c r="L140" t="n">
-        <v>246</v>
+        <v>262</v>
       </c>
     </row>
     <row r="141">
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="144">
@@ -13084,7 +13084,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>472</v>
+        <v>480</v>
       </c>
     </row>
     <row r="145">
@@ -13172,7 +13172,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>271</v>
+        <v>270</v>
       </c>
     </row>
     <row r="147">
@@ -14000,7 +14000,7 @@
         </is>
       </c>
       <c r="L161" t="n">
-        <v>18</v>
+        <v>21</v>
       </c>
     </row>
     <row r="162">
@@ -14088,7 +14088,7 @@
         </is>
       </c>
       <c r="L163" t="n">
-        <v>1418</v>
+        <v>1432</v>
       </c>
     </row>
     <row r="164">
@@ -14220,7 +14220,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>271</v>
+        <v>285</v>
       </c>
     </row>
     <row r="167">
@@ -14440,7 +14440,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
     </row>
     <row r="172">
@@ -16572,7 +16572,7 @@
         </is>
       </c>
       <c r="L211" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
     </row>
     <row r="212">
@@ -16616,7 +16616,7 @@
         </is>
       </c>
       <c r="L212" t="n">
-        <v>56</v>
+        <v>53</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-02 07:40) - 124 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="31">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="34">
@@ -1845,7 +1845,7 @@
         </is>
       </c>
       <c r="H38" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="39">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="40">
@@ -2205,7 +2205,7 @@
         </is>
       </c>
       <c r="H48" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="49">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>28</v>
+        <v>29</v>
       </c>
     </row>
     <row r="50">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="53">
@@ -3661,7 +3661,7 @@
         </is>
       </c>
       <c r="H88" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="89">
@@ -3805,7 +3805,7 @@
         </is>
       </c>
       <c r="H92" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="93">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="96">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="97">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="99">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>1432</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="114">
@@ -4597,7 +4597,7 @@
         </is>
       </c>
       <c r="H114" t="n">
-        <v>622</v>
+        <v>643</v>
       </c>
     </row>
     <row r="115">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>622</v>
+        <v>643</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>480</v>
+        <v>498</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>357</v>
+        <v>372</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>285</v>
+        <v>277</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>62</v>
+        <v>63</v>
       </c>
     </row>
     <row r="123">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
     </row>
     <row r="128">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d94b898b-ca9a-4f65-bd76-5a049696c931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="130">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="131">
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="132">
@@ -5297,12 +5297,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5513,12 +5513,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5585,12 +5585,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5621,12 +5621,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5657,12 +5657,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5729,12 +5729,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5801,12 +5801,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -5837,12 +5837,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -6320,7 +6320,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>13</v>
+        <v>18</v>
       </c>
     </row>
     <row r="8">
@@ -6364,7 +6364,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>53</v>
+        <v>56</v>
       </c>
     </row>
     <row r="9">
@@ -6540,7 +6540,7 @@
         </is>
       </c>
       <c r="L12" t="n">
-        <v>31</v>
+        <v>33</v>
       </c>
     </row>
     <row r="13">
@@ -6628,7 +6628,7 @@
         </is>
       </c>
       <c r="L14" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="15">
@@ -7732,7 +7732,7 @@
         </is>
       </c>
       <c r="L35" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="36">
@@ -7996,7 +7996,7 @@
         </is>
       </c>
       <c r="L41" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="42">
@@ -8812,7 +8812,7 @@
         </is>
       </c>
       <c r="L56" t="n">
-        <v>21</v>
+        <v>11</v>
       </c>
     </row>
     <row r="57">
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="L99" t="n">
-        <v>90</v>
+        <v>92</v>
       </c>
     </row>
     <row r="100">
@@ -11124,7 +11124,7 @@
         </is>
       </c>
       <c r="L103" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="104">
@@ -11632,7 +11632,7 @@
         </is>
       </c>
       <c r="L114" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
     </row>
     <row r="115">
@@ -11720,7 +11720,7 @@
         </is>
       </c>
       <c r="L116" t="n">
-        <v>98</v>
+        <v>105</v>
       </c>
     </row>
     <row r="117">
@@ -11984,7 +11984,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>92</v>
+        <v>94</v>
       </c>
     </row>
     <row r="123">
@@ -12116,7 +12116,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>127</v>
+        <v>128</v>
       </c>
     </row>
     <row r="126">
@@ -12204,7 +12204,7 @@
         </is>
       </c>
       <c r="L127" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="128">
@@ -12372,7 +12372,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
     </row>
     <row r="131">
@@ -12764,7 +12764,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="138">
@@ -12820,7 +12820,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>38</v>
+        <v>22</v>
       </c>
     </row>
     <row r="139">
@@ -12876,7 +12876,7 @@
         </is>
       </c>
       <c r="L139" t="n">
-        <v>400</v>
+        <v>389</v>
       </c>
     </row>
     <row r="140">
@@ -12988,7 +12988,7 @@
         </is>
       </c>
       <c r="L141" t="n">
-        <v>262</v>
+        <v>283</v>
       </c>
     </row>
     <row r="142">
@@ -13032,7 +13032,7 @@
         </is>
       </c>
       <c r="L142" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="143">
@@ -13120,7 +13120,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="145">
@@ -13164,7 +13164,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>480</v>
+        <v>498</v>
       </c>
     </row>
     <row r="146">
@@ -13252,7 +13252,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>270</v>
+        <v>272</v>
       </c>
     </row>
     <row r="148">
@@ -13912,7 +13912,7 @@
         </is>
       </c>
       <c r="L159" t="n">
-        <v>14</v>
+        <v>12</v>
       </c>
     </row>
     <row r="160">
@@ -14080,7 +14080,7 @@
         </is>
       </c>
       <c r="L162" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="163">
@@ -14168,7 +14168,7 @@
         </is>
       </c>
       <c r="L164" t="n">
-        <v>1432</v>
+        <v>1476</v>
       </c>
     </row>
     <row r="165">
@@ -14256,7 +14256,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>357</v>
+        <v>372</v>
       </c>
     </row>
     <row r="167">
@@ -14300,7 +14300,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>285</v>
+        <v>277</v>
       </c>
     </row>
     <row r="168">
@@ -14476,7 +14476,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>257</v>
+        <v>261</v>
       </c>
     </row>
     <row r="172">
@@ -14520,7 +14520,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="173">
@@ -14820,7 +14820,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="179">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-06 07:43) - 127 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="30">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="31">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="41">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="47">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2581,12 +2581,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="H59" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="60">
@@ -2617,12 +2617,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2637,7 +2637,7 @@
         </is>
       </c>
       <c r="H60" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="61">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="99">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="100">
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="112">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="113">
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>1487</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>500</v>
+        <v>514</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>299</v>
+        <v>320</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>299</v>
+        <v>320</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="123">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="125">
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="127">
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="128">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>CONSUMOS POR CLIENTE</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>16</v>
+        <v>22</v>
       </c>
     </row>
     <row r="130">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>CONSUMOS POR CLIENTE</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e6b113ec-729a-4d3c-934c-f54c1f9689d9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
     </row>
     <row r="131">
@@ -5189,12 +5189,12 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D131" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E131" t="inlineStr"/>
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>7</v>
+        <v>13</v>
       </c>
     </row>
     <row r="132">
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="134">
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="135">
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="136">
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="138">
@@ -6516,7 +6516,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>64</v>
+        <v>68</v>
       </c>
     </row>
     <row r="10">
@@ -6692,7 +6692,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
@@ -6780,7 +6780,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>50</v>
+        <v>51</v>
       </c>
     </row>
     <row r="16">
@@ -6868,7 +6868,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
     </row>
     <row r="18">
@@ -7716,7 +7716,7 @@
         </is>
       </c>
       <c r="L33" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
     </row>
     <row r="34">
@@ -7772,7 +7772,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
     </row>
     <row r="35">
@@ -9020,7 +9020,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="59">
@@ -9496,7 +9496,7 @@
         </is>
       </c>
       <c r="L68" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="69">
@@ -10948,7 +10948,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
     </row>
     <row r="97">
@@ -11912,7 +11912,7 @@
         </is>
       </c>
       <c r="L117" t="n">
-        <v>52</v>
+        <v>53</v>
       </c>
     </row>
     <row r="118">
@@ -12088,7 +12088,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>42</v>
+        <v>43</v>
       </c>
     </row>
     <row r="122">
@@ -12132,7 +12132,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>45</v>
+        <v>48</v>
       </c>
     </row>
     <row r="123">
@@ -12396,7 +12396,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>99</v>
+        <v>102</v>
       </c>
     </row>
     <row r="129">
@@ -12440,7 +12440,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="130">
@@ -13176,7 +13176,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>43</v>
+        <v>41</v>
       </c>
     </row>
     <row r="144">
@@ -13288,7 +13288,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>376</v>
+        <v>359</v>
       </c>
     </row>
     <row r="146">
@@ -13400,7 +13400,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>292</v>
+        <v>302</v>
       </c>
     </row>
     <row r="148">
@@ -13456,7 +13456,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>7</v>
+        <v>18</v>
       </c>
     </row>
     <row r="149">
@@ -13544,7 +13544,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
     </row>
     <row r="151">
@@ -13632,7 +13632,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>500</v>
+        <v>514</v>
       </c>
     </row>
     <row r="153">
@@ -13720,7 +13720,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>272</v>
+        <v>274</v>
       </c>
     </row>
     <row r="155">
@@ -14436,7 +14436,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>41</v>
+        <v>39</v>
       </c>
     </row>
     <row r="168">
@@ -14548,7 +14548,7 @@
         </is>
       </c>
       <c r="L169" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
     </row>
     <row r="170">
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>1487</v>
+        <v>1468</v>
       </c>
     </row>
     <row r="173">
@@ -14780,7 +14780,7 @@
         </is>
       </c>
       <c r="L174" t="n">
-        <v>386</v>
+        <v>389</v>
       </c>
     </row>
     <row r="175">
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>279</v>
+        <v>275</v>
       </c>
     </row>
     <row r="176">
@@ -14912,7 +14912,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>1</v>
+        <v>22</v>
       </c>
     </row>
     <row r="178">
@@ -15044,7 +15044,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>268</v>
+        <v>266</v>
       </c>
     </row>
     <row r="181">
@@ -17272,7 +17272,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>48</v>
+        <v>46</v>
       </c>
     </row>
     <row r="223">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-07 07:37) - 127 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -4633,7 +4633,7 @@
         </is>
       </c>
       <c r="H115" t="n">
-        <v>1468</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="116">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>514</v>
+        <v>503</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>389</v>
+        <v>365</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>320</v>
+        <v>324</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>266</v>
+        <v>255</v>
       </c>
     </row>
     <row r="123">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="125">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="127">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="129">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
     </row>
     <row r="133">
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="134">
@@ -5297,12 +5297,12 @@
       </c>
       <c r="C134" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D134" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E134" t="inlineStr"/>
@@ -5317,7 +5317,7 @@
         </is>
       </c>
       <c r="H134" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
     </row>
     <row r="135">
@@ -9020,7 +9020,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="59">
@@ -13176,7 +13176,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>41</v>
+        <v>40</v>
       </c>
     </row>
     <row r="144">
@@ -13232,7 +13232,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>17</v>
+        <v>3</v>
       </c>
     </row>
     <row r="145">
@@ -13288,7 +13288,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>359</v>
+        <v>330</v>
       </c>
     </row>
     <row r="146">
@@ -13400,7 +13400,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>302</v>
+        <v>306</v>
       </c>
     </row>
     <row r="148">
@@ -13544,7 +13544,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>6</v>
+        <v>12</v>
       </c>
     </row>
     <row r="151">
@@ -13632,7 +13632,7 @@
         </is>
       </c>
       <c r="L152" t="n">
-        <v>514</v>
+        <v>503</v>
       </c>
     </row>
     <row r="153">
@@ -13720,7 +13720,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>274</v>
+        <v>270</v>
       </c>
     </row>
     <row r="155">
@@ -14380,7 +14380,7 @@
         </is>
       </c>
       <c r="L166" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
     </row>
     <row r="167">
@@ -14436,7 +14436,7 @@
         </is>
       </c>
       <c r="L167" t="n">
-        <v>39</v>
+        <v>36</v>
       </c>
     </row>
     <row r="168">
@@ -14692,7 +14692,7 @@
         </is>
       </c>
       <c r="L172" t="n">
-        <v>1468</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="173">
@@ -14780,7 +14780,7 @@
         </is>
       </c>
       <c r="L174" t="n">
-        <v>389</v>
+        <v>365</v>
       </c>
     </row>
     <row r="175">
@@ -14824,7 +14824,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>275</v>
+        <v>271</v>
       </c>
     </row>
     <row r="176">
@@ -14912,7 +14912,7 @@
         </is>
       </c>
       <c r="L177" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="178">
@@ -15044,7 +15044,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>266</v>
+        <v>255</v>
       </c>
     </row>
     <row r="181">
@@ -17000,7 +17000,7 @@
         </is>
       </c>
       <c r="L216" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="217">
@@ -17272,7 +17272,7 @@
         </is>
       </c>
       <c r="L222" t="n">
-        <v>46</v>
+        <v>44</v>
       </c>
     </row>
     <row r="223">

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-08 07:43) - 128 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -12,7 +12,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$156</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$224</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$225</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="30">
@@ -1557,7 +1557,7 @@
         </is>
       </c>
       <c r="H30" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="31">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="33">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="41">
@@ -2241,7 +2241,7 @@
         </is>
       </c>
       <c r="H49" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="50">
@@ -2401,12 +2401,12 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D54" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E54" t="inlineStr"/>
@@ -2421,7 +2421,7 @@
         </is>
       </c>
       <c r="H54" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="55">
@@ -2437,12 +2437,12 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D55" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=db3b1962-96b8-49b8-ab8b-c7c13fd197df&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E55" t="inlineStr"/>
@@ -2457,7 +2457,7 @@
         </is>
       </c>
       <c r="H55" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="56">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8e7f08c1-fd17-4367-85f0-9af0618ec50f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="57">
@@ -2545,12 +2545,12 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>BRANCA</t>
         </is>
       </c>
       <c r="D58" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E58" t="inlineStr"/>
@@ -2565,7 +2565,7 @@
         </is>
       </c>
       <c r="H58" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="59">
@@ -2581,12 +2581,12 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>BRANCA</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D59" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=363d9b37-f245-4192-9224-0b00b4fd1ea5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3d9a0917-34b5-4ac6-8b6a-f2244892db15&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E59" t="inlineStr"/>
@@ -2617,12 +2617,12 @@
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>MARGENES MAYORISTA</t>
         </is>
       </c>
       <c r="D60" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E60" t="inlineStr"/>
@@ -2653,12 +2653,12 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>MARGENES MAYORISTA</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D61" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3bc172f4-88c0-403c-9c60-483089c17d75&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E61" t="inlineStr"/>
@@ -2673,7 +2673,7 @@
         </is>
       </c>
       <c r="H61" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="62">
@@ -2689,12 +2689,12 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D62" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=b427136c-6785-4e5f-8e88-026b03a2bbe1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E62" t="inlineStr"/>
@@ -2725,12 +2725,12 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>CONSUMOS DE CLIENTES</t>
         </is>
       </c>
       <c r="D63" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=45ca0371-6f94-430e-be96-2ec8fc691b21&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E63" t="inlineStr"/>
@@ -2761,12 +2761,12 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CONSUMOS DE CLIENTES</t>
+          <t>EFECTIVIDADES</t>
         </is>
       </c>
       <c r="D64" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27dfaf71-9641-46a8-a9d2-21a7299ca705&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ba02793b-9173-406b-b100-198d9dbaae73&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E64" t="inlineStr"/>
@@ -2797,12 +2797,12 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D65" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ba02793b-9173-406b-b100-198d9dbaae73&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E65" t="inlineStr"/>
@@ -2833,12 +2833,12 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>FINAL FOUR</t>
         </is>
       </c>
       <c r="D66" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=899444c9-cd01-4bcf-b726-d4ae8d7fa432&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E66" t="inlineStr"/>
@@ -2869,12 +2869,12 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>FINAL FOUR</t>
+          <t>INCENTIVOS ALTA</t>
         </is>
       </c>
       <c r="D67" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=883ebe8e-09ee-4631-b55b-337f9560d8ac&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=66f1d933-90ed-49d1-89e5-dbb9e765b851&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E67" t="inlineStr"/>
@@ -2905,12 +2905,12 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D68" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=66f1d933-90ed-49d1-89e5-dbb9e765b851&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=cf82ea28-f534-4da8-9786-e89dba954b17&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E68" t="inlineStr"/>
@@ -2941,12 +2941,12 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>INCENTIVOS BLACK</t>
         </is>
       </c>
       <c r="D69" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=cf82ea28-f534-4da8-9786-e89dba954b17&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=fee017c6-a239-4e81-987a-fede32524903&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E69" t="inlineStr"/>
@@ -2977,12 +2977,12 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>INCENTIVOS BLACK</t>
+          <t>INCENTIVOS COUSTLAIN</t>
         </is>
       </c>
       <c r="D70" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=fee017c6-a239-4e81-987a-fede32524903&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9e51941e-8703-4d9c-814e-c80d8be9fde2&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E70" t="inlineStr"/>
@@ -3013,12 +3013,12 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D71" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9e51941e-8703-4d9c-814e-c80d8be9fde2&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E71" t="inlineStr"/>
@@ -3049,12 +3049,12 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D72" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8a7194e4-c02a-4fb6-a108-b214302c8a96&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E72" t="inlineStr"/>
@@ -3085,12 +3085,12 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D73" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=34982d0f-52be-4a8b-935f-9aa3ee3915bb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=220bac31-1b58-44ff-8b44-2e0dffd8fc5a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E73" t="inlineStr"/>
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="99">
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="101">
@@ -4129,7 +4129,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="102">
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="112">
@@ -4525,7 +4525,7 @@
         </is>
       </c>
       <c r="H112" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="113">
@@ -4561,7 +4561,7 @@
         </is>
       </c>
       <c r="H113" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="114">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>1456</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>503</v>
+        <v>507</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>324</v>
+        <v>337</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>324</v>
+        <v>337</v>
       </c>
     </row>
     <row r="121">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="124">
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>44</v>
+        <v>43</v>
       </c>
     </row>
     <row r="126">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>FRATELLI REPRESENTADAS 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>31</v>
+        <v>40</v>
       </c>
     </row>
     <row r="127">
@@ -5045,12 +5045,12 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>FRATELLI REPRESENTADAS 2026</t>
         </is>
       </c>
       <c r="D127" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=aacc1cbf-8839-4b44-933e-085a3fe7eb66&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E127" t="inlineStr"/>
@@ -5065,7 +5065,7 @@
         </is>
       </c>
       <c r="H127" t="n">
-        <v>29</v>
+        <v>31</v>
       </c>
     </row>
     <row r="128">
@@ -5081,12 +5081,12 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D128" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E128" t="inlineStr"/>
@@ -5101,7 +5101,7 @@
         </is>
       </c>
       <c r="H128" t="n">
-        <v>25</v>
+        <v>29</v>
       </c>
     </row>
     <row r="129">
@@ -5117,12 +5117,12 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="D129" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8534dc2b-7ee4-484d-b3e3-d151ed93adaf&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E129" t="inlineStr"/>
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="130">
@@ -5153,12 +5153,12 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="D130" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=5d2131f2-f6b5-41f6-b864-e0534c499950&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c1ba4bda-9414-4968-b1f0-98ceb9b4e37b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E130" t="inlineStr"/>
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>22</v>
+        <v>26</v>
       </c>
     </row>
     <row r="131">
@@ -5225,12 +5225,12 @@
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D132" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E132" t="inlineStr"/>
@@ -5261,12 +5261,12 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="D133" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7de99d39-41a8-4578-994d-377c9a1c334e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7bcd2a2e-06f8-496e-9a39-a3b30deba2ae&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E133" t="inlineStr"/>
@@ -5281,7 +5281,7 @@
         </is>
       </c>
       <c r="H133" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="134">
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5441,12 +5441,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="139">
@@ -5477,12 +5477,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5513,12 +5513,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5549,12 +5549,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ea6316b-51ca-4d99-80cb-c767aeaeb217&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5585,12 +5585,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5621,12 +5621,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5641,7 +5641,7 @@
         </is>
       </c>
       <c r="H143" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -5657,12 +5657,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5729,12 +5729,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5801,12 +5801,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -6124,7 +6124,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L224"/>
+  <dimension ref="A1:L225"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>23</v>
+        <v>26</v>
       </c>
     </row>
     <row r="9">
@@ -6552,7 +6552,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>68</v>
+        <v>71</v>
       </c>
     </row>
     <row r="10">
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>46</v>
+        <v>48</v>
       </c>
     </row>
     <row r="14">
@@ -6816,7 +6816,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
     </row>
     <row r="16">
@@ -6904,7 +6904,7 @@
         </is>
       </c>
       <c r="L17" t="n">
-        <v>45</v>
+        <v>46</v>
       </c>
     </row>
     <row r="18">
@@ -7808,7 +7808,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
     </row>
     <row r="35">
@@ -8240,7 +8240,7 @@
         </is>
       </c>
       <c r="L43" t="n">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="44">
@@ -9000,7 +9000,7 @@
         </is>
       </c>
       <c r="L57" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="58">
@@ -9056,7 +9056,7 @@
         </is>
       </c>
       <c r="L58" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59">
@@ -9224,7 +9224,7 @@
         </is>
       </c>
       <c r="L61" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
     </row>
     <row r="62">
@@ -9532,7 +9532,7 @@
         </is>
       </c>
       <c r="L68" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="69">
@@ -11164,7 +11164,7 @@
         </is>
       </c>
       <c r="L100" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
     </row>
     <row r="101">
@@ -12124,7 +12124,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
     </row>
     <row r="122">
@@ -12168,7 +12168,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>43</v>
+        <v>50</v>
       </c>
     </row>
     <row r="123">
@@ -12212,7 +12212,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>48</v>
+        <v>49</v>
       </c>
     </row>
     <row r="124">
@@ -12256,7 +12256,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>112</v>
+        <v>118</v>
       </c>
     </row>
     <row r="125">
@@ -12476,7 +12476,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>102</v>
+        <v>106</v>
       </c>
     </row>
     <row r="130">
@@ -12520,7 +12520,7 @@
         </is>
       </c>
       <c r="L130" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="131">
@@ -12564,7 +12564,7 @@
         </is>
       </c>
       <c r="L131" t="n">
-        <v>50</v>
+        <v>56</v>
       </c>
     </row>
     <row r="132">
@@ -12652,7 +12652,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>22</v>
+        <v>29</v>
       </c>
     </row>
     <row r="134">
@@ -12864,7 +12864,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
     </row>
     <row r="138">
@@ -13200,7 +13200,7 @@
         </is>
       </c>
       <c r="L143" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="144">
@@ -13256,7 +13256,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>40</v>
+        <v>35</v>
       </c>
     </row>
     <row r="145">
@@ -13312,7 +13312,7 @@
         </is>
       </c>
       <c r="L145" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
     </row>
     <row r="146">
@@ -13368,7 +13368,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="147">
@@ -13480,7 +13480,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>306</v>
+        <v>312</v>
       </c>
     </row>
     <row r="149">
@@ -13536,7 +13536,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>18</v>
+        <v>25</v>
       </c>
     </row>
     <row r="150">
@@ -13624,7 +13624,7 @@
         </is>
       </c>
       <c r="L151" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
     </row>
     <row r="152">
@@ -13712,7 +13712,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>503</v>
+        <v>507</v>
       </c>
     </row>
     <row r="154">
@@ -14628,7 +14628,7 @@
         </is>
       </c>
       <c r="L170" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
     </row>
     <row r="171">
@@ -14772,7 +14772,7 @@
         </is>
       </c>
       <c r="L173" t="n">
-        <v>1456</v>
+        <v>1446</v>
       </c>
     </row>
     <row r="174">
@@ -14860,7 +14860,7 @@
         </is>
       </c>
       <c r="L175" t="n">
-        <v>365</v>
+        <v>362</v>
       </c>
     </row>
     <row r="176">
@@ -14992,7 +14992,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>29</v>
+        <v>40</v>
       </c>
     </row>
     <row r="179">
@@ -15080,7 +15080,7 @@
         </is>
       </c>
       <c r="L180" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="181">
@@ -15124,7 +15124,7 @@
         </is>
       </c>
       <c r="L181" t="n">
-        <v>255</v>
+        <v>251</v>
       </c>
     </row>
     <row r="182">
@@ -16317,30 +16317,26 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
       <c r="F204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
+          <t>SEGUIMIENTO DE MARCAS</t>
         </is>
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
-        </is>
-      </c>
-      <c r="I204" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I204" t="inlineStr"/>
       <c r="J204" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -16348,11 +16344,11 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
         </is>
       </c>
       <c r="L204" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="205">
@@ -16373,7 +16369,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16384,17 +16380,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16404,11 +16400,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="206">
@@ -16429,7 +16425,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16440,17 +16436,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16460,7 +16456,7 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L206" t="n">
@@ -16485,7 +16481,7 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
@@ -16496,17 +16492,17 @@
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16516,11 +16512,11 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L207" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -16541,7 +16537,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -16552,17 +16548,17 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -16572,11 +16568,11 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L208" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="209">
@@ -16597,7 +16593,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16608,17 +16604,17 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -16628,7 +16624,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L209" t="n">
@@ -16653,7 +16649,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16664,17 +16660,17 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -16684,7 +16680,7 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L210" t="n">
@@ -16709,7 +16705,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16720,17 +16716,17 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -16740,7 +16736,7 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L211" t="n">
@@ -16765,7 +16761,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16776,17 +16772,17 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -16796,7 +16792,7 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L212" t="n">
@@ -16821,7 +16817,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16832,17 +16828,17 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -16852,11 +16848,11 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L213" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="214">
@@ -16877,7 +16873,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E214" t="inlineStr"/>
@@ -16888,17 +16884,17 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -16908,11 +16904,11 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L214" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="215">
@@ -16933,7 +16929,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -16944,17 +16940,17 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -16964,11 +16960,11 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L215" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="216">
@@ -16989,7 +16985,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -17000,17 +16996,17 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -17020,11 +17016,11 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L216" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="217">
@@ -17045,7 +17041,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -17056,17 +17052,17 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -17076,11 +17072,11 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L217" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="218">
@@ -17101,7 +17097,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -17112,15 +17108,19 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
-        </is>
-      </c>
-      <c r="I218" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+        </is>
+      </c>
+      <c r="I218" t="inlineStr">
+        <is>
+          <t>Agosto - 26</t>
+        </is>
+      </c>
       <c r="J218" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -17128,11 +17128,11 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L218" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="219">
@@ -17153,15 +17153,23 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
-      <c r="F219" t="inlineStr"/>
-      <c r="G219" t="inlineStr"/>
+      <c r="F219" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
+        </is>
+      </c>
+      <c r="G219" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>Sabores por PDV - ALTA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
       <c r="I219" t="inlineStr"/>
@@ -17172,7 +17180,7 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L219" t="n">
@@ -17197,7 +17205,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -17205,7 +17213,7 @@
       <c r="G220" t="inlineStr"/>
       <c r="H220" t="inlineStr">
         <is>
-          <t>Sabores por PDV - COUSTLAIN</t>
+          <t>Sabores por PDV - ALTA</t>
         </is>
       </c>
       <c r="I220" t="inlineStr"/>
@@ -17216,7 +17224,7 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
+          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
         </is>
       </c>
       <c r="L220" t="n">
@@ -17241,7 +17249,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -17249,7 +17257,7 @@
       <c r="G221" t="inlineStr"/>
       <c r="H221" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>Sabores por PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="I221" t="inlineStr"/>
@@ -17260,11 +17268,11 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
         </is>
       </c>
       <c r="L221" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="222">
@@ -17285,7 +17293,7 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
@@ -17293,7 +17301,7 @@
       <c r="G222" t="inlineStr"/>
       <c r="H222" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I222" t="inlineStr"/>
@@ -17304,11 +17312,11 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L222" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="223">
@@ -17329,7 +17337,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -17337,7 +17345,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -17348,11 +17356,11 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L223" t="n">
-        <v>44</v>
+        <v>2</v>
       </c>
     </row>
     <row r="224">
@@ -17373,7 +17381,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
@@ -17381,7 +17389,7 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
-          <t>stock por proveedores</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -17392,17 +17400,61 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
+        </is>
+      </c>
+      <c r="L224" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="225">
+      <c r="A225" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B225" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C225" t="inlineStr">
+        <is>
+          <t>HERGO - DISTRIBUCION</t>
+        </is>
+      </c>
+      <c r="D225" t="inlineStr">
+        <is>
+          <t>STOCK POR PROVEEDORES</t>
+        </is>
+      </c>
+      <c r="E225" t="inlineStr"/>
+      <c r="F225" t="inlineStr"/>
+      <c r="G225" t="inlineStr"/>
+      <c r="H225" t="inlineStr">
+        <is>
+          <t>stock por proveedores</t>
+        </is>
+      </c>
+      <c r="I225" t="inlineStr"/>
+      <c r="J225" t="inlineStr">
+        <is>
+          <t>Grupo Hergo - Jefes</t>
+        </is>
+      </c>
+      <c r="K225" t="inlineStr">
+        <is>
           <t>bdfe582a-c303-4732-b9b7-2390e04aa58e</t>
         </is>
       </c>
-      <c r="L224" t="n">
+      <c r="L225" t="n">
         <v>53</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L224"/>
+  <autoFilter ref="A1:L225"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A224" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A225" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-09 08:57) - 128 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="30">
@@ -1573,12 +1573,12 @@
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>MARGENES</t>
         </is>
       </c>
       <c r="D31" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E31" t="inlineStr"/>
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="32">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>MARGENES</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D32" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e4b97365-464a-4d0f-812e-fc26afeaf650&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c6276b41-9847-4111-82e8-146d32636229&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E32" t="inlineStr"/>
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="34">
@@ -1717,12 +1717,12 @@
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>COMPORTAMIENTO CLIENTES</t>
         </is>
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E35" t="inlineStr"/>
@@ -1753,12 +1753,12 @@
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>COMPORTAMIENTO CLIENTES</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e3a781e9-fe9b-4885-9e7d-8de8c003cfdd&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0411b9ac-d5bf-4e97-9b38-5d2fe2deb931&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E36" t="inlineStr"/>
@@ -1773,7 +1773,7 @@
         </is>
       </c>
       <c r="H36" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="37">
@@ -1789,12 +1789,12 @@
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E37" t="inlineStr"/>
@@ -1809,7 +1809,7 @@
         </is>
       </c>
       <c r="H37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -1825,12 +1825,12 @@
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0396d9e8-9644-4db9-867b-89d090fb95a3&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=277cb203-8263-4fb5-b0c7-0a309ac24ee5&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E38" t="inlineStr"/>
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="40">
@@ -2133,7 +2133,7 @@
         </is>
       </c>
       <c r="H46" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="47">
@@ -2313,7 +2313,7 @@
         </is>
       </c>
       <c r="H51" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="52">
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="53">
@@ -2473,12 +2473,12 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
         </is>
       </c>
       <c r="D56" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E56" t="inlineStr"/>
@@ -2493,7 +2493,7 @@
         </is>
       </c>
       <c r="H56" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="57">
@@ -2509,12 +2509,12 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS y MARGENES</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D57" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e00515fb-8071-400a-bf39-fa070c0f663c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ae8549ef-1d06-44e3-b0ec-228ba42aaafe&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E57" t="inlineStr"/>
@@ -2529,7 +2529,7 @@
         </is>
       </c>
       <c r="H57" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="58">
@@ -3505,7 +3505,7 @@
         </is>
       </c>
       <c r="H84" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="85">
@@ -3545,7 +3545,7 @@
         </is>
       </c>
       <c r="H85" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="86">
@@ -3585,7 +3585,7 @@
         </is>
       </c>
       <c r="H86" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="87">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="90">
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="97">
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="98">
@@ -4021,7 +4021,7 @@
         </is>
       </c>
       <c r="H98" t="n">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="99">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="100">
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="101">
@@ -4129,7 +4129,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="102">
@@ -4669,7 +4669,7 @@
         </is>
       </c>
       <c r="H116" t="n">
-        <v>1446</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="117">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>507</v>
+        <v>517</v>
       </c>
     </row>
     <row r="118">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>337</v>
+        <v>350</v>
       </c>
     </row>
     <row r="121">
@@ -4829,12 +4829,12 @@
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN</t>
+          <t>EVOLUCION</t>
         </is>
       </c>
       <c r="D121" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=f62bbf09-eca6-4bb8-8caa-e88da0c3184d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E121" t="inlineStr"/>
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>271</v>
+        <v>274</v>
       </c>
     </row>
     <row r="122">
@@ -4865,12 +4865,12 @@
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>EVOLUCION</t>
+          <t>INCENTIVOS COUSTLAIN</t>
         </is>
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=849ac12f-c28b-4306-a0fe-6a00c6c9c8e8&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=f62bbf09-eca6-4bb8-8caa-e88da0c3184d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E122" t="inlineStr"/>
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>270</v>
+        <v>273</v>
       </c>
     </row>
     <row r="123">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="124">
@@ -4973,12 +4973,12 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D125" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E125" t="inlineStr"/>
@@ -4993,7 +4993,7 @@
         </is>
       </c>
       <c r="H125" t="n">
-        <v>43</v>
+        <v>49</v>
       </c>
     </row>
     <row r="126">
@@ -5009,12 +5009,12 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="D126" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=42c67b63-aaa5-49af-9e3f-48f033c78aeb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d33e3dcd-18b9-4114-83d8-42300c627ebc&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E126" t="inlineStr"/>
@@ -5029,7 +5029,7 @@
         </is>
       </c>
       <c r="H126" t="n">
-        <v>40</v>
+        <v>43</v>
       </c>
     </row>
     <row r="127">
@@ -5137,7 +5137,7 @@
         </is>
       </c>
       <c r="H129" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="130">
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
     </row>
     <row r="131">
@@ -6244,7 +6244,7 @@
         </is>
       </c>
       <c r="L2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -6464,7 +6464,7 @@
         </is>
       </c>
       <c r="L7" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -6508,7 +6508,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9">
@@ -6552,7 +6552,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>71</v>
+        <v>72</v>
       </c>
     </row>
     <row r="10">
@@ -6728,7 +6728,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>48</v>
+        <v>51</v>
       </c>
     </row>
     <row r="14">
@@ -6948,7 +6948,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>22</v>
+        <v>25</v>
       </c>
     </row>
     <row r="19">
@@ -7808,7 +7808,7 @@
         </is>
       </c>
       <c r="L34" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
     </row>
     <row r="35">
@@ -7920,7 +7920,7 @@
         </is>
       </c>
       <c r="L36" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
     </row>
     <row r="37">
@@ -7976,7 +7976,7 @@
         </is>
       </c>
       <c r="L37" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="38">
@@ -9668,7 +9668,7 @@
         </is>
       </c>
       <c r="L71" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
     </row>
     <row r="72">
@@ -9712,7 +9712,7 @@
         </is>
       </c>
       <c r="L72" t="n">
-        <v>6</v>
+        <v>9</v>
       </c>
     </row>
     <row r="73">
@@ -10928,7 +10928,11 @@
           <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
-      <c r="I95" t="inlineStr"/>
+      <c r="I95" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J95" t="inlineStr">
         <is>
           <t>Directorio</t>
@@ -10984,7 +10988,7 @@
         </is>
       </c>
       <c r="L96" t="n">
-        <v>57</v>
+        <v>58</v>
       </c>
     </row>
     <row r="97">
@@ -11076,7 +11080,7 @@
         </is>
       </c>
       <c r="L98" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
     </row>
     <row r="99">
@@ -11256,7 +11260,7 @@
         </is>
       </c>
       <c r="L102" t="n">
-        <v>29</v>
+        <v>27</v>
       </c>
     </row>
     <row r="103">
@@ -11520,7 +11524,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="109">
@@ -11992,7 +11996,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>53</v>
+        <v>55</v>
       </c>
     </row>
     <row r="119">
@@ -12124,7 +12128,7 @@
         </is>
       </c>
       <c r="L121" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
     </row>
     <row r="122">
@@ -12168,7 +12172,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>50</v>
+        <v>53</v>
       </c>
     </row>
     <row r="123">
@@ -12256,7 +12260,7 @@
         </is>
       </c>
       <c r="L124" t="n">
-        <v>118</v>
+        <v>119</v>
       </c>
     </row>
     <row r="125">
@@ -12476,7 +12480,7 @@
         </is>
       </c>
       <c r="L129" t="n">
-        <v>106</v>
+        <v>114</v>
       </c>
     </row>
     <row r="130">
@@ -12608,7 +12612,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>129</v>
+        <v>130</v>
       </c>
     </row>
     <row r="133">
@@ -12864,7 +12868,7 @@
         </is>
       </c>
       <c r="L137" t="n">
-        <v>38</v>
+        <v>39</v>
       </c>
     </row>
     <row r="138">
@@ -13256,7 +13260,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="145">
@@ -13368,7 +13372,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>328</v>
+        <v>316</v>
       </c>
     </row>
     <row r="147">
@@ -13480,7 +13484,7 @@
         </is>
       </c>
       <c r="L148" t="n">
-        <v>312</v>
+        <v>313</v>
       </c>
     </row>
     <row r="149">
@@ -13536,7 +13540,7 @@
         </is>
       </c>
       <c r="L149" t="n">
-        <v>25</v>
+        <v>37</v>
       </c>
     </row>
     <row r="150">
@@ -13712,7 +13716,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>507</v>
+        <v>517</v>
       </c>
     </row>
     <row r="154">
@@ -13800,7 +13804,7 @@
         </is>
       </c>
       <c r="L155" t="n">
-        <v>270</v>
+        <v>274</v>
       </c>
     </row>
     <row r="156">
@@ -14516,7 +14520,7 @@
         </is>
       </c>
       <c r="L168" t="n">
-        <v>36</v>
+        <v>34</v>
       </c>
     </row>
     <row r="169">
@@ -14684,7 +14688,7 @@
         </is>
       </c>
       <c r="L171" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="172">
@@ -14772,7 +14776,7 @@
         </is>
       </c>
       <c r="L173" t="n">
-        <v>1446</v>
+        <v>1456</v>
       </c>
     </row>
     <row r="174">
@@ -14904,7 +14908,7 @@
         </is>
       </c>
       <c r="L176" t="n">
-        <v>271</v>
+        <v>273</v>
       </c>
     </row>
     <row r="177">
@@ -14992,7 +14996,7 @@
         </is>
       </c>
       <c r="L178" t="n">
-        <v>40</v>
+        <v>49</v>
       </c>
     </row>
     <row r="179">
@@ -15124,7 +15128,7 @@
         </is>
       </c>
       <c r="L181" t="n">
-        <v>251</v>
+        <v>245</v>
       </c>
     </row>
     <row r="182">
@@ -16336,7 +16340,11 @@
           <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
         </is>
       </c>
-      <c r="I204" t="inlineStr"/>
+      <c r="I204" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J204" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -17076,7 +17084,7 @@
         </is>
       </c>
       <c r="L217" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
     </row>
     <row r="218">
@@ -17172,7 +17180,11 @@
           <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
         </is>
       </c>
-      <c r="I219" t="inlineStr"/>
+      <c r="I219" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J219" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>

</xml_diff>

<commit_message>
Actualizo tableros (2026-09-12 08:09) - 133 informes de Power BI y 27 links a mano
</commit_message>
<xml_diff>
--- a/LINKS POWER BI.xlsx
+++ b/LINKS POWER BI.xlsx
@@ -11,8 +11,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Catalogo" sheetId="2" state="visible" r:id="rId2"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$160</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$229</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Tableros'!$A$1:$H$161</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'Catalogo'!$A$1:$L$230</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H160"/>
+  <dimension ref="A1:H161"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -1521,7 +1521,7 @@
         </is>
       </c>
       <c r="H29" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="30">
@@ -1593,7 +1593,7 @@
         </is>
       </c>
       <c r="H31" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="32">
@@ -1629,7 +1629,7 @@
         </is>
       </c>
       <c r="H32" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="33">
@@ -1665,7 +1665,7 @@
         </is>
       </c>
       <c r="H33" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="34">
@@ -1881,7 +1881,7 @@
         </is>
       </c>
       <c r="H39" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="40">
@@ -1917,7 +1917,7 @@
         </is>
       </c>
       <c r="H40" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="41">
@@ -2257,12 +2257,12 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>AVANCE PEÑAFLOR</t>
         </is>
       </c>
       <c r="D50" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E50" t="inlineStr"/>
@@ -2293,12 +2293,12 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D51" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4e0903c4-5dde-45ce-ad9f-6aed6e2a4136&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E51" t="inlineStr"/>
@@ -2329,12 +2329,12 @@
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>AVANCE PEÑAFLOR</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D52" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=18fd2917-e128-47d7-b930-81698225d577&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9387acc1-2f91-4921-9891-fb194c770f25&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E52" t="inlineStr"/>
@@ -2349,7 +2349,7 @@
         </is>
       </c>
       <c r="H52" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="53">
@@ -3697,7 +3697,7 @@
         </is>
       </c>
       <c r="H89" t="n">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="90">
@@ -3877,7 +3877,7 @@
         </is>
       </c>
       <c r="H94" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="95">
@@ -3913,7 +3913,7 @@
         </is>
       </c>
       <c r="H95" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="96">
@@ -3929,12 +3929,12 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
         </is>
       </c>
       <c r="D96" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c6b3722f-f2be-40b3-a553-6fb690c3adea&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=8bdb45d1-c1c9-4ee3-9658-d4ab30fb67b9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E96" t="inlineStr"/>
@@ -3949,7 +3949,7 @@
         </is>
       </c>
       <c r="H96" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="97">
@@ -3965,12 +3965,12 @@
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS Y MARGENES</t>
+          <t>STOCK POR PROVEEDORES</t>
         </is>
       </c>
       <c r="D97" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=8bdb45d1-c1c9-4ee3-9658-d4ab30fb67b9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c6b3722f-f2be-40b3-a553-6fb690c3adea&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E97" t="inlineStr"/>
@@ -3985,7 +3985,7 @@
         </is>
       </c>
       <c r="H97" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="98">
@@ -4057,7 +4057,7 @@
         </is>
       </c>
       <c r="H99" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="100">
@@ -4093,7 +4093,7 @@
         </is>
       </c>
       <c r="H100" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="101">
@@ -4129,7 +4129,7 @@
         </is>
       </c>
       <c r="H101" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="102">
@@ -4181,12 +4181,12 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>COMPARATIVO 08-2026</t>
+          <t>PAPELERA</t>
         </is>
       </c>
       <c r="D103" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E103" t="inlineStr"/>
@@ -4201,7 +4201,7 @@
         </is>
       </c>
       <c r="H103" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="104">
@@ -4217,12 +4217,12 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>COMPARATIVO 09-2026</t>
+          <t>COMPARATIVO 08-2026</t>
         </is>
       </c>
       <c r="D104" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=855b1a3d-085c-4aa0-a601-07463be25697&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E104" t="inlineStr"/>
@@ -4253,12 +4253,12 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>COMPARATIVO 09-2026</t>
         </is>
       </c>
       <c r="D105" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ce211e51-d8ab-47c6-a04b-5ecfabd982c0&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E105" t="inlineStr"/>
@@ -4289,12 +4289,12 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="D106" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c813b301-39f1-437a-9c86-03044d1c976f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E106" t="inlineStr"/>
@@ -4325,12 +4325,12 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>PAPELERA</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D107" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=164998e9-90bc-46f7-8360-efbbe3f5da7f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=e8151a94-ab3c-4362-8aeb-160dc3ff5ed9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E107" t="inlineStr"/>
@@ -4489,7 +4489,7 @@
         </is>
       </c>
       <c r="H111" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="112">
@@ -4705,7 +4705,7 @@
         </is>
       </c>
       <c r="H117" t="n">
-        <v>1481</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="118">
@@ -4741,7 +4741,7 @@
         </is>
       </c>
       <c r="H118" t="n">
-        <v>509</v>
+        <v>521</v>
       </c>
     </row>
     <row r="119">
@@ -4777,7 +4777,7 @@
         </is>
       </c>
       <c r="H119" t="n">
-        <v>370</v>
+        <v>382</v>
       </c>
     </row>
     <row r="120">
@@ -4813,7 +4813,7 @@
         </is>
       </c>
       <c r="H120" t="n">
-        <v>370</v>
+        <v>382</v>
       </c>
     </row>
     <row r="121">
@@ -4849,7 +4849,7 @@
         </is>
       </c>
       <c r="H121" t="n">
-        <v>355</v>
+        <v>356</v>
       </c>
     </row>
     <row r="122">
@@ -4885,7 +4885,7 @@
         </is>
       </c>
       <c r="H122" t="n">
-        <v>273</v>
+        <v>275</v>
       </c>
     </row>
     <row r="123">
@@ -4921,7 +4921,7 @@
         </is>
       </c>
       <c r="H123" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="124">
@@ -4957,7 +4957,7 @@
         </is>
       </c>
       <c r="H124" t="n">
-        <v>244</v>
+        <v>248</v>
       </c>
     </row>
     <row r="125">
@@ -5173,7 +5173,7 @@
         </is>
       </c>
       <c r="H130" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="131">
@@ -5209,7 +5209,7 @@
         </is>
       </c>
       <c r="H131" t="n">
-        <v>27</v>
+        <v>30</v>
       </c>
     </row>
     <row r="132">
@@ -5245,7 +5245,7 @@
         </is>
       </c>
       <c r="H132" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="133">
@@ -5333,12 +5333,12 @@
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="D135" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E135" t="inlineStr"/>
@@ -5353,7 +5353,7 @@
         </is>
       </c>
       <c r="H135" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
     </row>
     <row r="136">
@@ -5369,12 +5369,12 @@
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="D136" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d3503eaf-eda8-492e-9a13-46088a447d3f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E136" t="inlineStr"/>
@@ -5405,12 +5405,12 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>ANALISISOFERTAS</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=059b36e9-ab26-4fb2-8647-67f060e36c7c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E137" t="inlineStr"/>
@@ -5425,7 +5425,7 @@
         </is>
       </c>
       <c r="H137" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="138">
@@ -5441,12 +5441,12 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E138" t="inlineStr"/>
@@ -5461,7 +5461,7 @@
         </is>
       </c>
       <c r="H138" t="n">
-        <v>3</v>
+        <v>7</v>
       </c>
     </row>
     <row r="139">
@@ -5477,12 +5477,12 @@
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>ANALISISOFERTAS</t>
         </is>
       </c>
       <c r="D139" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=034fc54a-d18c-44b2-9915-aa86bd8b02f1&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E139" t="inlineStr"/>
@@ -5497,7 +5497,7 @@
         </is>
       </c>
       <c r="H139" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="140">
@@ -5513,12 +5513,12 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=4ae4d5e5-5b71-43a1-ae96-169f12bb778d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E140" t="inlineStr"/>
@@ -5533,7 +5533,7 @@
         </is>
       </c>
       <c r="H140" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="141">
@@ -5549,12 +5549,12 @@
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="D141" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=d4c771ab-037f-4dd0-a7d4-0bb133878a30&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E141" t="inlineStr"/>
@@ -5569,7 +5569,7 @@
         </is>
       </c>
       <c r="H141" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="142">
@@ -5585,12 +5585,12 @@
       </c>
       <c r="C142" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="D142" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=0044864d-c76b-4257-95df-ddc0c9aa2d0e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E142" t="inlineStr"/>
@@ -5621,12 +5621,12 @@
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="D143" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=154d97f3-0014-41a3-b840-4704ad8d886f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E143" t="inlineStr"/>
@@ -5657,12 +5657,12 @@
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="D144" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=3c32ea4c-88e3-473f-8690-fbd5c62a4a7d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E144" t="inlineStr"/>
@@ -5693,12 +5693,12 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="D145" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=40805cb7-8f94-4203-86c8-49c563a4dfd9&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E145" t="inlineStr"/>
@@ -5729,12 +5729,12 @@
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>COMPARATIVO CERVEZAS</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="D146" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=982f2555-a3ca-499b-8d07-13f975303e56&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E146" t="inlineStr"/>
@@ -5749,7 +5749,7 @@
         </is>
       </c>
       <c r="H146" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="147">
@@ -5765,12 +5765,12 @@
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>EFECTIVIDADES MAYORISTA</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="D147" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=9eded255-affc-41f1-82a7-38bb12771cde&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E147" t="inlineStr"/>
@@ -5785,7 +5785,7 @@
         </is>
       </c>
       <c r="H147" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="148">
@@ -5801,12 +5801,12 @@
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>COMPARATIVO CERVEZAS</t>
         </is>
       </c>
       <c r="D148" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=30580dcd-18a8-4764-b965-e447e8860cf4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E148" t="inlineStr"/>
@@ -5837,12 +5837,12 @@
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>EFECTIVIDADES MAYORISTA</t>
         </is>
       </c>
       <c r="D149" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=1632e5a1-1d96-42be-b9c6-a2d58321335e&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E149" t="inlineStr"/>
@@ -5873,12 +5873,12 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="D150" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=73fcaa5b-374d-40ed-ac92-cd2009bb1c6d&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E150" t="inlineStr"/>
@@ -5909,12 +5909,12 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="D151" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=14432aec-0724-4c98-905f-1f2681948b2f&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E151" t="inlineStr"/>
@@ -5945,12 +5945,12 @@
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="D152" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=7f57b337-e918-4c13-aa6e-3e42d193d9b4&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E152" t="inlineStr"/>
@@ -5981,12 +5981,12 @@
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="D153" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=c2bc6772-69d9-4a1b-a1f6-b5c36c53c999&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E153" t="inlineStr"/>
@@ -6017,12 +6017,12 @@
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="D154" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=ee814c80-8be3-47a9-af5a-1132ad0f4f31&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E154" t="inlineStr"/>
@@ -6053,12 +6053,12 @@
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="D155" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=95773ea4-d11f-4574-b74e-a0675a8dd346&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E155" t="inlineStr"/>
@@ -6089,12 +6089,12 @@
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="D156" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=27c984a1-8a8c-4da5-bb04-fc0b98239a0a&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=784d6896-dd8a-4b7a-9c5c-962ea6c5e49c&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E156" t="inlineStr"/>
@@ -6125,12 +6125,12 @@
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="D157" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=08eee5c2-f90d-483d-9382-0726090489f7&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E157" t="inlineStr"/>
@@ -6161,12 +6161,12 @@
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=65db6ab7-0b7f-4010-bc49-7c986f097c10&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
@@ -6197,12 +6197,12 @@
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=88b79c83-6c87-449b-b022-42b61ebf934b&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=16acb159-f0ec-4a26-8221-f63c9516d249&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -6228,17 +6228,17 @@
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+          <t>https://app.powerbi.com/reportEmbed?reportId=6c931870-e5c9-4cbc-9aac-e0368aab3ffb&amp;autoAuth=true</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -6256,8 +6256,44 @@
         <v>0</v>
       </c>
     </row>
+    <row r="161">
+      <c r="A161" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="B161" t="inlineStr">
+        <is>
+          <t>MENOR COSTE</t>
+        </is>
+      </c>
+      <c r="C161" t="inlineStr">
+        <is>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+        </is>
+      </c>
+      <c r="D161" t="inlineStr">
+        <is>
+          <t>https://app.powerbi.com/reportEmbed?reportId=002a3f72-0d37-46fa-8cee-aa0b67dcb88c&amp;autoAuth=true</t>
+        </is>
+      </c>
+      <c r="E161" t="inlineStr"/>
+      <c r="F161" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+      <c r="G161" t="inlineStr">
+        <is>
+          <t>INFORME</t>
+        </is>
+      </c>
+      <c r="H161" t="n">
+        <v>0</v>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H160"/>
+  <autoFilter ref="A1:H161"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -6268,7 +6304,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L229"/>
+  <dimension ref="A1:L230"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="10" customWidth="1" min="1" max="1"/>
@@ -6432,7 +6468,7 @@
         </is>
       </c>
       <c r="L3" t="n">
-        <v>28</v>
+        <v>30</v>
       </c>
     </row>
     <row r="4">
@@ -6652,7 +6688,7 @@
         </is>
       </c>
       <c r="L8" t="n">
-        <v>36</v>
+        <v>37</v>
       </c>
     </row>
     <row r="9">
@@ -6696,7 +6732,7 @@
         </is>
       </c>
       <c r="L9" t="n">
-        <v>80</v>
+        <v>82</v>
       </c>
     </row>
     <row r="10">
@@ -6872,7 +6908,7 @@
         </is>
       </c>
       <c r="L13" t="n">
-        <v>63</v>
+        <v>67</v>
       </c>
     </row>
     <row r="14">
@@ -6960,7 +6996,7 @@
         </is>
       </c>
       <c r="L15" t="n">
-        <v>55</v>
+        <v>57</v>
       </c>
     </row>
     <row r="16">
@@ -7092,7 +7128,7 @@
         </is>
       </c>
       <c r="L18" t="n">
-        <v>27</v>
+        <v>29</v>
       </c>
     </row>
     <row r="19">
@@ -7136,7 +7172,7 @@
         </is>
       </c>
       <c r="L19" t="n">
-        <v>23</v>
+        <v>25</v>
       </c>
     </row>
     <row r="20">
@@ -11624,7 +11660,7 @@
         </is>
       </c>
       <c r="L107" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
     </row>
     <row r="108">
@@ -11668,7 +11704,7 @@
         </is>
       </c>
       <c r="L108" t="n">
-        <v>168</v>
+        <v>172</v>
       </c>
     </row>
     <row r="109">
@@ -11712,7 +11748,7 @@
         </is>
       </c>
       <c r="L109" t="n">
-        <v>2</v>
+        <v>13</v>
       </c>
     </row>
     <row r="110">
@@ -12140,7 +12176,7 @@
         </is>
       </c>
       <c r="L118" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
     </row>
     <row r="119">
@@ -12316,7 +12352,7 @@
         </is>
       </c>
       <c r="L122" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
     </row>
     <row r="123">
@@ -12360,7 +12396,7 @@
         </is>
       </c>
       <c r="L123" t="n">
-        <v>54</v>
+        <v>56</v>
       </c>
     </row>
     <row r="124">
@@ -12448,7 +12484,7 @@
         </is>
       </c>
       <c r="L125" t="n">
-        <v>126</v>
+        <v>131</v>
       </c>
     </row>
     <row r="126">
@@ -12580,7 +12616,7 @@
         </is>
       </c>
       <c r="L128" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
     </row>
     <row r="129">
@@ -12756,7 +12792,7 @@
         </is>
       </c>
       <c r="L132" t="n">
-        <v>58</v>
+        <v>60</v>
       </c>
     </row>
     <row r="133">
@@ -12800,7 +12836,7 @@
         </is>
       </c>
       <c r="L133" t="n">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="134">
@@ -13056,7 +13092,7 @@
         </is>
       </c>
       <c r="L138" t="n">
-        <v>39</v>
+        <v>41</v>
       </c>
     </row>
     <row r="139">
@@ -13392,7 +13428,7 @@
         </is>
       </c>
       <c r="L144" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="145">
@@ -13504,7 +13540,7 @@
         </is>
       </c>
       <c r="L146" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
     </row>
     <row r="147">
@@ -13560,7 +13596,7 @@
         </is>
       </c>
       <c r="L147" t="n">
-        <v>291</v>
+        <v>292</v>
       </c>
     </row>
     <row r="148">
@@ -13728,7 +13764,7 @@
         </is>
       </c>
       <c r="L150" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
     </row>
     <row r="151">
@@ -13860,7 +13896,7 @@
         </is>
       </c>
       <c r="L153" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
     </row>
     <row r="154">
@@ -13904,7 +13940,7 @@
         </is>
       </c>
       <c r="L154" t="n">
-        <v>509</v>
+        <v>521</v>
       </c>
     </row>
     <row r="155">
@@ -13992,7 +14028,7 @@
         </is>
       </c>
       <c r="L156" t="n">
-        <v>270</v>
+        <v>271</v>
       </c>
     </row>
     <row r="157">
@@ -14057,30 +14093,18 @@
       </c>
       <c r="D158" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2025</t>
+          <t>GRUPO CLIENTES BLACK 2026</t>
         </is>
       </c>
       <c r="E158" t="inlineStr"/>
-      <c r="F158" t="inlineStr">
-        <is>
-          <t>HECTOLITROS</t>
-        </is>
-      </c>
-      <c r="G158" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F158" t="inlineStr"/>
+      <c r="G158" t="inlineStr"/>
       <c r="H158" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 25</t>
-        </is>
-      </c>
-      <c r="I158" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>Grupo Clientes BLACK 2026</t>
+        </is>
+      </c>
+      <c r="I158" t="inlineStr"/>
       <c r="J158" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14088,11 +14112,11 @@
       </c>
       <c r="K158" t="inlineStr">
         <is>
-          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
+          <t>73fcaa5b-374d-40ed-ac92-cd2009bb1c6d</t>
         </is>
       </c>
       <c r="L158" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="159">
@@ -14113,7 +14137,7 @@
       </c>
       <c r="D159" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2025</t>
+          <t>HECTOLITROS 07-2025</t>
         </is>
       </c>
       <c r="E159" t="inlineStr"/>
@@ -14124,17 +14148,17 @@
       </c>
       <c r="G159" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H159" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 25</t>
+          <t>Informe Hctos - Julio 25</t>
         </is>
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -14144,11 +14168,11 @@
       </c>
       <c r="K159" t="inlineStr">
         <is>
-          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
+          <t>502a205e-9f71-4d24-862a-52d839f1e116</t>
         </is>
       </c>
       <c r="L159" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="160">
@@ -14169,7 +14193,7 @@
       </c>
       <c r="D160" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2025</t>
+          <t>HECTOLITROS 08-2025</t>
         </is>
       </c>
       <c r="E160" t="inlineStr"/>
@@ -14180,17 +14204,17 @@
       </c>
       <c r="G160" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H160" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 25</t>
+          <t>Informe Hctos - Agosto 25</t>
         </is>
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -14200,7 +14224,7 @@
       </c>
       <c r="K160" t="inlineStr">
         <is>
-          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
+          <t>b4d6b026-7a58-416c-918b-834458a06075</t>
         </is>
       </c>
       <c r="L160" t="n">
@@ -14225,7 +14249,7 @@
       </c>
       <c r="D161" t="inlineStr">
         <is>
-          <t>HECTOLITROS 10-2025</t>
+          <t>HECTOLITROS 09-2025</t>
         </is>
       </c>
       <c r="E161" t="inlineStr"/>
@@ -14236,17 +14260,17 @@
       </c>
       <c r="G161" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H161" t="inlineStr">
         <is>
-          <t>Informe Hctos - Octubre 25</t>
+          <t>Informe Hctos - Septiembre 25</t>
         </is>
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -14256,7 +14280,7 @@
       </c>
       <c r="K161" t="inlineStr">
         <is>
-          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
+          <t>dd06ecfb-25a3-4f06-b6ac-c74dd4f5d5e7</t>
         </is>
       </c>
       <c r="L161" t="n">
@@ -14281,7 +14305,7 @@
       </c>
       <c r="D162" t="inlineStr">
         <is>
-          <t>HECTOLITROS 11-2025</t>
+          <t>HECTOLITROS 10-2025</t>
         </is>
       </c>
       <c r="E162" t="inlineStr"/>
@@ -14292,17 +14316,17 @@
       </c>
       <c r="G162" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H162" t="inlineStr">
         <is>
-          <t>Informe Hctos - Noviembre 25</t>
+          <t>Informe Hctos - Octubre 25</t>
         </is>
       </c>
       <c r="I162" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J162" t="inlineStr">
@@ -14312,7 +14336,7 @@
       </c>
       <c r="K162" t="inlineStr">
         <is>
-          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
+          <t>002d561c-4948-4eed-8a69-c915d548675e</t>
         </is>
       </c>
       <c r="L162" t="n">
@@ -14337,7 +14361,7 @@
       </c>
       <c r="D163" t="inlineStr">
         <is>
-          <t>HECTOLITROS 12-2025</t>
+          <t>HECTOLITROS 11-2025</t>
         </is>
       </c>
       <c r="E163" t="inlineStr"/>
@@ -14348,17 +14372,17 @@
       </c>
       <c r="G163" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H163" t="inlineStr">
         <is>
-          <t>Informe Hctos - Diciembre 25</t>
+          <t>Informe Hctos - Noviembre 25</t>
         </is>
       </c>
       <c r="I163" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J163" t="inlineStr">
@@ -14368,7 +14392,7 @@
       </c>
       <c r="K163" t="inlineStr">
         <is>
-          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
+          <t>6c3448ae-712c-4df3-a42f-c986ffb0c26a</t>
         </is>
       </c>
       <c r="L163" t="n">
@@ -14393,7 +14417,7 @@
       </c>
       <c r="D164" t="inlineStr">
         <is>
-          <t>HECTOLITROS 01-2026</t>
+          <t>HECTOLITROS 12-2025</t>
         </is>
       </c>
       <c r="E164" t="inlineStr"/>
@@ -14404,17 +14428,17 @@
       </c>
       <c r="G164" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H164" t="inlineStr">
         <is>
-          <t>Informe Hctos - Enero 26</t>
+          <t>Informe Hctos - Diciembre 25</t>
         </is>
       </c>
       <c r="I164" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J164" t="inlineStr">
@@ -14424,7 +14448,7 @@
       </c>
       <c r="K164" t="inlineStr">
         <is>
-          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
+          <t>bace738c-d630-4912-b89d-fa72dd3f11e9</t>
         </is>
       </c>
       <c r="L164" t="n">
@@ -14449,7 +14473,7 @@
       </c>
       <c r="D165" t="inlineStr">
         <is>
-          <t>HECTOLITROS 02-2026</t>
+          <t>HECTOLITROS 01-2026</t>
         </is>
       </c>
       <c r="E165" t="inlineStr"/>
@@ -14460,17 +14484,17 @@
       </c>
       <c r="G165" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H165" t="inlineStr">
         <is>
-          <t>Informe Hctos - Febrero 26</t>
+          <t>Informe Hctos - Enero 26</t>
         </is>
       </c>
       <c r="I165" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J165" t="inlineStr">
@@ -14480,7 +14504,7 @@
       </c>
       <c r="K165" t="inlineStr">
         <is>
-          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
+          <t>469ea0a5-13da-4cbe-996f-d1b982c6f6b2</t>
         </is>
       </c>
       <c r="L165" t="n">
@@ -14505,7 +14529,7 @@
       </c>
       <c r="D166" t="inlineStr">
         <is>
-          <t>HECTOLITROS 03-2026</t>
+          <t>HECTOLITROS 02-2026</t>
         </is>
       </c>
       <c r="E166" t="inlineStr"/>
@@ -14516,17 +14540,17 @@
       </c>
       <c r="G166" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H166" t="inlineStr">
         <is>
-          <t>Informe Hctos - Marzo 26</t>
+          <t>Informe Hctos - Febrero 26</t>
         </is>
       </c>
       <c r="I166" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J166" t="inlineStr">
@@ -14536,7 +14560,7 @@
       </c>
       <c r="K166" t="inlineStr">
         <is>
-          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
+          <t>c8b20d51-5004-4ed9-b1e1-9ebde07fa251</t>
         </is>
       </c>
       <c r="L166" t="n">
@@ -14561,7 +14585,7 @@
       </c>
       <c r="D167" t="inlineStr">
         <is>
-          <t>HECTOLITROS 04-2026</t>
+          <t>HECTOLITROS 03-2026</t>
         </is>
       </c>
       <c r="E167" t="inlineStr"/>
@@ -14572,17 +14596,17 @@
       </c>
       <c r="G167" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H167" t="inlineStr">
         <is>
-          <t>Informe Hctos - Abril 26</t>
+          <t>Informe Hctos - Marzo 26</t>
         </is>
       </c>
       <c r="I167" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J167" t="inlineStr">
@@ -14592,11 +14616,11 @@
       </c>
       <c r="K167" t="inlineStr">
         <is>
-          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
+          <t>a1ce951a-4057-40e6-8c22-d789769790d6</t>
         </is>
       </c>
       <c r="L167" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="168">
@@ -14617,7 +14641,7 @@
       </c>
       <c r="D168" t="inlineStr">
         <is>
-          <t>HECTOLITROS 05-2026</t>
+          <t>HECTOLITROS 04-2026</t>
         </is>
       </c>
       <c r="E168" t="inlineStr"/>
@@ -14628,17 +14652,17 @@
       </c>
       <c r="G168" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H168" t="inlineStr">
         <is>
-          <t>Informe Hctos - Mayo 26</t>
+          <t>Informe Hctos - Abril 26</t>
         </is>
       </c>
       <c r="I168" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J168" t="inlineStr">
@@ -14648,11 +14672,11 @@
       </c>
       <c r="K168" t="inlineStr">
         <is>
-          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
+          <t>24c5543f-4401-4463-905d-783c3592b69c</t>
         </is>
       </c>
       <c r="L168" t="n">
-        <v>8</v>
+        <v>1</v>
       </c>
     </row>
     <row r="169">
@@ -14673,7 +14697,7 @@
       </c>
       <c r="D169" t="inlineStr">
         <is>
-          <t>HECTOLITROS 06-2026</t>
+          <t>HECTOLITROS 05-2026</t>
         </is>
       </c>
       <c r="E169" t="inlineStr"/>
@@ -14684,17 +14708,17 @@
       </c>
       <c r="G169" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H169" t="inlineStr">
         <is>
-          <t>Informe Hctos - Junio 26</t>
+          <t>Informe Hctos - Mayo 26</t>
         </is>
       </c>
       <c r="I169" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J169" t="inlineStr">
@@ -14704,11 +14728,11 @@
       </c>
       <c r="K169" t="inlineStr">
         <is>
-          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
+          <t>81a70b79-ca41-4482-8bdd-11b84b3ae000</t>
         </is>
       </c>
       <c r="L169" t="n">
-        <v>33</v>
+        <v>8</v>
       </c>
     </row>
     <row r="170">
@@ -14729,7 +14753,7 @@
       </c>
       <c r="D170" t="inlineStr">
         <is>
-          <t>HECTOLITROS 07-2026</t>
+          <t>HECTOLITROS 06-2026</t>
         </is>
       </c>
       <c r="E170" t="inlineStr"/>
@@ -14740,17 +14764,17 @@
       </c>
       <c r="G170" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H170" t="inlineStr">
         <is>
-          <t>Informe Hctos - Julio 26</t>
+          <t>Informe Hctos - Junio 26</t>
         </is>
       </c>
       <c r="I170" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J170" t="inlineStr">
@@ -14760,11 +14784,11 @@
       </c>
       <c r="K170" t="inlineStr">
         <is>
-          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
+          <t>2c9470fd-aaa7-4fe5-bee1-1adb70fe8f78</t>
         </is>
       </c>
       <c r="L170" t="n">
-        <v>41</v>
+        <v>33</v>
       </c>
     </row>
     <row r="171">
@@ -14785,7 +14809,7 @@
       </c>
       <c r="D171" t="inlineStr">
         <is>
-          <t>HECTOLITROS 08-2026</t>
+          <t>HECTOLITROS 07-2026</t>
         </is>
       </c>
       <c r="E171" t="inlineStr"/>
@@ -14796,17 +14820,17 @@
       </c>
       <c r="G171" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H171" t="inlineStr">
         <is>
-          <t>Informe Hctos - Agosto 26</t>
+          <t>Informe Hctos - Julio 26</t>
         </is>
       </c>
       <c r="I171" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J171" t="inlineStr">
@@ -14816,11 +14840,11 @@
       </c>
       <c r="K171" t="inlineStr">
         <is>
-          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
+          <t>5a75e8c7-9e82-4d6f-975a-72bbb3434a4d</t>
         </is>
       </c>
       <c r="L171" t="n">
-        <v>26</v>
+        <v>41</v>
       </c>
     </row>
     <row r="172">
@@ -14841,7 +14865,7 @@
       </c>
       <c r="D172" t="inlineStr">
         <is>
-          <t>HECTOLITROS 09-2026</t>
+          <t>HECTOLITROS 08-2026</t>
         </is>
       </c>
       <c r="E172" t="inlineStr"/>
@@ -14852,17 +14876,17 @@
       </c>
       <c r="G172" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H172" t="inlineStr">
         <is>
-          <t>Informe Hctos - Septiembre 26</t>
+          <t>Informe Hctos - Agosto 26</t>
         </is>
       </c>
       <c r="I172" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J172" t="inlineStr">
@@ -14872,11 +14896,11 @@
       </c>
       <c r="K172" t="inlineStr">
         <is>
-          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
+          <t>8534dc2b-7ee4-484d-b3e3-d151ed93adaf</t>
         </is>
       </c>
       <c r="L172" t="n">
-        <v>1</v>
+        <v>26</v>
       </c>
     </row>
     <row r="173">
@@ -14897,18 +14921,30 @@
       </c>
       <c r="D173" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
+          <t>HECTOLITROS 09-2026</t>
         </is>
       </c>
       <c r="E173" t="inlineStr"/>
-      <c r="F173" t="inlineStr"/>
-      <c r="G173" t="inlineStr"/>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>HECTOLITROS</t>
+        </is>
+      </c>
+      <c r="G173" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H173" t="inlineStr">
         <is>
-          <t>INFO MARCA CORE CCU</t>
-        </is>
-      </c>
-      <c r="I173" t="inlineStr"/>
+          <t>Informe Hctos - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I173" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J173" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -14916,11 +14952,11 @@
       </c>
       <c r="K173" t="inlineStr">
         <is>
-          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
+          <t>c1ba4bda-9414-4968-b1f0-98ceb9b4e37b</t>
         </is>
       </c>
       <c r="L173" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="174">
@@ -14941,7 +14977,7 @@
       </c>
       <c r="D174" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="E174" t="inlineStr"/>
@@ -14949,7 +14985,7 @@
       <c r="G174" t="inlineStr"/>
       <c r="H174" t="inlineStr">
         <is>
-          <t>Incentivos ALTA</t>
+          <t>INFO MARCA CORE CCU</t>
         </is>
       </c>
       <c r="I174" t="inlineStr"/>
@@ -14960,11 +14996,11 @@
       </c>
       <c r="K174" t="inlineStr">
         <is>
-          <t>fce7fec8-1591-4d36-937a-104080c89b4f</t>
+          <t>c2bc6772-69d9-4a1b-a1f6-b5c36c53c999</t>
         </is>
       </c>
       <c r="L174" t="n">
-        <v>1481</v>
+        <v>0</v>
       </c>
     </row>
     <row r="175">
@@ -14985,7 +15021,7 @@
       </c>
       <c r="D175" t="inlineStr">
         <is>
-          <t>INCENTIVOS ALTA - VOLUMEN</t>
+          <t>INCENTIVOS ALTA</t>
         </is>
       </c>
       <c r="E175" t="inlineStr"/>
@@ -14993,7 +15029,7 @@
       <c r="G175" t="inlineStr"/>
       <c r="H175" t="inlineStr">
         <is>
-          <t>Incentivos ALTA - VOLUMEN</t>
+          <t>Incentivos ALTA</t>
         </is>
       </c>
       <c r="I175" t="inlineStr"/>
@@ -15004,11 +15040,11 @@
       </c>
       <c r="K175" t="inlineStr">
         <is>
-          <t>14432aec-0724-4c98-905f-1f2681948b2f</t>
+          <t>fce7fec8-1591-4d36-937a-104080c89b4f</t>
         </is>
       </c>
       <c r="L175" t="n">
-        <v>0</v>
+        <v>1494</v>
       </c>
     </row>
     <row r="176">
@@ -15029,7 +15065,7 @@
       </c>
       <c r="D176" t="inlineStr">
         <is>
-          <t>INCENTIVOS BLACK</t>
+          <t>INCENTIVOS ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="E176" t="inlineStr"/>
@@ -15037,7 +15073,7 @@
       <c r="G176" t="inlineStr"/>
       <c r="H176" t="inlineStr">
         <is>
-          <t>Incentivos BLACK</t>
+          <t>Incentivos ALTA - VOLUMEN</t>
         </is>
       </c>
       <c r="I176" t="inlineStr"/>
@@ -15048,11 +15084,11 @@
       </c>
       <c r="K176" t="inlineStr">
         <is>
-          <t>ca6214b2-3622-4950-9f7f-cb22dc1697f8</t>
+          <t>14432aec-0724-4c98-905f-1f2681948b2f</t>
         </is>
       </c>
       <c r="L176" t="n">
-        <v>355</v>
+        <v>0</v>
       </c>
     </row>
     <row r="177">
@@ -15073,7 +15109,7 @@
       </c>
       <c r="D177" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN</t>
+          <t>INCENTIVOS BLACK</t>
         </is>
       </c>
       <c r="E177" t="inlineStr"/>
@@ -15081,7 +15117,7 @@
       <c r="G177" t="inlineStr"/>
       <c r="H177" t="inlineStr">
         <is>
-          <t>Incentivos COUSTLAIN</t>
+          <t>Incentivos BLACK</t>
         </is>
       </c>
       <c r="I177" t="inlineStr"/>
@@ -15092,11 +15128,11 @@
       </c>
       <c r="K177" t="inlineStr">
         <is>
-          <t>f62bbf09-eca6-4bb8-8caa-e88da0c3184d</t>
+          <t>ca6214b2-3622-4950-9f7f-cb22dc1697f8</t>
         </is>
       </c>
       <c r="L177" t="n">
-        <v>273</v>
+        <v>356</v>
       </c>
     </row>
     <row r="178">
@@ -15117,7 +15153,7 @@
       </c>
       <c r="D178" t="inlineStr">
         <is>
-          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
+          <t>INCENTIVOS COUSTLAIN</t>
         </is>
       </c>
       <c r="E178" t="inlineStr"/>
@@ -15125,7 +15161,7 @@
       <c r="G178" t="inlineStr"/>
       <c r="H178" t="inlineStr">
         <is>
-          <t>Incentivos COUSTLAIN - VOLUMEN</t>
+          <t>Incentivos COUSTLAIN</t>
         </is>
       </c>
       <c r="I178" t="inlineStr"/>
@@ -15136,11 +15172,11 @@
       </c>
       <c r="K178" t="inlineStr">
         <is>
-          <t>7f57b337-e918-4c13-aa6e-3e42d193d9b4</t>
+          <t>f62bbf09-eca6-4bb8-8caa-e88da0c3184d</t>
         </is>
       </c>
       <c r="L178" t="n">
-        <v>0</v>
+        <v>275</v>
       </c>
     </row>
     <row r="179">
@@ -15161,7 +15197,7 @@
       </c>
       <c r="D179" t="inlineStr">
         <is>
-          <t>INCORPORACIONES</t>
+          <t>INCENTIVOS COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="E179" t="inlineStr"/>
@@ -15169,7 +15205,7 @@
       <c r="G179" t="inlineStr"/>
       <c r="H179" t="inlineStr">
         <is>
-          <t>Incorporaciones</t>
+          <t>Incentivos COUSTLAIN - VOLUMEN</t>
         </is>
       </c>
       <c r="I179" t="inlineStr"/>
@@ -15180,11 +15216,11 @@
       </c>
       <c r="K179" t="inlineStr">
         <is>
-          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
+          <t>7f57b337-e918-4c13-aa6e-3e42d193d9b4</t>
         </is>
       </c>
       <c r="L179" t="n">
-        <v>59</v>
+        <v>0</v>
       </c>
     </row>
     <row r="180">
@@ -15205,7 +15241,7 @@
       </c>
       <c r="D180" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2025</t>
+          <t>INCORPORACIONES</t>
         </is>
       </c>
       <c r="E180" t="inlineStr"/>
@@ -15213,7 +15249,7 @@
       <c r="G180" t="inlineStr"/>
       <c r="H180" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2025</t>
+          <t>Incorporaciones</t>
         </is>
       </c>
       <c r="I180" t="inlineStr"/>
@@ -15224,11 +15260,11 @@
       </c>
       <c r="K180" t="inlineStr">
         <is>
-          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
+          <t>42c67b63-aaa5-49af-9e3f-48f033c78aeb</t>
         </is>
       </c>
       <c r="L180" t="n">
-        <v>1</v>
+        <v>59</v>
       </c>
     </row>
     <row r="181">
@@ -15249,7 +15285,7 @@
       </c>
       <c r="D181" t="inlineStr">
         <is>
-          <t>INFORME DE PROVEEDORES 2026</t>
+          <t>INFORME DE PROVEEDORES 2025</t>
         </is>
       </c>
       <c r="E181" t="inlineStr"/>
@@ -15257,7 +15293,7 @@
       <c r="G181" t="inlineStr"/>
       <c r="H181" t="inlineStr">
         <is>
-          <t>Informe de Proveedores 2026</t>
+          <t>Informe de Proveedores 2025</t>
         </is>
       </c>
       <c r="I181" t="inlineStr"/>
@@ -15268,11 +15304,11 @@
       </c>
       <c r="K181" t="inlineStr">
         <is>
-          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
+          <t>0044864d-c76b-4257-95df-ddc0c9aa2d0e</t>
         </is>
       </c>
       <c r="L181" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="182">
@@ -15293,7 +15329,7 @@
       </c>
       <c r="D182" t="inlineStr">
         <is>
-          <t>LISTA DE PRECIOS</t>
+          <t>INFORME DE PROVEEDORES 2026</t>
         </is>
       </c>
       <c r="E182" t="inlineStr"/>
@@ -15301,7 +15337,7 @@
       <c r="G182" t="inlineStr"/>
       <c r="H182" t="inlineStr">
         <is>
-          <t>Lista de precios</t>
+          <t>Informe de Proveedores 2026</t>
         </is>
       </c>
       <c r="I182" t="inlineStr"/>
@@ -15312,11 +15348,11 @@
       </c>
       <c r="K182" t="inlineStr">
         <is>
-          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
+          <t>ee814c80-8be3-47a9-af5a-1132ad0f4f31</t>
         </is>
       </c>
       <c r="L182" t="n">
-        <v>244</v>
+        <v>0</v>
       </c>
     </row>
     <row r="183">
@@ -15337,7 +15373,7 @@
       </c>
       <c r="D183" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>LISTA DE PRECIOS</t>
         </is>
       </c>
       <c r="E183" t="inlineStr"/>
@@ -15345,7 +15381,7 @@
       <c r="G183" t="inlineStr"/>
       <c r="H183" t="inlineStr">
         <is>
-          <t>MOLINOS COUSTLAIN VENTAS</t>
+          <t>Lista de precios</t>
         </is>
       </c>
       <c r="I183" t="inlineStr"/>
@@ -15356,11 +15392,11 @@
       </c>
       <c r="K183" t="inlineStr">
         <is>
-          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
+          <t>6afd1ddb-25f2-4631-bf59-fbaceff88e1b</t>
         </is>
       </c>
       <c r="L183" t="n">
-        <v>13</v>
+        <v>248</v>
       </c>
     </row>
     <row r="184">
@@ -15381,30 +15417,18 @@
       </c>
       <c r="D184" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU 07-2025</t>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
         </is>
       </c>
       <c r="E184" t="inlineStr"/>
-      <c r="F184" t="inlineStr">
-        <is>
-          <t>PARTICIPACION VENTAS CCU</t>
-        </is>
-      </c>
-      <c r="G184" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F184" t="inlineStr"/>
+      <c r="G184" t="inlineStr"/>
       <c r="H184" t="inlineStr">
         <is>
-          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
-        </is>
-      </c>
-      <c r="I184" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>MOLINOS COUSTLAIN VENTAS</t>
+        </is>
+      </c>
+      <c r="I184" t="inlineStr"/>
       <c r="J184" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15412,11 +15436,11 @@
       </c>
       <c r="K184" t="inlineStr">
         <is>
-          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
+          <t>7bcd2a2e-06f8-496e-9a39-a3b30deba2ae</t>
         </is>
       </c>
       <c r="L184" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
     </row>
     <row r="185">
@@ -15437,18 +15461,30 @@
       </c>
       <c r="D185" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
+          <t>PARTICIPACION VENTAS CCU 07-2025</t>
         </is>
       </c>
       <c r="E185" t="inlineStr"/>
-      <c r="F185" t="inlineStr"/>
-      <c r="G185" t="inlineStr"/>
+      <c r="F185" t="inlineStr">
+        <is>
+          <t>PARTICIPACION VENTAS CCU</t>
+        </is>
+      </c>
+      <c r="G185" t="inlineStr">
+        <is>
+          <t>07-2025</t>
+        </is>
+      </c>
       <c r="H185" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA</t>
-        </is>
-      </c>
-      <c r="I185" t="inlineStr"/>
+          <t>PARTICIPACION VENTAS CCU - Julio 25</t>
+        </is>
+      </c>
+      <c r="I185" t="inlineStr">
+        <is>
+          <t>Julio - 25</t>
+        </is>
+      </c>
       <c r="J185" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15456,7 +15492,7 @@
       </c>
       <c r="K185" t="inlineStr">
         <is>
-          <t>784d6896-dd8a-4b7a-9c5c-962ea6c5e49c</t>
+          <t>95773ea4-d11f-4574-b74e-a0675a8dd346</t>
         </is>
       </c>
       <c r="L185" t="n">
@@ -15481,30 +15517,18 @@
       </c>
       <c r="D186" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP ALTA 08-2025</t>
+          <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
       <c r="E186" t="inlineStr"/>
-      <c r="F186" t="inlineStr">
+      <c r="F186" t="inlineStr"/>
+      <c r="G186" t="inlineStr"/>
+      <c r="H186" t="inlineStr">
         <is>
           <t>PLAN ESPACIO APP ALTA</t>
         </is>
       </c>
-      <c r="G186" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
-      <c r="H186" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
-        </is>
-      </c>
-      <c r="I186" t="inlineStr">
-        <is>
-          <t>Agosto - 25</t>
-        </is>
-      </c>
+      <c r="I186" t="inlineStr"/>
       <c r="J186" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15512,11 +15536,11 @@
       </c>
       <c r="K186" t="inlineStr">
         <is>
-          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
+          <t>784d6896-dd8a-4b7a-9c5c-962ea6c5e49c</t>
         </is>
       </c>
       <c r="L186" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="187">
@@ -15537,18 +15561,30 @@
       </c>
       <c r="D187" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
+          <t>PLAN ESPACIO APP ALTA 08-2025</t>
         </is>
       </c>
       <c r="E187" t="inlineStr"/>
-      <c r="F187" t="inlineStr"/>
-      <c r="G187" t="inlineStr"/>
+      <c r="F187" t="inlineStr">
+        <is>
+          <t>PLAN ESPACIO APP ALTA</t>
+        </is>
+      </c>
+      <c r="G187" t="inlineStr">
+        <is>
+          <t>08-2025</t>
+        </is>
+      </c>
       <c r="H187" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA</t>
-        </is>
-      </c>
-      <c r="I187" t="inlineStr"/>
+          <t>PLAN ESPACIO APP ALTA - Agosto 25</t>
+        </is>
+      </c>
+      <c r="I187" t="inlineStr">
+        <is>
+          <t>Agosto - 25</t>
+        </is>
+      </c>
       <c r="J187" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15556,11 +15592,11 @@
       </c>
       <c r="K187" t="inlineStr">
         <is>
-          <t>08eee5c2-f90d-483d-9382-0726090489f7</t>
+          <t>154d97f3-0014-41a3-b840-4704ad8d886f</t>
         </is>
       </c>
       <c r="L187" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="188">
@@ -15581,30 +15617,18 @@
       </c>
       <c r="D188" t="inlineStr">
         <is>
-          <t>PLAN ESPACIO APP COSTA 08-2025</t>
+          <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
       <c r="E188" t="inlineStr"/>
-      <c r="F188" t="inlineStr">
+      <c r="F188" t="inlineStr"/>
+      <c r="G188" t="inlineStr"/>
+      <c r="H188" t="inlineStr">
         <is>
           <t>PLAN ESPACIO APP COSTA</t>
         </is>
       </c>
-      <c r="G188" t="inlineStr">
-        <is>
-          <t>08-2025</t>
-        </is>
-      </c>
-      <c r="H188" t="inlineStr">
-        <is>
-          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
-        </is>
-      </c>
-      <c r="I188" t="inlineStr">
-        <is>
-          <t>Agosto - 25</t>
-        </is>
-      </c>
+      <c r="I188" t="inlineStr"/>
       <c r="J188" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15612,7 +15636,7 @@
       </c>
       <c r="K188" t="inlineStr">
         <is>
-          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
+          <t>08eee5c2-f90d-483d-9382-0726090489f7</t>
         </is>
       </c>
       <c r="L188" t="n">
@@ -15637,18 +15661,30 @@
       </c>
       <c r="D189" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
+          <t>PLAN ESPACIO APP COSTA 08-2025</t>
         </is>
       </c>
       <c r="E189" t="inlineStr"/>
-      <c r="F189" t="inlineStr"/>
-      <c r="G189" t="inlineStr"/>
+      <c r="F189" t="inlineStr">
+        <is>
+          <t>PLAN ESPACIO APP COSTA</t>
+        </is>
+      </c>
+      <c r="G189" t="inlineStr">
+        <is>
+          <t>08-2025</t>
+        </is>
+      </c>
       <c r="H189" t="inlineStr">
         <is>
-          <t>PLAN TRADI</t>
-        </is>
-      </c>
-      <c r="I189" t="inlineStr"/>
+          <t>PLAN ESPACIO APP COSTA- Agosto 25</t>
+        </is>
+      </c>
+      <c r="I189" t="inlineStr">
+        <is>
+          <t>Agosto - 25</t>
+        </is>
+      </c>
       <c r="J189" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15656,11 +15692,11 @@
       </c>
       <c r="K189" t="inlineStr">
         <is>
-          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
+          <t>65db6ab7-0b7f-4010-bc49-7c986f097c10</t>
         </is>
       </c>
       <c r="L189" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="190">
@@ -15676,12 +15712,12 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>MENOR COSTE</t>
+          <t>HERGO - DISTRIBUCION</t>
         </is>
       </c>
       <c r="D190" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="E190" t="inlineStr"/>
@@ -15689,7 +15725,7 @@
       <c r="G190" t="inlineStr"/>
       <c r="H190" t="inlineStr">
         <is>
-          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
+          <t>PLAN TRADI</t>
         </is>
       </c>
       <c r="I190" t="inlineStr"/>
@@ -15700,11 +15736,11 @@
       </c>
       <c r="K190" t="inlineStr">
         <is>
-          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
+          <t>d4c771ab-037f-4dd0-a7d4-0bb133878a30</t>
         </is>
       </c>
       <c r="L190" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="191">
@@ -15720,12 +15756,12 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>HERGO - DISTRIBUCION</t>
+          <t>MENOR COSTE</t>
         </is>
       </c>
       <c r="D191" t="inlineStr">
         <is>
-          <t>RECHAZOS AGO 26</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="E191" t="inlineStr"/>
@@ -15733,7 +15769,7 @@
       <c r="G191" t="inlineStr"/>
       <c r="H191" t="inlineStr">
         <is>
-          <t>RECHAZOS ago 26</t>
+          <t>PLANOGRAMA - MENOR COSTE ALBERTI</t>
         </is>
       </c>
       <c r="I191" t="inlineStr"/>
@@ -15744,7 +15780,7 @@
       </c>
       <c r="K191" t="inlineStr">
         <is>
-          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
+          <t>002a3f72-0d37-46fa-8cee-aa0b67dcb88c</t>
         </is>
       </c>
       <c r="L191" t="n">
@@ -15769,30 +15805,18 @@
       </c>
       <c r="D192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
+          <t>RECHAZOS AGO 26</t>
         </is>
       </c>
       <c r="E192" t="inlineStr"/>
-      <c r="F192" t="inlineStr">
-        <is>
-          <t>SEGUIMIENTO DE MARCAS</t>
-        </is>
-      </c>
-      <c r="G192" t="inlineStr">
-        <is>
-          <t>07-2025</t>
-        </is>
-      </c>
+      <c r="F192" t="inlineStr"/>
+      <c r="G192" t="inlineStr"/>
       <c r="H192" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
-        </is>
-      </c>
-      <c r="I192" t="inlineStr">
-        <is>
-          <t>Julio - 25</t>
-        </is>
-      </c>
+          <t>RECHAZOS ago 26</t>
+        </is>
+      </c>
+      <c r="I192" t="inlineStr"/>
       <c r="J192" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -15800,11 +15824,11 @@
       </c>
       <c r="K192" t="inlineStr">
         <is>
-          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
+          <t>27c984a1-8a8c-4da5-bb04-fc0b98239a0a</t>
         </is>
       </c>
       <c r="L192" t="n">
-        <v>0</v>
+        <v>7</v>
       </c>
     </row>
     <row r="193">
@@ -15825,7 +15849,7 @@
       </c>
       <c r="D193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2025</t>
         </is>
       </c>
       <c r="E193" t="inlineStr"/>
@@ -15836,17 +15860,17 @@
       </c>
       <c r="G193" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H193" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 25</t>
         </is>
       </c>
       <c r="I193" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J193" t="inlineStr">
@@ -15856,7 +15880,7 @@
       </c>
       <c r="K193" t="inlineStr">
         <is>
-          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
+          <t>232ad65b-14dd-4f73-b798-bd942ce09f67</t>
         </is>
       </c>
       <c r="L193" t="n">
@@ -15881,7 +15905,7 @@
       </c>
       <c r="D194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2025</t>
         </is>
       </c>
       <c r="E194" t="inlineStr"/>
@@ -15892,17 +15916,17 @@
       </c>
       <c r="G194" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H194" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 25</t>
         </is>
       </c>
       <c r="I194" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J194" t="inlineStr">
@@ -15912,7 +15936,7 @@
       </c>
       <c r="K194" t="inlineStr">
         <is>
-          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
+          <t>6d1ee9f1-c6d0-4bce-ad51-6d6eaab4f86a</t>
         </is>
       </c>
       <c r="L194" t="n">
@@ -15937,7 +15961,7 @@
       </c>
       <c r="D195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2025</t>
         </is>
       </c>
       <c r="E195" t="inlineStr"/>
@@ -15948,17 +15972,17 @@
       </c>
       <c r="G195" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H195" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 25</t>
         </is>
       </c>
       <c r="I195" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J195" t="inlineStr">
@@ -15968,7 +15992,7 @@
       </c>
       <c r="K195" t="inlineStr">
         <is>
-          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
+          <t>5bdfd660-16b1-4b24-95cd-4168bd06d8c0</t>
         </is>
       </c>
       <c r="L195" t="n">
@@ -15993,7 +16017,7 @@
       </c>
       <c r="D196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 10-2025</t>
         </is>
       </c>
       <c r="E196" t="inlineStr"/>
@@ -16004,17 +16028,17 @@
       </c>
       <c r="G196" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H196" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Octubre 25</t>
         </is>
       </c>
       <c r="I196" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J196" t="inlineStr">
@@ -16024,7 +16048,7 @@
       </c>
       <c r="K196" t="inlineStr">
         <is>
-          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
+          <t>d8308de5-2860-4ddd-b8db-a98ff4e0c240</t>
         </is>
       </c>
       <c r="L196" t="n">
@@ -16049,7 +16073,7 @@
       </c>
       <c r="D197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 11-2025</t>
         </is>
       </c>
       <c r="E197" t="inlineStr"/>
@@ -16060,17 +16084,17 @@
       </c>
       <c r="G197" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H197" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Noviembre 25</t>
         </is>
       </c>
       <c r="I197" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J197" t="inlineStr">
@@ -16080,7 +16104,7 @@
       </c>
       <c r="K197" t="inlineStr">
         <is>
-          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
+          <t>e4aa2462-35bc-4944-92c3-da25fef46805</t>
         </is>
       </c>
       <c r="L197" t="n">
@@ -16105,7 +16129,7 @@
       </c>
       <c r="D198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 12-2025</t>
         </is>
       </c>
       <c r="E198" t="inlineStr"/>
@@ -16116,17 +16140,17 @@
       </c>
       <c r="G198" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H198" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Diciembre 25</t>
         </is>
       </c>
       <c r="I198" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J198" t="inlineStr">
@@ -16136,7 +16160,7 @@
       </c>
       <c r="K198" t="inlineStr">
         <is>
-          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
+          <t>e55586bb-28ea-4588-b1cd-58ddc21b26be</t>
         </is>
       </c>
       <c r="L198" t="n">
@@ -16161,7 +16185,7 @@
       </c>
       <c r="D199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 01-2026</t>
         </is>
       </c>
       <c r="E199" t="inlineStr"/>
@@ -16172,17 +16196,17 @@
       </c>
       <c r="G199" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H199" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Enero 26</t>
         </is>
       </c>
       <c r="I199" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J199" t="inlineStr">
@@ -16192,7 +16216,7 @@
       </c>
       <c r="K199" t="inlineStr">
         <is>
-          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
+          <t>ed4bbb7b-39ab-47a1-a01c-6c3187be287c</t>
         </is>
       </c>
       <c r="L199" t="n">
@@ -16217,7 +16241,7 @@
       </c>
       <c r="D200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 02-2026</t>
         </is>
       </c>
       <c r="E200" t="inlineStr"/>
@@ -16228,17 +16252,17 @@
       </c>
       <c r="G200" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H200" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Febrero 26</t>
         </is>
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -16248,7 +16272,7 @@
       </c>
       <c r="K200" t="inlineStr">
         <is>
-          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
+          <t>275b6f24-424a-43ac-9ef5-7aa9ef7081af</t>
         </is>
       </c>
       <c r="L200" t="n">
@@ -16273,7 +16297,7 @@
       </c>
       <c r="D201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 03-2026</t>
         </is>
       </c>
       <c r="E201" t="inlineStr"/>
@@ -16284,17 +16308,17 @@
       </c>
       <c r="G201" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H201" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Marzo 26</t>
         </is>
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -16304,7 +16328,7 @@
       </c>
       <c r="K201" t="inlineStr">
         <is>
-          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
+          <t>29930ce6-3879-4a6b-9243-71e6c015449f</t>
         </is>
       </c>
       <c r="L201" t="n">
@@ -16329,7 +16353,7 @@
       </c>
       <c r="D202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 04-2026</t>
         </is>
       </c>
       <c r="E202" t="inlineStr"/>
@@ -16340,17 +16364,17 @@
       </c>
       <c r="G202" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H202" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Abril 26</t>
         </is>
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -16360,7 +16384,7 @@
       </c>
       <c r="K202" t="inlineStr">
         <is>
-          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
+          <t>21b74ad7-1c37-4b51-9f78-58f0466a4b18</t>
         </is>
       </c>
       <c r="L202" t="n">
@@ -16385,7 +16409,7 @@
       </c>
       <c r="D203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 05-2026</t>
         </is>
       </c>
       <c r="E203" t="inlineStr"/>
@@ -16396,17 +16420,17 @@
       </c>
       <c r="G203" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H203" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Mayo 26</t>
         </is>
       </c>
       <c r="I203" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J203" t="inlineStr">
@@ -16416,7 +16440,7 @@
       </c>
       <c r="K203" t="inlineStr">
         <is>
-          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
+          <t>944cbced-2cfb-4264-9e87-eabc1808950f</t>
         </is>
       </c>
       <c r="L203" t="n">
@@ -16441,7 +16465,7 @@
       </c>
       <c r="D204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 06-2026</t>
         </is>
       </c>
       <c r="E204" t="inlineStr"/>
@@ -16452,17 +16476,17 @@
       </c>
       <c r="G204" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H204" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Junio 26</t>
         </is>
       </c>
       <c r="I204" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J204" t="inlineStr">
@@ -16472,7 +16496,7 @@
       </c>
       <c r="K204" t="inlineStr">
         <is>
-          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
+          <t>34bedd93-1f17-4d2f-9de8-368673f29c6a</t>
         </is>
       </c>
       <c r="L204" t="n">
@@ -16497,7 +16521,7 @@
       </c>
       <c r="D205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 07-2026</t>
         </is>
       </c>
       <c r="E205" t="inlineStr"/>
@@ -16508,17 +16532,17 @@
       </c>
       <c r="G205" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H205" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Julio 26</t>
         </is>
       </c>
       <c r="I205" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J205" t="inlineStr">
@@ -16528,11 +16552,11 @@
       </c>
       <c r="K205" t="inlineStr">
         <is>
-          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
+          <t>4ea6316b-51ca-4d99-80cb-c767aeaeb217</t>
         </is>
       </c>
       <c r="L205" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="206">
@@ -16553,7 +16577,7 @@
       </c>
       <c r="D206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
+          <t>SEGUIMIENTO DE MARCAS 08-2026</t>
         </is>
       </c>
       <c r="E206" t="inlineStr"/>
@@ -16564,17 +16588,17 @@
       </c>
       <c r="G206" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H206" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
+          <t>SEGUIMIENTO DE MARCAS - Agosto 26</t>
         </is>
       </c>
       <c r="I206" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J206" t="inlineStr">
@@ -16584,11 +16608,11 @@
       </c>
       <c r="K206" t="inlineStr">
         <is>
-          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
+          <t>40805cb7-8f94-4203-86c8-49c563a4dfd9</t>
         </is>
       </c>
       <c r="L206" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="207">
@@ -16609,28 +16633,28 @@
       </c>
       <c r="D207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
+          <t>SEGUIMIENTO DE MARCAS 09-2026</t>
         </is>
       </c>
       <c r="E207" t="inlineStr"/>
       <c r="F207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO</t>
+          <t>SEGUIMIENTO DE MARCAS</t>
         </is>
       </c>
       <c r="G207" t="inlineStr">
         <is>
-          <t>07-2025</t>
+          <t>09-2026</t>
         </is>
       </c>
       <c r="H207" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
+          <t>SEGUIMIENTO DE MARCAS - Septiembre 26</t>
         </is>
       </c>
       <c r="I207" t="inlineStr">
         <is>
-          <t>Julio - 25</t>
+          <t>Septiembre - 26</t>
         </is>
       </c>
       <c r="J207" t="inlineStr">
@@ -16640,11 +16664,11 @@
       </c>
       <c r="K207" t="inlineStr">
         <is>
-          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
+          <t>982f2555-a3ca-499b-8d07-13f975303e56</t>
         </is>
       </c>
       <c r="L207" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="208">
@@ -16665,7 +16689,7 @@
       </c>
       <c r="D208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2025</t>
         </is>
       </c>
       <c r="E208" t="inlineStr"/>
@@ -16676,17 +16700,17 @@
       </c>
       <c r="G208" t="inlineStr">
         <is>
-          <t>08-2025</t>
+          <t>07-2025</t>
         </is>
       </c>
       <c r="H208" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 25</t>
         </is>
       </c>
       <c r="I208" t="inlineStr">
         <is>
-          <t>Agosto - 25</t>
+          <t>Julio - 25</t>
         </is>
       </c>
       <c r="J208" t="inlineStr">
@@ -16696,11 +16720,11 @@
       </c>
       <c r="K208" t="inlineStr">
         <is>
-          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
+          <t>ec4eda03-3d48-4add-ab38-6ef3a40418ab</t>
         </is>
       </c>
       <c r="L208" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="209">
@@ -16721,7 +16745,7 @@
       </c>
       <c r="D209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2025</t>
         </is>
       </c>
       <c r="E209" t="inlineStr"/>
@@ -16732,17 +16756,17 @@
       </c>
       <c r="G209" t="inlineStr">
         <is>
-          <t>09-2025</t>
+          <t>08-2025</t>
         </is>
       </c>
       <c r="H209" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 25</t>
         </is>
       </c>
       <c r="I209" t="inlineStr">
         <is>
-          <t>Septiembre - 25</t>
+          <t>Agosto - 25</t>
         </is>
       </c>
       <c r="J209" t="inlineStr">
@@ -16752,7 +16776,7 @@
       </c>
       <c r="K209" t="inlineStr">
         <is>
-          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
+          <t>f6f6bc57-4253-4ba5-a0d4-dccd1e8005c6</t>
         </is>
       </c>
       <c r="L209" t="n">
@@ -16777,7 +16801,7 @@
       </c>
       <c r="D210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2025</t>
         </is>
       </c>
       <c r="E210" t="inlineStr"/>
@@ -16788,17 +16812,17 @@
       </c>
       <c r="G210" t="inlineStr">
         <is>
-          <t>10-2025</t>
+          <t>09-2025</t>
         </is>
       </c>
       <c r="H210" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 25</t>
         </is>
       </c>
       <c r="I210" t="inlineStr">
         <is>
-          <t>Octubre - 25</t>
+          <t>Septiembre - 25</t>
         </is>
       </c>
       <c r="J210" t="inlineStr">
@@ -16808,11 +16832,11 @@
       </c>
       <c r="K210" t="inlineStr">
         <is>
-          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
+          <t>efe4c31b-0b0f-403f-9824-14331c4d8ff6</t>
         </is>
       </c>
       <c r="L210" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="211">
@@ -16833,7 +16857,7 @@
       </c>
       <c r="D211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 10-2025</t>
         </is>
       </c>
       <c r="E211" t="inlineStr"/>
@@ -16844,17 +16868,17 @@
       </c>
       <c r="G211" t="inlineStr">
         <is>
-          <t>11-2025</t>
+          <t>10-2025</t>
         </is>
       </c>
       <c r="H211" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Octubre 25</t>
         </is>
       </c>
       <c r="I211" t="inlineStr">
         <is>
-          <t>Noviembre - 25</t>
+          <t>Octubre - 25</t>
         </is>
       </c>
       <c r="J211" t="inlineStr">
@@ -16864,11 +16888,11 @@
       </c>
       <c r="K211" t="inlineStr">
         <is>
-          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
+          <t>02d71732-3391-447c-a5b5-1cab4690361c</t>
         </is>
       </c>
       <c r="L211" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="212">
@@ -16889,7 +16913,7 @@
       </c>
       <c r="D212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 11-2025</t>
         </is>
       </c>
       <c r="E212" t="inlineStr"/>
@@ -16900,17 +16924,17 @@
       </c>
       <c r="G212" t="inlineStr">
         <is>
-          <t>12-2025</t>
+          <t>11-2025</t>
         </is>
       </c>
       <c r="H212" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Noviembre 25</t>
         </is>
       </c>
       <c r="I212" t="inlineStr">
         <is>
-          <t>Diciembre - 25</t>
+          <t>Noviembre - 25</t>
         </is>
       </c>
       <c r="J212" t="inlineStr">
@@ -16920,7 +16944,7 @@
       </c>
       <c r="K212" t="inlineStr">
         <is>
-          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
+          <t>a45f1f4f-95cc-4323-91f3-4522e54b8760</t>
         </is>
       </c>
       <c r="L212" t="n">
@@ -16945,7 +16969,7 @@
       </c>
       <c r="D213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 12-2025</t>
         </is>
       </c>
       <c r="E213" t="inlineStr"/>
@@ -16956,17 +16980,17 @@
       </c>
       <c r="G213" t="inlineStr">
         <is>
-          <t>01-2026</t>
+          <t>12-2025</t>
         </is>
       </c>
       <c r="H213" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Diciembre 25</t>
         </is>
       </c>
       <c r="I213" t="inlineStr">
         <is>
-          <t>Enero - 26</t>
+          <t>Diciembre - 25</t>
         </is>
       </c>
       <c r="J213" t="inlineStr">
@@ -16976,7 +17000,7 @@
       </c>
       <c r="K213" t="inlineStr">
         <is>
-          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
+          <t>8b7d7d20-5664-4a72-9d79-70e225ee8c63</t>
         </is>
       </c>
       <c r="L213" t="n">
@@ -17001,7 +17025,7 @@
       </c>
       <c r="D214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 01-2026</t>
         </is>
       </c>
       <c r="E214" t="inlineStr"/>
@@ -17012,17 +17036,17 @@
       </c>
       <c r="G214" t="inlineStr">
         <is>
-          <t>02-2026</t>
+          <t>01-2026</t>
         </is>
       </c>
       <c r="H214" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Enero 26</t>
         </is>
       </c>
       <c r="I214" t="inlineStr">
         <is>
-          <t>Febrero - 26</t>
+          <t>Enero - 26</t>
         </is>
       </c>
       <c r="J214" t="inlineStr">
@@ -17032,7 +17056,7 @@
       </c>
       <c r="K214" t="inlineStr">
         <is>
-          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
+          <t>aa8b12f0-1f59-4742-9fc6-139a392d3535</t>
         </is>
       </c>
       <c r="L214" t="n">
@@ -17057,7 +17081,7 @@
       </c>
       <c r="D215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 02-2026</t>
         </is>
       </c>
       <c r="E215" t="inlineStr"/>
@@ -17068,17 +17092,17 @@
       </c>
       <c r="G215" t="inlineStr">
         <is>
-          <t>03-2026</t>
+          <t>02-2026</t>
         </is>
       </c>
       <c r="H215" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Febrero 26</t>
         </is>
       </c>
       <c r="I215" t="inlineStr">
         <is>
-          <t>Marzo - 26</t>
+          <t>Febrero - 26</t>
         </is>
       </c>
       <c r="J215" t="inlineStr">
@@ -17088,7 +17112,7 @@
       </c>
       <c r="K215" t="inlineStr">
         <is>
-          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
+          <t>79c800f7-e947-4fc1-ae74-6f44ee243796</t>
         </is>
       </c>
       <c r="L215" t="n">
@@ -17113,7 +17137,7 @@
       </c>
       <c r="D216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 03-2026</t>
         </is>
       </c>
       <c r="E216" t="inlineStr"/>
@@ -17124,17 +17148,17 @@
       </c>
       <c r="G216" t="inlineStr">
         <is>
-          <t>04-2026</t>
+          <t>03-2026</t>
         </is>
       </c>
       <c r="H216" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Marzo 26</t>
         </is>
       </c>
       <c r="I216" t="inlineStr">
         <is>
-          <t>Abril - 26</t>
+          <t>Marzo - 26</t>
         </is>
       </c>
       <c r="J216" t="inlineStr">
@@ -17144,11 +17168,11 @@
       </c>
       <c r="K216" t="inlineStr">
         <is>
-          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
+          <t>20067df5-8ddf-4fda-bfda-c5ff88485713</t>
         </is>
       </c>
       <c r="L216" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
     </row>
     <row r="217">
@@ -17169,7 +17193,7 @@
       </c>
       <c r="D217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 04-2026</t>
         </is>
       </c>
       <c r="E217" t="inlineStr"/>
@@ -17180,17 +17204,17 @@
       </c>
       <c r="G217" t="inlineStr">
         <is>
-          <t>05-2026</t>
+          <t>04-2026</t>
         </is>
       </c>
       <c r="H217" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Abril 26</t>
         </is>
       </c>
       <c r="I217" t="inlineStr">
         <is>
-          <t>Mayo - 26</t>
+          <t>Abril - 26</t>
         </is>
       </c>
       <c r="J217" t="inlineStr">
@@ -17200,11 +17224,11 @@
       </c>
       <c r="K217" t="inlineStr">
         <is>
-          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
+          <t>9665a25d-07b0-47df-9aaa-6214c22a6932</t>
         </is>
       </c>
       <c r="L217" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
     </row>
     <row r="218">
@@ -17225,7 +17249,7 @@
       </c>
       <c r="D218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 05-2026</t>
         </is>
       </c>
       <c r="E218" t="inlineStr"/>
@@ -17236,17 +17260,17 @@
       </c>
       <c r="G218" t="inlineStr">
         <is>
-          <t>06-2026</t>
+          <t>05-2026</t>
         </is>
       </c>
       <c r="H218" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Mayo 26</t>
         </is>
       </c>
       <c r="I218" t="inlineStr">
         <is>
-          <t>Junio - 26</t>
+          <t>Mayo - 26</t>
         </is>
       </c>
       <c r="J218" t="inlineStr">
@@ -17256,11 +17280,11 @@
       </c>
       <c r="K218" t="inlineStr">
         <is>
-          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
+          <t>5e5627f5-bd0f-4a37-b33d-3132b6f8cd2c</t>
         </is>
       </c>
       <c r="L218" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
     </row>
     <row r="219">
@@ -17281,7 +17305,7 @@
       </c>
       <c r="D219" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 06-2026</t>
         </is>
       </c>
       <c r="E219" t="inlineStr"/>
@@ -17292,17 +17316,17 @@
       </c>
       <c r="G219" t="inlineStr">
         <is>
-          <t>07-2026</t>
+          <t>06-2026</t>
         </is>
       </c>
       <c r="H219" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Junio 26</t>
         </is>
       </c>
       <c r="I219" t="inlineStr">
         <is>
-          <t>Julio - 26</t>
+          <t>Junio - 26</t>
         </is>
       </c>
       <c r="J219" t="inlineStr">
@@ -17312,11 +17336,11 @@
       </c>
       <c r="K219" t="inlineStr">
         <is>
-          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
+          <t>aa3feb1b-df68-411a-9c01-d9fa739081a6</t>
         </is>
       </c>
       <c r="L219" t="n">
-        <v>7</v>
+        <v>9</v>
       </c>
     </row>
     <row r="220">
@@ -17337,7 +17361,7 @@
       </c>
       <c r="D220" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 07-2026</t>
         </is>
       </c>
       <c r="E220" t="inlineStr"/>
@@ -17348,17 +17372,17 @@
       </c>
       <c r="G220" t="inlineStr">
         <is>
-          <t>08-2026</t>
+          <t>07-2026</t>
         </is>
       </c>
       <c r="H220" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Julio 26</t>
         </is>
       </c>
       <c r="I220" t="inlineStr">
         <is>
-          <t>Agosto - 26</t>
+          <t>Julio - 26</t>
         </is>
       </c>
       <c r="J220" t="inlineStr">
@@ -17368,11 +17392,11 @@
       </c>
       <c r="K220" t="inlineStr">
         <is>
-          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
+          <t>d94b898b-ca9a-4f65-bd76-5a049696c931</t>
         </is>
       </c>
       <c r="L220" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
     </row>
     <row r="221">
@@ -17393,7 +17417,7 @@
       </c>
       <c r="D221" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 08-2026</t>
         </is>
       </c>
       <c r="E221" t="inlineStr"/>
@@ -17404,17 +17428,17 @@
       </c>
       <c r="G221" t="inlineStr">
         <is>
-          <t>09-2026</t>
+          <t>08-2026</t>
         </is>
       </c>
       <c r="H221" t="inlineStr">
         <is>
-          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+          <t>SEGUIMIENTO PLAN ESPACIO - Agosto 26</t>
         </is>
       </c>
       <c r="I221" t="inlineStr">
         <is>
-          <t>Septiembre - 26</t>
+          <t>Agosto - 26</t>
         </is>
       </c>
       <c r="J221" t="inlineStr">
@@ -17424,11 +17448,11 @@
       </c>
       <c r="K221" t="inlineStr">
         <is>
-          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
+          <t>d3503eaf-eda8-492e-9a13-46088a447d3f</t>
         </is>
       </c>
       <c r="L221" t="n">
-        <v>0</v>
+        <v>8</v>
       </c>
     </row>
     <row r="222">
@@ -17449,18 +17473,30 @@
       </c>
       <c r="D222" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - ALTA</t>
+          <t>SEGUIMIENTO PLAN ESPACIO 09-2026</t>
         </is>
       </c>
       <c r="E222" t="inlineStr"/>
-      <c r="F222" t="inlineStr"/>
-      <c r="G222" t="inlineStr"/>
+      <c r="F222" t="inlineStr">
+        <is>
+          <t>SEGUIMIENTO PLAN ESPACIO</t>
+        </is>
+      </c>
+      <c r="G222" t="inlineStr">
+        <is>
+          <t>09-2026</t>
+        </is>
+      </c>
       <c r="H222" t="inlineStr">
         <is>
-          <t>Sabores por PDV - ALTA</t>
-        </is>
-      </c>
-      <c r="I222" t="inlineStr"/>
+          <t>SEGUIMIENTO PLAN ESPACIO - Septiembre 26</t>
+        </is>
+      </c>
+      <c r="I222" t="inlineStr">
+        <is>
+          <t>Septiembre - 26</t>
+        </is>
+      </c>
       <c r="J222" t="inlineStr">
         <is>
           <t>Grupo Hergo - Jefes</t>
@@ -17468,7 +17504,7 @@
       </c>
       <c r="K222" t="inlineStr">
         <is>
-          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
+          <t>059b36e9-ab26-4fb2-8647-67f060e36c7c</t>
         </is>
       </c>
       <c r="L222" t="n">
@@ -17493,7 +17529,7 @@
       </c>
       <c r="D223" t="inlineStr">
         <is>
-          <t>SABORES POR PDV - COUSTLAIN</t>
+          <t>SABORES POR PDV - ALTA</t>
         </is>
       </c>
       <c r="E223" t="inlineStr"/>
@@ -17501,7 +17537,7 @@
       <c r="G223" t="inlineStr"/>
       <c r="H223" t="inlineStr">
         <is>
-          <t>Sabores por PDV - COUSTLAIN</t>
+          <t>Sabores por PDV - ALTA</t>
         </is>
       </c>
       <c r="I223" t="inlineStr"/>
@@ -17512,11 +17548,11 @@
       </c>
       <c r="K223" t="inlineStr">
         <is>
-          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
+          <t>16acb159-f0ec-4a26-8221-f63c9516d249</t>
         </is>
       </c>
       <c r="L223" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="224">
@@ -17537,7 +17573,7 @@
       </c>
       <c r="D224" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>SABORES POR PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="E224" t="inlineStr"/>
@@ -17545,7 +17581,7 @@
       <c r="G224" t="inlineStr"/>
       <c r="H224" t="inlineStr">
         <is>
-          <t>TASA MODIFICACION DE PEDIDOS</t>
+          <t>Sabores por PDV - COUSTLAIN</t>
         </is>
       </c>
       <c r="I224" t="inlineStr"/>
@@ -17556,7 +17592,7 @@
       </c>
       <c r="K224" t="inlineStr">
         <is>
-          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
+          <t>3c32ea4c-88e3-473f-8690-fbd5c62a4a7d</t>
         </is>
       </c>
       <c r="L224" t="n">
@@ -17581,7 +17617,7 @@
       </c>
       <c r="D225" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="E225" t="inlineStr"/>
@@ -17589,7 +17625,7 @@
       <c r="G225" t="inlineStr"/>
       <c r="H225" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO</t>
+          <t>TASA MODIFICACION DE PEDIDOS</t>
         </is>
       </c>
       <c r="I225" t="inlineStr"/>
@@ -17600,11 +17636,11 @@
       </c>
       <c r="K225" t="inlineStr">
         <is>
-          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
+          <t>9eded255-affc-41f1-82a7-38bb12771cde</t>
         </is>
       </c>
       <c r="L225" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="226">
@@ -17625,7 +17661,7 @@
       </c>
       <c r="D226" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="E226" t="inlineStr"/>
@@ -17633,7 +17669,7 @@
       <c r="G226" t="inlineStr"/>
       <c r="H226" t="inlineStr">
         <is>
-          <t>TRAFICO - DIARIO COSTA</t>
+          <t>TRAFICO - DIARIO</t>
         </is>
       </c>
       <c r="I226" t="inlineStr"/>
@@ -17644,7 +17680,7 @@
       </c>
       <c r="K226" t="inlineStr">
         <is>
-          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
+          <t>6c931870-e5c9-4cbc-9aac-e0368aab3ffb</t>
         </is>
       </c>
       <c r="L226" t="n">
@@ -17669,7 +17705,7 @@
       </c>
       <c r="D227" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="E227" t="inlineStr"/>
@@ -17677,7 +17713,7 @@
       <c r="G227" t="inlineStr"/>
       <c r="H227" t="inlineStr">
         <is>
-          <t>VENTAS SMK</t>
+          <t>TRAFICO - DIARIO COSTA</t>
         </is>
       </c>
       <c r="I227" t="inlineStr"/>
@@ -17688,11 +17724,11 @@
       </c>
       <c r="K227" t="inlineStr">
         <is>
-          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
+          <t>88b79c83-6c87-449b-b022-42b61ebf934b</t>
         </is>
       </c>
       <c r="L227" t="n">
-        <v>3</v>
+        <v>12</v>
       </c>
     </row>
     <row r="228">
@@ -17713,7 +17749,7 @@
       </c>
       <c r="D228" t="inlineStr">
         <is>
-          <t>VENTA MAYORISTA DETALLE</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="E228" t="inlineStr"/>
@@ -17721,7 +17757,7 @@
       <c r="G228" t="inlineStr"/>
       <c r="H228" t="inlineStr">
         <is>
-          <t>Venta Mayorista Detalle</t>
+          <t>VENTAS SMK</t>
         </is>
       </c>
       <c r="I228" t="inlineStr"/>
@@ -17732,11 +17768,11 @@
       </c>
       <c r="K228" t="inlineStr">
         <is>
-          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
+          <t>4ae4d5e5-5b71-43a1-ae96-169f12bb778d</t>
         </is>
       </c>
       <c r="L228" t="n">
-        <v>44</v>
+        <v>3</v>
       </c>
     </row>
     <row r="229">
@@ -17757,7 +17793,7 @@
       </c>
       <c r="D229" t="inlineStr">
         <is>
-          <t>STOCK POR PROVEEDORES</t>
+          <t>VENTA MAYORISTA DETALLE</t>
         </is>
       </c>
       <c r="E229" t="inlineStr"/>
@@ -17765,7 +17801,7 @@
       <c r="G229" t="inlineStr"/>
       <c r="H229" t="inlineStr">
         <is>
-          <t>stock por proveedores</t>
+          <t>Venta Mayorista Detalle</t>
         </is>
       </c>
       <c r="I229" t="inlineStr"/>
@@ -17776,17 +17812,61 @@
       </c>
       <c r="K229" t="inlineStr">
         <is>
+          <t>d33e3dcd-18b9-4114-83d8-42300c627ebc</t>
+        </is>
+      </c>
+      <c r="L229" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="230">
+      <c r="A230" s="2" t="inlineStr">
+        <is>
+          <t>SI</t>
+        </is>
+      </c>
+      <c r="B230" t="inlineStr">
+        <is>
+          <t>JEFES</t>
+        </is>
+      </c>
+      <c r="C230" t="inlineStr">
+        <is>
+          <t>HERGO - DISTRIBUCION</t>
+        </is>
+      </c>
+      <c r="D230" t="inlineStr">
+        <is>
+          <t>STOCK POR PROVEEDORES</t>
+        </is>
+      </c>
+      <c r="E230" t="inlineStr"/>
+      <c r="F230" t="inlineStr"/>
+      <c r="G230" t="inlineStr"/>
+      <c r="H230" t="inlineStr">
+        <is>
+          <t>stock por proveedores</t>
+        </is>
+      </c>
+      <c r="I230" t="inlineStr"/>
+      <c r="J230" t="inlineStr">
+        <is>
+          <t>Grupo Hergo - Jefes</t>
+        </is>
+      </c>
+      <c r="K230" t="inlineStr">
+        <is>
           <t>bdfe582a-c303-4732-b9b7-2390e04aa58e</t>
         </is>
       </c>
-      <c r="L229" t="n">
+      <c r="L230" t="n">
         <v>53</v>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L229"/>
+  <autoFilter ref="A1:L230"/>
   <dataValidations count="1">
-    <dataValidation sqref="A2:A229" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
+    <dataValidation sqref="A2:A230" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" promptTitle="Publicar" prompt="SI publica en el tablero. NO lo descarta. Vacio = no publica." type="list">
       <formula1>"SI,NO"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>